<commit_message>
Anchor benefit resets to signup dates
</commit_message>
<xml_diff>
--- a/templates/VIP-Tracker-Template.xlsx
+++ b/templates/VIP-Tracker-Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIP Signups" sheetId="1" r:id="Rbfed072f45e34bee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plugin Export" sheetId="2" r:id="Re3925a91caca43ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benefit Resets" sheetId="3" r:id="R9a8867be6134425c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup Guide" sheetId="4" r:id="R7ff04e0fc7294964"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="R1b869dfa08a64b50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIP Signups" sheetId="1" r:id="R661ad5d51aef4ee7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plugin Export" sheetId="2" r:id="Re997efb859e84399"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benefit Resets" sheetId="3" r:id="R9806aecaa1544a1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup Guide" sheetId="4" r:id="R87a4b546df944546"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="R9a1a57fb456c4fea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -172,7 +172,7 @@
         <x:color rgb="FF2F7D4C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF6EE"/>
         </x:patternFill>
       </x:fill>
@@ -183,7 +183,7 @@
         <x:color rgb="FFB7791F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4DE"/>
         </x:patternFill>
       </x:fill>
@@ -194,7 +194,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -205,7 +205,7 @@
         <x:color rgb="FF2F7D4C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF6EE"/>
         </x:patternFill>
       </x:fill>
@@ -216,7 +216,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -597,11 +597,11 @@
       </x:c>
       <x:c r="L5" s="20" t="str">
         <x:f>IF(A5="","",IFERROR(TEXTJOIN("; ",TRUE,FILTER('Benefit Resets'!$G$5:$G$204,'Benefit Resets'!$A$5:$A$204=A5,'Benefit Resets'!$I$5:$I$204="Yes")),""))</x:f>
-        <x:v>Photo Slot: Available; Gamba Token: Resets 2026-06-17</x:v>
+        <x:v>Photo Slot: Resets 2026-07-01; Gamba Token: Available</x:v>
       </x:c>
       <x:c r="M5" s="20" t="str">
         <x:f>IF(A5="","",IF(L5="",G5,G5&amp;" | "&amp;L5))</x:f>
-        <x:v>Queue Priority; Photo Slot; Gamba Token | Photo Slot: Available; Gamba Token: Resets 2026-06-17</x:v>
+        <x:v>Queue Priority; Photo Slot; Gamba Token | Photo Slot: Resets 2026-07-01; Gamba Token: Available</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -5734,46 +5734,58 @@
       <x:c r="A5" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!A$5:A$204,MATCH(ROWS($A$5:A5),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
       </x:c>
-      <x:c r="B5" s="20" t="str">
+      <x:c r="B5" s="20" t="n">
         <x:f>IFERROR(INDEX('VIP Signups'!D$5:D$204,MATCH(ROWS($A$5:A5),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>46204</x:v>
       </x:c>
       <x:c r="C5" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!F$5:F$204,MATCH(ROWS($A$5:A5),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>Gold</x:v>
       </x:c>
       <x:c r="D5" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!M$5:M$204,MATCH(ROWS($A$5:A5),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>Queue Priority; Photo Slot; Gamba Token | Photo Slot: Resets 2026-07-01; Gamba Token: Available</x:v>
       </x:c>
       <x:c r="E5" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!C$5:C$204,MATCH(ROWS($A$5:A5),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>30 Days</x:v>
       </x:c>
       <x:c r="F5" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!E$5:E$204,MATCH(ROWS($A$5:A5),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="G5" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!H$5:H$204,MATCH(ROWS($A$5:A5),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>Renewal reminder one week before expiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!A$5:A$204,MATCH(ROWS($A$5:A6),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
       </x:c>
-      <x:c r="B6" s="20" t="str">
+      <x:c r="B6" s="20" t="n">
         <x:f>IFERROR(INDEX('VIP Signups'!D$5:D$204,MATCH(ROWS($A$5:A6),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>46189</x:v>
       </x:c>
       <x:c r="C6" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!F$5:F$204,MATCH(ROWS($A$5:A6),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="D6" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!M$5:M$204,MATCH(ROWS($A$5:A6),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>Event Access; Photo Slot | true</x:v>
       </x:c>
       <x:c r="E6" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!C$5:C$204,MATCH(ROWS($A$5:A6),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>Event Only</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!E$5:E$204,MATCH(ROWS($A$5:A6),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>Expiring Soon</x:v>
       </x:c>
       <x:c r="G6" s="20" t="str">
         <x:f>IFERROR(INDEX('VIP Signups'!H$5:H$204,MATCH(ROWS($A$5:A6),'VIP Signups'!$K$5:$K$204,0)),"")</x:f>
+        <x:v>One-night venue pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10471,19 +10483,19 @@
         <x:v>Monthly</x:v>
       </x:c>
       <x:c r="D5" s="21" t="n">
-        <x:v>46143</x:v>
+        <x:v>46192</x:v>
       </x:c>
       <x:c r="E5" s="21" t="n">
-        <x:f>IF(A5="","",IF(D5="","Available",SWITCH(C5,"Daily",D5+1,"Weekly",D5+7,"Monthly",EDATE(D5,1),"Quarterly",EDATE(D5,3),"Yearly",EDATE(D5,12),"One-time","Used","Manual","Manual",D5)))</x:f>
-        <x:v>46174</x:v>
+        <x:f>IF(A5="","",IF(D5="","Available",SWITCH(C5,"Daily",D5+1,"Weekly",IFERROR(VLOOKUP(A5,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D5-VLOOKUP(A5,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D5+7),"Monthly",IFERROR(EDATE(VLOOKUP(A5,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A5,'VIP Signups'!$A$5:$B$204,2,FALSE),D5,"M")+1),EDATE(D5,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A5,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A5,'VIP Signups'!$A$5:$B$204,2,FALSE),D5,"M")/3)+1)*3),EDATE(D5,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A5,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A5,'VIP Signups'!$A$5:$B$204,2,FALSE),D5,"Y")+1)*12),EDATE(D5,12)),"One-time","Used","Manual","Manual",D5)))</x:f>
+        <x:v>46204</x:v>
       </x:c>
       <x:c r="F5" s="20" t="str">
         <x:f>IF(A5="","",IF(D5="","Yes",IF(E5="Manual","Manual",IF(E5="Used","No",IF(E5&lt;=TODAY(),"Yes","No")))))</x:f>
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="G5" s="20" t="str">
         <x:f>IF(A5="","",B5&amp;": "&amp;IF(F5="Yes","Available",IF(F5="Manual","Manual check",IF(ISNUMBER(E5),"Resets "&amp;TEXT(E5,"yyyy-mm-dd"),"Used"))))</x:f>
-        <x:v>Photo Slot: Available</x:v>
+        <x:v>Photo Slot: Resets 2026-07-01</x:v>
       </x:c>
       <x:c r="H5" s="20" t="str">
         <x:v>Example monthly benefit.</x:v>
@@ -10511,16 +10523,16 @@
         <x:v>46183</x:v>
       </x:c>
       <x:c r="E6" s="21" t="n">
-        <x:f>IF(A6="","",IF(D6="","Available",SWITCH(C6,"Daily",D6+1,"Weekly",D6+7,"Monthly",EDATE(D6,1),"Quarterly",EDATE(D6,3),"Yearly",EDATE(D6,12),"One-time","Used","Manual","Manual",D6)))</x:f>
-        <x:v>46190</x:v>
+        <x:f>IF(A6="","",IF(D6="","Available",SWITCH(C6,"Daily",D6+1,"Weekly",IFERROR(VLOOKUP(A6,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D6-VLOOKUP(A6,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D6+7),"Monthly",IFERROR(EDATE(VLOOKUP(A6,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A6,'VIP Signups'!$A$5:$B$204,2,FALSE),D6,"M")+1),EDATE(D6,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A6,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A6,'VIP Signups'!$A$5:$B$204,2,FALSE),D6,"M")/3)+1)*3),EDATE(D6,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A6,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A6,'VIP Signups'!$A$5:$B$204,2,FALSE),D6,"Y")+1)*12),EDATE(D6,12)),"One-time","Used","Manual","Manual",D6)))</x:f>
+        <x:v>46188</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
         <x:f>IF(A6="","",IF(D6="","Yes",IF(E6="Manual","Manual",IF(E6="Used","No",IF(E6&lt;=TODAY(),"Yes","No")))))</x:f>
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G6" s="20" t="str">
         <x:f>IF(A6="","",B6&amp;": "&amp;IF(F6="Yes","Available",IF(F6="Manual","Manual check",IF(ISNUMBER(E6),"Resets "&amp;TEXT(E6,"yyyy-mm-dd"),"Used"))))</x:f>
-        <x:v>Gamba Token: Resets 2026-06-17</x:v>
+        <x:v>Gamba Token: Available</x:v>
       </x:c>
       <x:c r="H6" s="20" t="str">
         <x:v>Example weekly benefit.</x:v>
@@ -10540,7 +10552,7 @@
       <x:c r="C7" s="20"/>
       <x:c r="D7" s="21"/>
       <x:c r="E7" s="21" t="str">
-        <x:f>IF(A7="","",IF(D7="","Available",SWITCH(C7,"Daily",D7+1,"Weekly",D7+7,"Monthly",EDATE(D7,1),"Quarterly",EDATE(D7,3),"Yearly",EDATE(D7,12),"One-time","Used","Manual","Manual",D7)))</x:f>
+        <x:f>IF(A7="","",IF(D7="","Available",SWITCH(C7,"Daily",D7+1,"Weekly",IFERROR(VLOOKUP(A7,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D7-VLOOKUP(A7,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D7+7),"Monthly",IFERROR(EDATE(VLOOKUP(A7,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A7,'VIP Signups'!$A$5:$B$204,2,FALSE),D7,"M")+1),EDATE(D7,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A7,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A7,'VIP Signups'!$A$5:$B$204,2,FALSE),D7,"M")/3)+1)*3),EDATE(D7,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A7,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A7,'VIP Signups'!$A$5:$B$204,2,FALSE),D7,"Y")+1)*12),EDATE(D7,12)),"One-time","Used","Manual","Manual",D7)))</x:f>
       </x:c>
       <x:c r="F7" s="20" t="str">
         <x:f>IF(A7="","",IF(D7="","Yes",IF(E7="Manual","Manual",IF(E7="Used","No",IF(E7&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10563,7 +10575,7 @@
       <x:c r="C8" s="20"/>
       <x:c r="D8" s="21"/>
       <x:c r="E8" s="21" t="str">
-        <x:f>IF(A8="","",IF(D8="","Available",SWITCH(C8,"Daily",D8+1,"Weekly",D8+7,"Monthly",EDATE(D8,1),"Quarterly",EDATE(D8,3),"Yearly",EDATE(D8,12),"One-time","Used","Manual","Manual",D8)))</x:f>
+        <x:f>IF(A8="","",IF(D8="","Available",SWITCH(C8,"Daily",D8+1,"Weekly",IFERROR(VLOOKUP(A8,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D8-VLOOKUP(A8,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D8+7),"Monthly",IFERROR(EDATE(VLOOKUP(A8,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A8,'VIP Signups'!$A$5:$B$204,2,FALSE),D8,"M")+1),EDATE(D8,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A8,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A8,'VIP Signups'!$A$5:$B$204,2,FALSE),D8,"M")/3)+1)*3),EDATE(D8,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A8,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A8,'VIP Signups'!$A$5:$B$204,2,FALSE),D8,"Y")+1)*12),EDATE(D8,12)),"One-time","Used","Manual","Manual",D8)))</x:f>
       </x:c>
       <x:c r="F8" s="20" t="str">
         <x:f>IF(A8="","",IF(D8="","Yes",IF(E8="Manual","Manual",IF(E8="Used","No",IF(E8&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10586,7 +10598,7 @@
       <x:c r="C9" s="20"/>
       <x:c r="D9" s="21"/>
       <x:c r="E9" s="21" t="str">
-        <x:f>IF(A9="","",IF(D9="","Available",SWITCH(C9,"Daily",D9+1,"Weekly",D9+7,"Monthly",EDATE(D9,1),"Quarterly",EDATE(D9,3),"Yearly",EDATE(D9,12),"One-time","Used","Manual","Manual",D9)))</x:f>
+        <x:f>IF(A9="","",IF(D9="","Available",SWITCH(C9,"Daily",D9+1,"Weekly",IFERROR(VLOOKUP(A9,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D9-VLOOKUP(A9,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D9+7),"Monthly",IFERROR(EDATE(VLOOKUP(A9,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A9,'VIP Signups'!$A$5:$B$204,2,FALSE),D9,"M")+1),EDATE(D9,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A9,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A9,'VIP Signups'!$A$5:$B$204,2,FALSE),D9,"M")/3)+1)*3),EDATE(D9,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A9,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A9,'VIP Signups'!$A$5:$B$204,2,FALSE),D9,"Y")+1)*12),EDATE(D9,12)),"One-time","Used","Manual","Manual",D9)))</x:f>
       </x:c>
       <x:c r="F9" s="20" t="str">
         <x:f>IF(A9="","",IF(D9="","Yes",IF(E9="Manual","Manual",IF(E9="Used","No",IF(E9&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10609,7 +10621,7 @@
       <x:c r="C10" s="20"/>
       <x:c r="D10" s="21"/>
       <x:c r="E10" s="21" t="str">
-        <x:f>IF(A10="","",IF(D10="","Available",SWITCH(C10,"Daily",D10+1,"Weekly",D10+7,"Monthly",EDATE(D10,1),"Quarterly",EDATE(D10,3),"Yearly",EDATE(D10,12),"One-time","Used","Manual","Manual",D10)))</x:f>
+        <x:f>IF(A10="","",IF(D10="","Available",SWITCH(C10,"Daily",D10+1,"Weekly",IFERROR(VLOOKUP(A10,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D10-VLOOKUP(A10,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D10+7),"Monthly",IFERROR(EDATE(VLOOKUP(A10,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A10,'VIP Signups'!$A$5:$B$204,2,FALSE),D10,"M")+1),EDATE(D10,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A10,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A10,'VIP Signups'!$A$5:$B$204,2,FALSE),D10,"M")/3)+1)*3),EDATE(D10,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A10,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A10,'VIP Signups'!$A$5:$B$204,2,FALSE),D10,"Y")+1)*12),EDATE(D10,12)),"One-time","Used","Manual","Manual",D10)))</x:f>
       </x:c>
       <x:c r="F10" s="20" t="str">
         <x:f>IF(A10="","",IF(D10="","Yes",IF(E10="Manual","Manual",IF(E10="Used","No",IF(E10&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10632,7 +10644,7 @@
       <x:c r="C11" s="20"/>
       <x:c r="D11" s="21"/>
       <x:c r="E11" s="21" t="str">
-        <x:f>IF(A11="","",IF(D11="","Available",SWITCH(C11,"Daily",D11+1,"Weekly",D11+7,"Monthly",EDATE(D11,1),"Quarterly",EDATE(D11,3),"Yearly",EDATE(D11,12),"One-time","Used","Manual","Manual",D11)))</x:f>
+        <x:f>IF(A11="","",IF(D11="","Available",SWITCH(C11,"Daily",D11+1,"Weekly",IFERROR(VLOOKUP(A11,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D11-VLOOKUP(A11,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D11+7),"Monthly",IFERROR(EDATE(VLOOKUP(A11,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A11,'VIP Signups'!$A$5:$B$204,2,FALSE),D11,"M")+1),EDATE(D11,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A11,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A11,'VIP Signups'!$A$5:$B$204,2,FALSE),D11,"M")/3)+1)*3),EDATE(D11,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A11,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A11,'VIP Signups'!$A$5:$B$204,2,FALSE),D11,"Y")+1)*12),EDATE(D11,12)),"One-time","Used","Manual","Manual",D11)))</x:f>
       </x:c>
       <x:c r="F11" s="20" t="str">
         <x:f>IF(A11="","",IF(D11="","Yes",IF(E11="Manual","Manual",IF(E11="Used","No",IF(E11&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10655,7 +10667,7 @@
       <x:c r="C12" s="20"/>
       <x:c r="D12" s="21"/>
       <x:c r="E12" s="21" t="str">
-        <x:f>IF(A12="","",IF(D12="","Available",SWITCH(C12,"Daily",D12+1,"Weekly",D12+7,"Monthly",EDATE(D12,1),"Quarterly",EDATE(D12,3),"Yearly",EDATE(D12,12),"One-time","Used","Manual","Manual",D12)))</x:f>
+        <x:f>IF(A12="","",IF(D12="","Available",SWITCH(C12,"Daily",D12+1,"Weekly",IFERROR(VLOOKUP(A12,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D12-VLOOKUP(A12,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D12+7),"Monthly",IFERROR(EDATE(VLOOKUP(A12,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A12,'VIP Signups'!$A$5:$B$204,2,FALSE),D12,"M")+1),EDATE(D12,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A12,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A12,'VIP Signups'!$A$5:$B$204,2,FALSE),D12,"M")/3)+1)*3),EDATE(D12,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A12,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A12,'VIP Signups'!$A$5:$B$204,2,FALSE),D12,"Y")+1)*12),EDATE(D12,12)),"One-time","Used","Manual","Manual",D12)))</x:f>
       </x:c>
       <x:c r="F12" s="20" t="str">
         <x:f>IF(A12="","",IF(D12="","Yes",IF(E12="Manual","Manual",IF(E12="Used","No",IF(E12&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10678,7 +10690,7 @@
       <x:c r="C13" s="20"/>
       <x:c r="D13" s="21"/>
       <x:c r="E13" s="21" t="str">
-        <x:f>IF(A13="","",IF(D13="","Available",SWITCH(C13,"Daily",D13+1,"Weekly",D13+7,"Monthly",EDATE(D13,1),"Quarterly",EDATE(D13,3),"Yearly",EDATE(D13,12),"One-time","Used","Manual","Manual",D13)))</x:f>
+        <x:f>IF(A13="","",IF(D13="","Available",SWITCH(C13,"Daily",D13+1,"Weekly",IFERROR(VLOOKUP(A13,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D13-VLOOKUP(A13,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D13+7),"Monthly",IFERROR(EDATE(VLOOKUP(A13,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A13,'VIP Signups'!$A$5:$B$204,2,FALSE),D13,"M")+1),EDATE(D13,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A13,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A13,'VIP Signups'!$A$5:$B$204,2,FALSE),D13,"M")/3)+1)*3),EDATE(D13,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A13,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A13,'VIP Signups'!$A$5:$B$204,2,FALSE),D13,"Y")+1)*12),EDATE(D13,12)),"One-time","Used","Manual","Manual",D13)))</x:f>
       </x:c>
       <x:c r="F13" s="20" t="str">
         <x:f>IF(A13="","",IF(D13="","Yes",IF(E13="Manual","Manual",IF(E13="Used","No",IF(E13&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10701,7 +10713,7 @@
       <x:c r="C14" s="20"/>
       <x:c r="D14" s="21"/>
       <x:c r="E14" s="21" t="str">
-        <x:f>IF(A14="","",IF(D14="","Available",SWITCH(C14,"Daily",D14+1,"Weekly",D14+7,"Monthly",EDATE(D14,1),"Quarterly",EDATE(D14,3),"Yearly",EDATE(D14,12),"One-time","Used","Manual","Manual",D14)))</x:f>
+        <x:f>IF(A14="","",IF(D14="","Available",SWITCH(C14,"Daily",D14+1,"Weekly",IFERROR(VLOOKUP(A14,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D14-VLOOKUP(A14,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D14+7),"Monthly",IFERROR(EDATE(VLOOKUP(A14,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A14,'VIP Signups'!$A$5:$B$204,2,FALSE),D14,"M")+1),EDATE(D14,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A14,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A14,'VIP Signups'!$A$5:$B$204,2,FALSE),D14,"M")/3)+1)*3),EDATE(D14,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A14,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A14,'VIP Signups'!$A$5:$B$204,2,FALSE),D14,"Y")+1)*12),EDATE(D14,12)),"One-time","Used","Manual","Manual",D14)))</x:f>
       </x:c>
       <x:c r="F14" s="20" t="str">
         <x:f>IF(A14="","",IF(D14="","Yes",IF(E14="Manual","Manual",IF(E14="Used","No",IF(E14&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10724,7 +10736,7 @@
       <x:c r="C15" s="20"/>
       <x:c r="D15" s="21"/>
       <x:c r="E15" s="21" t="str">
-        <x:f>IF(A15="","",IF(D15="","Available",SWITCH(C15,"Daily",D15+1,"Weekly",D15+7,"Monthly",EDATE(D15,1),"Quarterly",EDATE(D15,3),"Yearly",EDATE(D15,12),"One-time","Used","Manual","Manual",D15)))</x:f>
+        <x:f>IF(A15="","",IF(D15="","Available",SWITCH(C15,"Daily",D15+1,"Weekly",IFERROR(VLOOKUP(A15,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D15-VLOOKUP(A15,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D15+7),"Monthly",IFERROR(EDATE(VLOOKUP(A15,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A15,'VIP Signups'!$A$5:$B$204,2,FALSE),D15,"M")+1),EDATE(D15,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A15,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A15,'VIP Signups'!$A$5:$B$204,2,FALSE),D15,"M")/3)+1)*3),EDATE(D15,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A15,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A15,'VIP Signups'!$A$5:$B$204,2,FALSE),D15,"Y")+1)*12),EDATE(D15,12)),"One-time","Used","Manual","Manual",D15)))</x:f>
       </x:c>
       <x:c r="F15" s="20" t="str">
         <x:f>IF(A15="","",IF(D15="","Yes",IF(E15="Manual","Manual",IF(E15="Used","No",IF(E15&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10747,7 +10759,7 @@
       <x:c r="C16" s="20"/>
       <x:c r="D16" s="21"/>
       <x:c r="E16" s="21" t="str">
-        <x:f>IF(A16="","",IF(D16="","Available",SWITCH(C16,"Daily",D16+1,"Weekly",D16+7,"Monthly",EDATE(D16,1),"Quarterly",EDATE(D16,3),"Yearly",EDATE(D16,12),"One-time","Used","Manual","Manual",D16)))</x:f>
+        <x:f>IF(A16="","",IF(D16="","Available",SWITCH(C16,"Daily",D16+1,"Weekly",IFERROR(VLOOKUP(A16,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D16-VLOOKUP(A16,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D16+7),"Monthly",IFERROR(EDATE(VLOOKUP(A16,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A16,'VIP Signups'!$A$5:$B$204,2,FALSE),D16,"M")+1),EDATE(D16,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A16,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A16,'VIP Signups'!$A$5:$B$204,2,FALSE),D16,"M")/3)+1)*3),EDATE(D16,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A16,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A16,'VIP Signups'!$A$5:$B$204,2,FALSE),D16,"Y")+1)*12),EDATE(D16,12)),"One-time","Used","Manual","Manual",D16)))</x:f>
       </x:c>
       <x:c r="F16" s="20" t="str">
         <x:f>IF(A16="","",IF(D16="","Yes",IF(E16="Manual","Manual",IF(E16="Used","No",IF(E16&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10770,7 +10782,7 @@
       <x:c r="C17" s="20"/>
       <x:c r="D17" s="21"/>
       <x:c r="E17" s="21" t="str">
-        <x:f>IF(A17="","",IF(D17="","Available",SWITCH(C17,"Daily",D17+1,"Weekly",D17+7,"Monthly",EDATE(D17,1),"Quarterly",EDATE(D17,3),"Yearly",EDATE(D17,12),"One-time","Used","Manual","Manual",D17)))</x:f>
+        <x:f>IF(A17="","",IF(D17="","Available",SWITCH(C17,"Daily",D17+1,"Weekly",IFERROR(VLOOKUP(A17,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D17-VLOOKUP(A17,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D17+7),"Monthly",IFERROR(EDATE(VLOOKUP(A17,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A17,'VIP Signups'!$A$5:$B$204,2,FALSE),D17,"M")+1),EDATE(D17,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A17,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A17,'VIP Signups'!$A$5:$B$204,2,FALSE),D17,"M")/3)+1)*3),EDATE(D17,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A17,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A17,'VIP Signups'!$A$5:$B$204,2,FALSE),D17,"Y")+1)*12),EDATE(D17,12)),"One-time","Used","Manual","Manual",D17)))</x:f>
       </x:c>
       <x:c r="F17" s="20" t="str">
         <x:f>IF(A17="","",IF(D17="","Yes",IF(E17="Manual","Manual",IF(E17="Used","No",IF(E17&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10793,7 +10805,7 @@
       <x:c r="C18" s="20"/>
       <x:c r="D18" s="21"/>
       <x:c r="E18" s="21" t="str">
-        <x:f>IF(A18="","",IF(D18="","Available",SWITCH(C18,"Daily",D18+1,"Weekly",D18+7,"Monthly",EDATE(D18,1),"Quarterly",EDATE(D18,3),"Yearly",EDATE(D18,12),"One-time","Used","Manual","Manual",D18)))</x:f>
+        <x:f>IF(A18="","",IF(D18="","Available",SWITCH(C18,"Daily",D18+1,"Weekly",IFERROR(VLOOKUP(A18,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D18-VLOOKUP(A18,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D18+7),"Monthly",IFERROR(EDATE(VLOOKUP(A18,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A18,'VIP Signups'!$A$5:$B$204,2,FALSE),D18,"M")+1),EDATE(D18,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A18,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A18,'VIP Signups'!$A$5:$B$204,2,FALSE),D18,"M")/3)+1)*3),EDATE(D18,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A18,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A18,'VIP Signups'!$A$5:$B$204,2,FALSE),D18,"Y")+1)*12),EDATE(D18,12)),"One-time","Used","Manual","Manual",D18)))</x:f>
       </x:c>
       <x:c r="F18" s="20" t="str">
         <x:f>IF(A18="","",IF(D18="","Yes",IF(E18="Manual","Manual",IF(E18="Used","No",IF(E18&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10816,7 +10828,7 @@
       <x:c r="C19" s="20"/>
       <x:c r="D19" s="21"/>
       <x:c r="E19" s="21" t="str">
-        <x:f>IF(A19="","",IF(D19="","Available",SWITCH(C19,"Daily",D19+1,"Weekly",D19+7,"Monthly",EDATE(D19,1),"Quarterly",EDATE(D19,3),"Yearly",EDATE(D19,12),"One-time","Used","Manual","Manual",D19)))</x:f>
+        <x:f>IF(A19="","",IF(D19="","Available",SWITCH(C19,"Daily",D19+1,"Weekly",IFERROR(VLOOKUP(A19,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D19-VLOOKUP(A19,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D19+7),"Monthly",IFERROR(EDATE(VLOOKUP(A19,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A19,'VIP Signups'!$A$5:$B$204,2,FALSE),D19,"M")+1),EDATE(D19,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A19,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A19,'VIP Signups'!$A$5:$B$204,2,FALSE),D19,"M")/3)+1)*3),EDATE(D19,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A19,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A19,'VIP Signups'!$A$5:$B$204,2,FALSE),D19,"Y")+1)*12),EDATE(D19,12)),"One-time","Used","Manual","Manual",D19)))</x:f>
       </x:c>
       <x:c r="F19" s="20" t="str">
         <x:f>IF(A19="","",IF(D19="","Yes",IF(E19="Manual","Manual",IF(E19="Used","No",IF(E19&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10839,7 +10851,7 @@
       <x:c r="C20" s="20"/>
       <x:c r="D20" s="21"/>
       <x:c r="E20" s="21" t="str">
-        <x:f>IF(A20="","",IF(D20="","Available",SWITCH(C20,"Daily",D20+1,"Weekly",D20+7,"Monthly",EDATE(D20,1),"Quarterly",EDATE(D20,3),"Yearly",EDATE(D20,12),"One-time","Used","Manual","Manual",D20)))</x:f>
+        <x:f>IF(A20="","",IF(D20="","Available",SWITCH(C20,"Daily",D20+1,"Weekly",IFERROR(VLOOKUP(A20,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D20-VLOOKUP(A20,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D20+7),"Monthly",IFERROR(EDATE(VLOOKUP(A20,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A20,'VIP Signups'!$A$5:$B$204,2,FALSE),D20,"M")+1),EDATE(D20,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A20,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A20,'VIP Signups'!$A$5:$B$204,2,FALSE),D20,"M")/3)+1)*3),EDATE(D20,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A20,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A20,'VIP Signups'!$A$5:$B$204,2,FALSE),D20,"Y")+1)*12),EDATE(D20,12)),"One-time","Used","Manual","Manual",D20)))</x:f>
       </x:c>
       <x:c r="F20" s="20" t="str">
         <x:f>IF(A20="","",IF(D20="","Yes",IF(E20="Manual","Manual",IF(E20="Used","No",IF(E20&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10862,7 +10874,7 @@
       <x:c r="C21" s="20"/>
       <x:c r="D21" s="21"/>
       <x:c r="E21" s="21" t="str">
-        <x:f>IF(A21="","",IF(D21="","Available",SWITCH(C21,"Daily",D21+1,"Weekly",D21+7,"Monthly",EDATE(D21,1),"Quarterly",EDATE(D21,3),"Yearly",EDATE(D21,12),"One-time","Used","Manual","Manual",D21)))</x:f>
+        <x:f>IF(A21="","",IF(D21="","Available",SWITCH(C21,"Daily",D21+1,"Weekly",IFERROR(VLOOKUP(A21,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D21-VLOOKUP(A21,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D21+7),"Monthly",IFERROR(EDATE(VLOOKUP(A21,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A21,'VIP Signups'!$A$5:$B$204,2,FALSE),D21,"M")+1),EDATE(D21,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A21,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A21,'VIP Signups'!$A$5:$B$204,2,FALSE),D21,"M")/3)+1)*3),EDATE(D21,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A21,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A21,'VIP Signups'!$A$5:$B$204,2,FALSE),D21,"Y")+1)*12),EDATE(D21,12)),"One-time","Used","Manual","Manual",D21)))</x:f>
       </x:c>
       <x:c r="F21" s="20" t="str">
         <x:f>IF(A21="","",IF(D21="","Yes",IF(E21="Manual","Manual",IF(E21="Used","No",IF(E21&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10885,7 +10897,7 @@
       <x:c r="C22" s="20"/>
       <x:c r="D22" s="21"/>
       <x:c r="E22" s="21" t="str">
-        <x:f>IF(A22="","",IF(D22="","Available",SWITCH(C22,"Daily",D22+1,"Weekly",D22+7,"Monthly",EDATE(D22,1),"Quarterly",EDATE(D22,3),"Yearly",EDATE(D22,12),"One-time","Used","Manual","Manual",D22)))</x:f>
+        <x:f>IF(A22="","",IF(D22="","Available",SWITCH(C22,"Daily",D22+1,"Weekly",IFERROR(VLOOKUP(A22,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D22-VLOOKUP(A22,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D22+7),"Monthly",IFERROR(EDATE(VLOOKUP(A22,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A22,'VIP Signups'!$A$5:$B$204,2,FALSE),D22,"M")+1),EDATE(D22,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A22,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A22,'VIP Signups'!$A$5:$B$204,2,FALSE),D22,"M")/3)+1)*3),EDATE(D22,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A22,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A22,'VIP Signups'!$A$5:$B$204,2,FALSE),D22,"Y")+1)*12),EDATE(D22,12)),"One-time","Used","Manual","Manual",D22)))</x:f>
       </x:c>
       <x:c r="F22" s="20" t="str">
         <x:f>IF(A22="","",IF(D22="","Yes",IF(E22="Manual","Manual",IF(E22="Used","No",IF(E22&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10908,7 +10920,7 @@
       <x:c r="C23" s="20"/>
       <x:c r="D23" s="21"/>
       <x:c r="E23" s="21" t="str">
-        <x:f>IF(A23="","",IF(D23="","Available",SWITCH(C23,"Daily",D23+1,"Weekly",D23+7,"Monthly",EDATE(D23,1),"Quarterly",EDATE(D23,3),"Yearly",EDATE(D23,12),"One-time","Used","Manual","Manual",D23)))</x:f>
+        <x:f>IF(A23="","",IF(D23="","Available",SWITCH(C23,"Daily",D23+1,"Weekly",IFERROR(VLOOKUP(A23,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D23-VLOOKUP(A23,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D23+7),"Monthly",IFERROR(EDATE(VLOOKUP(A23,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A23,'VIP Signups'!$A$5:$B$204,2,FALSE),D23,"M")+1),EDATE(D23,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A23,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A23,'VIP Signups'!$A$5:$B$204,2,FALSE),D23,"M")/3)+1)*3),EDATE(D23,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A23,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A23,'VIP Signups'!$A$5:$B$204,2,FALSE),D23,"Y")+1)*12),EDATE(D23,12)),"One-time","Used","Manual","Manual",D23)))</x:f>
       </x:c>
       <x:c r="F23" s="20" t="str">
         <x:f>IF(A23="","",IF(D23="","Yes",IF(E23="Manual","Manual",IF(E23="Used","No",IF(E23&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10931,7 +10943,7 @@
       <x:c r="C24" s="20"/>
       <x:c r="D24" s="21"/>
       <x:c r="E24" s="21" t="str">
-        <x:f>IF(A24="","",IF(D24="","Available",SWITCH(C24,"Daily",D24+1,"Weekly",D24+7,"Monthly",EDATE(D24,1),"Quarterly",EDATE(D24,3),"Yearly",EDATE(D24,12),"One-time","Used","Manual","Manual",D24)))</x:f>
+        <x:f>IF(A24="","",IF(D24="","Available",SWITCH(C24,"Daily",D24+1,"Weekly",IFERROR(VLOOKUP(A24,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D24-VLOOKUP(A24,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D24+7),"Monthly",IFERROR(EDATE(VLOOKUP(A24,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A24,'VIP Signups'!$A$5:$B$204,2,FALSE),D24,"M")+1),EDATE(D24,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A24,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A24,'VIP Signups'!$A$5:$B$204,2,FALSE),D24,"M")/3)+1)*3),EDATE(D24,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A24,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A24,'VIP Signups'!$A$5:$B$204,2,FALSE),D24,"Y")+1)*12),EDATE(D24,12)),"One-time","Used","Manual","Manual",D24)))</x:f>
       </x:c>
       <x:c r="F24" s="20" t="str">
         <x:f>IF(A24="","",IF(D24="","Yes",IF(E24="Manual","Manual",IF(E24="Used","No",IF(E24&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10954,7 +10966,7 @@
       <x:c r="C25" s="20"/>
       <x:c r="D25" s="21"/>
       <x:c r="E25" s="21" t="str">
-        <x:f>IF(A25="","",IF(D25="","Available",SWITCH(C25,"Daily",D25+1,"Weekly",D25+7,"Monthly",EDATE(D25,1),"Quarterly",EDATE(D25,3),"Yearly",EDATE(D25,12),"One-time","Used","Manual","Manual",D25)))</x:f>
+        <x:f>IF(A25="","",IF(D25="","Available",SWITCH(C25,"Daily",D25+1,"Weekly",IFERROR(VLOOKUP(A25,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D25-VLOOKUP(A25,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D25+7),"Monthly",IFERROR(EDATE(VLOOKUP(A25,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A25,'VIP Signups'!$A$5:$B$204,2,FALSE),D25,"M")+1),EDATE(D25,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A25,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A25,'VIP Signups'!$A$5:$B$204,2,FALSE),D25,"M")/3)+1)*3),EDATE(D25,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A25,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A25,'VIP Signups'!$A$5:$B$204,2,FALSE),D25,"Y")+1)*12),EDATE(D25,12)),"One-time","Used","Manual","Manual",D25)))</x:f>
       </x:c>
       <x:c r="F25" s="20" t="str">
         <x:f>IF(A25="","",IF(D25="","Yes",IF(E25="Manual","Manual",IF(E25="Used","No",IF(E25&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -10977,7 +10989,7 @@
       <x:c r="C26" s="20"/>
       <x:c r="D26" s="21"/>
       <x:c r="E26" s="21" t="str">
-        <x:f>IF(A26="","",IF(D26="","Available",SWITCH(C26,"Daily",D26+1,"Weekly",D26+7,"Monthly",EDATE(D26,1),"Quarterly",EDATE(D26,3),"Yearly",EDATE(D26,12),"One-time","Used","Manual","Manual",D26)))</x:f>
+        <x:f>IF(A26="","",IF(D26="","Available",SWITCH(C26,"Daily",D26+1,"Weekly",IFERROR(VLOOKUP(A26,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D26-VLOOKUP(A26,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D26+7),"Monthly",IFERROR(EDATE(VLOOKUP(A26,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A26,'VIP Signups'!$A$5:$B$204,2,FALSE),D26,"M")+1),EDATE(D26,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A26,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A26,'VIP Signups'!$A$5:$B$204,2,FALSE),D26,"M")/3)+1)*3),EDATE(D26,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A26,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A26,'VIP Signups'!$A$5:$B$204,2,FALSE),D26,"Y")+1)*12),EDATE(D26,12)),"One-time","Used","Manual","Manual",D26)))</x:f>
       </x:c>
       <x:c r="F26" s="20" t="str">
         <x:f>IF(A26="","",IF(D26="","Yes",IF(E26="Manual","Manual",IF(E26="Used","No",IF(E26&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11000,7 +11012,7 @@
       <x:c r="C27" s="20"/>
       <x:c r="D27" s="21"/>
       <x:c r="E27" s="21" t="str">
-        <x:f>IF(A27="","",IF(D27="","Available",SWITCH(C27,"Daily",D27+1,"Weekly",D27+7,"Monthly",EDATE(D27,1),"Quarterly",EDATE(D27,3),"Yearly",EDATE(D27,12),"One-time","Used","Manual","Manual",D27)))</x:f>
+        <x:f>IF(A27="","",IF(D27="","Available",SWITCH(C27,"Daily",D27+1,"Weekly",IFERROR(VLOOKUP(A27,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D27-VLOOKUP(A27,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D27+7),"Monthly",IFERROR(EDATE(VLOOKUP(A27,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A27,'VIP Signups'!$A$5:$B$204,2,FALSE),D27,"M")+1),EDATE(D27,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A27,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A27,'VIP Signups'!$A$5:$B$204,2,FALSE),D27,"M")/3)+1)*3),EDATE(D27,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A27,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A27,'VIP Signups'!$A$5:$B$204,2,FALSE),D27,"Y")+1)*12),EDATE(D27,12)),"One-time","Used","Manual","Manual",D27)))</x:f>
       </x:c>
       <x:c r="F27" s="20" t="str">
         <x:f>IF(A27="","",IF(D27="","Yes",IF(E27="Manual","Manual",IF(E27="Used","No",IF(E27&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11023,7 +11035,7 @@
       <x:c r="C28" s="20"/>
       <x:c r="D28" s="21"/>
       <x:c r="E28" s="21" t="str">
-        <x:f>IF(A28="","",IF(D28="","Available",SWITCH(C28,"Daily",D28+1,"Weekly",D28+7,"Monthly",EDATE(D28,1),"Quarterly",EDATE(D28,3),"Yearly",EDATE(D28,12),"One-time","Used","Manual","Manual",D28)))</x:f>
+        <x:f>IF(A28="","",IF(D28="","Available",SWITCH(C28,"Daily",D28+1,"Weekly",IFERROR(VLOOKUP(A28,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D28-VLOOKUP(A28,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D28+7),"Monthly",IFERROR(EDATE(VLOOKUP(A28,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A28,'VIP Signups'!$A$5:$B$204,2,FALSE),D28,"M")+1),EDATE(D28,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A28,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A28,'VIP Signups'!$A$5:$B$204,2,FALSE),D28,"M")/3)+1)*3),EDATE(D28,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A28,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A28,'VIP Signups'!$A$5:$B$204,2,FALSE),D28,"Y")+1)*12),EDATE(D28,12)),"One-time","Used","Manual","Manual",D28)))</x:f>
       </x:c>
       <x:c r="F28" s="20" t="str">
         <x:f>IF(A28="","",IF(D28="","Yes",IF(E28="Manual","Manual",IF(E28="Used","No",IF(E28&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11046,7 +11058,7 @@
       <x:c r="C29" s="20"/>
       <x:c r="D29" s="21"/>
       <x:c r="E29" s="21" t="str">
-        <x:f>IF(A29="","",IF(D29="","Available",SWITCH(C29,"Daily",D29+1,"Weekly",D29+7,"Monthly",EDATE(D29,1),"Quarterly",EDATE(D29,3),"Yearly",EDATE(D29,12),"One-time","Used","Manual","Manual",D29)))</x:f>
+        <x:f>IF(A29="","",IF(D29="","Available",SWITCH(C29,"Daily",D29+1,"Weekly",IFERROR(VLOOKUP(A29,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D29-VLOOKUP(A29,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D29+7),"Monthly",IFERROR(EDATE(VLOOKUP(A29,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A29,'VIP Signups'!$A$5:$B$204,2,FALSE),D29,"M")+1),EDATE(D29,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A29,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A29,'VIP Signups'!$A$5:$B$204,2,FALSE),D29,"M")/3)+1)*3),EDATE(D29,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A29,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A29,'VIP Signups'!$A$5:$B$204,2,FALSE),D29,"Y")+1)*12),EDATE(D29,12)),"One-time","Used","Manual","Manual",D29)))</x:f>
       </x:c>
       <x:c r="F29" s="20" t="str">
         <x:f>IF(A29="","",IF(D29="","Yes",IF(E29="Manual","Manual",IF(E29="Used","No",IF(E29&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11069,7 +11081,7 @@
       <x:c r="C30" s="20"/>
       <x:c r="D30" s="21"/>
       <x:c r="E30" s="21" t="str">
-        <x:f>IF(A30="","",IF(D30="","Available",SWITCH(C30,"Daily",D30+1,"Weekly",D30+7,"Monthly",EDATE(D30,1),"Quarterly",EDATE(D30,3),"Yearly",EDATE(D30,12),"One-time","Used","Manual","Manual",D30)))</x:f>
+        <x:f>IF(A30="","",IF(D30="","Available",SWITCH(C30,"Daily",D30+1,"Weekly",IFERROR(VLOOKUP(A30,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D30-VLOOKUP(A30,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D30+7),"Monthly",IFERROR(EDATE(VLOOKUP(A30,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A30,'VIP Signups'!$A$5:$B$204,2,FALSE),D30,"M")+1),EDATE(D30,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A30,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A30,'VIP Signups'!$A$5:$B$204,2,FALSE),D30,"M")/3)+1)*3),EDATE(D30,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A30,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A30,'VIP Signups'!$A$5:$B$204,2,FALSE),D30,"Y")+1)*12),EDATE(D30,12)),"One-time","Used","Manual","Manual",D30)))</x:f>
       </x:c>
       <x:c r="F30" s="20" t="str">
         <x:f>IF(A30="","",IF(D30="","Yes",IF(E30="Manual","Manual",IF(E30="Used","No",IF(E30&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11092,7 +11104,7 @@
       <x:c r="C31" s="20"/>
       <x:c r="D31" s="21"/>
       <x:c r="E31" s="21" t="str">
-        <x:f>IF(A31="","",IF(D31="","Available",SWITCH(C31,"Daily",D31+1,"Weekly",D31+7,"Monthly",EDATE(D31,1),"Quarterly",EDATE(D31,3),"Yearly",EDATE(D31,12),"One-time","Used","Manual","Manual",D31)))</x:f>
+        <x:f>IF(A31="","",IF(D31="","Available",SWITCH(C31,"Daily",D31+1,"Weekly",IFERROR(VLOOKUP(A31,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D31-VLOOKUP(A31,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D31+7),"Monthly",IFERROR(EDATE(VLOOKUP(A31,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A31,'VIP Signups'!$A$5:$B$204,2,FALSE),D31,"M")+1),EDATE(D31,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A31,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A31,'VIP Signups'!$A$5:$B$204,2,FALSE),D31,"M")/3)+1)*3),EDATE(D31,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A31,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A31,'VIP Signups'!$A$5:$B$204,2,FALSE),D31,"Y")+1)*12),EDATE(D31,12)),"One-time","Used","Manual","Manual",D31)))</x:f>
       </x:c>
       <x:c r="F31" s="20" t="str">
         <x:f>IF(A31="","",IF(D31="","Yes",IF(E31="Manual","Manual",IF(E31="Used","No",IF(E31&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11115,7 +11127,7 @@
       <x:c r="C32" s="20"/>
       <x:c r="D32" s="21"/>
       <x:c r="E32" s="21" t="str">
-        <x:f>IF(A32="","",IF(D32="","Available",SWITCH(C32,"Daily",D32+1,"Weekly",D32+7,"Monthly",EDATE(D32,1),"Quarterly",EDATE(D32,3),"Yearly",EDATE(D32,12),"One-time","Used","Manual","Manual",D32)))</x:f>
+        <x:f>IF(A32="","",IF(D32="","Available",SWITCH(C32,"Daily",D32+1,"Weekly",IFERROR(VLOOKUP(A32,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D32-VLOOKUP(A32,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D32+7),"Monthly",IFERROR(EDATE(VLOOKUP(A32,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A32,'VIP Signups'!$A$5:$B$204,2,FALSE),D32,"M")+1),EDATE(D32,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A32,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A32,'VIP Signups'!$A$5:$B$204,2,FALSE),D32,"M")/3)+1)*3),EDATE(D32,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A32,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A32,'VIP Signups'!$A$5:$B$204,2,FALSE),D32,"Y")+1)*12),EDATE(D32,12)),"One-time","Used","Manual","Manual",D32)))</x:f>
       </x:c>
       <x:c r="F32" s="20" t="str">
         <x:f>IF(A32="","",IF(D32="","Yes",IF(E32="Manual","Manual",IF(E32="Used","No",IF(E32&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11138,7 +11150,7 @@
       <x:c r="C33" s="20"/>
       <x:c r="D33" s="21"/>
       <x:c r="E33" s="21" t="str">
-        <x:f>IF(A33="","",IF(D33="","Available",SWITCH(C33,"Daily",D33+1,"Weekly",D33+7,"Monthly",EDATE(D33,1),"Quarterly",EDATE(D33,3),"Yearly",EDATE(D33,12),"One-time","Used","Manual","Manual",D33)))</x:f>
+        <x:f>IF(A33="","",IF(D33="","Available",SWITCH(C33,"Daily",D33+1,"Weekly",IFERROR(VLOOKUP(A33,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D33-VLOOKUP(A33,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D33+7),"Monthly",IFERROR(EDATE(VLOOKUP(A33,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A33,'VIP Signups'!$A$5:$B$204,2,FALSE),D33,"M")+1),EDATE(D33,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A33,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A33,'VIP Signups'!$A$5:$B$204,2,FALSE),D33,"M")/3)+1)*3),EDATE(D33,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A33,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A33,'VIP Signups'!$A$5:$B$204,2,FALSE),D33,"Y")+1)*12),EDATE(D33,12)),"One-time","Used","Manual","Manual",D33)))</x:f>
       </x:c>
       <x:c r="F33" s="20" t="str">
         <x:f>IF(A33="","",IF(D33="","Yes",IF(E33="Manual","Manual",IF(E33="Used","No",IF(E33&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11161,7 +11173,7 @@
       <x:c r="C34" s="20"/>
       <x:c r="D34" s="21"/>
       <x:c r="E34" s="21" t="str">
-        <x:f>IF(A34="","",IF(D34="","Available",SWITCH(C34,"Daily",D34+1,"Weekly",D34+7,"Monthly",EDATE(D34,1),"Quarterly",EDATE(D34,3),"Yearly",EDATE(D34,12),"One-time","Used","Manual","Manual",D34)))</x:f>
+        <x:f>IF(A34="","",IF(D34="","Available",SWITCH(C34,"Daily",D34+1,"Weekly",IFERROR(VLOOKUP(A34,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D34-VLOOKUP(A34,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D34+7),"Monthly",IFERROR(EDATE(VLOOKUP(A34,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A34,'VIP Signups'!$A$5:$B$204,2,FALSE),D34,"M")+1),EDATE(D34,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A34,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A34,'VIP Signups'!$A$5:$B$204,2,FALSE),D34,"M")/3)+1)*3),EDATE(D34,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A34,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A34,'VIP Signups'!$A$5:$B$204,2,FALSE),D34,"Y")+1)*12),EDATE(D34,12)),"One-time","Used","Manual","Manual",D34)))</x:f>
       </x:c>
       <x:c r="F34" s="20" t="str">
         <x:f>IF(A34="","",IF(D34="","Yes",IF(E34="Manual","Manual",IF(E34="Used","No",IF(E34&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11184,7 +11196,7 @@
       <x:c r="C35" s="20"/>
       <x:c r="D35" s="21"/>
       <x:c r="E35" s="21" t="str">
-        <x:f>IF(A35="","",IF(D35="","Available",SWITCH(C35,"Daily",D35+1,"Weekly",D35+7,"Monthly",EDATE(D35,1),"Quarterly",EDATE(D35,3),"Yearly",EDATE(D35,12),"One-time","Used","Manual","Manual",D35)))</x:f>
+        <x:f>IF(A35="","",IF(D35="","Available",SWITCH(C35,"Daily",D35+1,"Weekly",IFERROR(VLOOKUP(A35,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D35-VLOOKUP(A35,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D35+7),"Monthly",IFERROR(EDATE(VLOOKUP(A35,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A35,'VIP Signups'!$A$5:$B$204,2,FALSE),D35,"M")+1),EDATE(D35,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A35,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A35,'VIP Signups'!$A$5:$B$204,2,FALSE),D35,"M")/3)+1)*3),EDATE(D35,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A35,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A35,'VIP Signups'!$A$5:$B$204,2,FALSE),D35,"Y")+1)*12),EDATE(D35,12)),"One-time","Used","Manual","Manual",D35)))</x:f>
       </x:c>
       <x:c r="F35" s="20" t="str">
         <x:f>IF(A35="","",IF(D35="","Yes",IF(E35="Manual","Manual",IF(E35="Used","No",IF(E35&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11207,7 +11219,7 @@
       <x:c r="C36" s="20"/>
       <x:c r="D36" s="21"/>
       <x:c r="E36" s="21" t="str">
-        <x:f>IF(A36="","",IF(D36="","Available",SWITCH(C36,"Daily",D36+1,"Weekly",D36+7,"Monthly",EDATE(D36,1),"Quarterly",EDATE(D36,3),"Yearly",EDATE(D36,12),"One-time","Used","Manual","Manual",D36)))</x:f>
+        <x:f>IF(A36="","",IF(D36="","Available",SWITCH(C36,"Daily",D36+1,"Weekly",IFERROR(VLOOKUP(A36,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D36-VLOOKUP(A36,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D36+7),"Monthly",IFERROR(EDATE(VLOOKUP(A36,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A36,'VIP Signups'!$A$5:$B$204,2,FALSE),D36,"M")+1),EDATE(D36,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A36,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A36,'VIP Signups'!$A$5:$B$204,2,FALSE),D36,"M")/3)+1)*3),EDATE(D36,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A36,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A36,'VIP Signups'!$A$5:$B$204,2,FALSE),D36,"Y")+1)*12),EDATE(D36,12)),"One-time","Used","Manual","Manual",D36)))</x:f>
       </x:c>
       <x:c r="F36" s="20" t="str">
         <x:f>IF(A36="","",IF(D36="","Yes",IF(E36="Manual","Manual",IF(E36="Used","No",IF(E36&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11230,7 +11242,7 @@
       <x:c r="C37" s="20"/>
       <x:c r="D37" s="21"/>
       <x:c r="E37" s="21" t="str">
-        <x:f>IF(A37="","",IF(D37="","Available",SWITCH(C37,"Daily",D37+1,"Weekly",D37+7,"Monthly",EDATE(D37,1),"Quarterly",EDATE(D37,3),"Yearly",EDATE(D37,12),"One-time","Used","Manual","Manual",D37)))</x:f>
+        <x:f>IF(A37="","",IF(D37="","Available",SWITCH(C37,"Daily",D37+1,"Weekly",IFERROR(VLOOKUP(A37,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D37-VLOOKUP(A37,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D37+7),"Monthly",IFERROR(EDATE(VLOOKUP(A37,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A37,'VIP Signups'!$A$5:$B$204,2,FALSE),D37,"M")+1),EDATE(D37,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A37,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A37,'VIP Signups'!$A$5:$B$204,2,FALSE),D37,"M")/3)+1)*3),EDATE(D37,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A37,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A37,'VIP Signups'!$A$5:$B$204,2,FALSE),D37,"Y")+1)*12),EDATE(D37,12)),"One-time","Used","Manual","Manual",D37)))</x:f>
       </x:c>
       <x:c r="F37" s="20" t="str">
         <x:f>IF(A37="","",IF(D37="","Yes",IF(E37="Manual","Manual",IF(E37="Used","No",IF(E37&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11253,7 +11265,7 @@
       <x:c r="C38" s="20"/>
       <x:c r="D38" s="21"/>
       <x:c r="E38" s="21" t="str">
-        <x:f>IF(A38="","",IF(D38="","Available",SWITCH(C38,"Daily",D38+1,"Weekly",D38+7,"Monthly",EDATE(D38,1),"Quarterly",EDATE(D38,3),"Yearly",EDATE(D38,12),"One-time","Used","Manual","Manual",D38)))</x:f>
+        <x:f>IF(A38="","",IF(D38="","Available",SWITCH(C38,"Daily",D38+1,"Weekly",IFERROR(VLOOKUP(A38,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D38-VLOOKUP(A38,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D38+7),"Monthly",IFERROR(EDATE(VLOOKUP(A38,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A38,'VIP Signups'!$A$5:$B$204,2,FALSE),D38,"M")+1),EDATE(D38,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A38,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A38,'VIP Signups'!$A$5:$B$204,2,FALSE),D38,"M")/3)+1)*3),EDATE(D38,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A38,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A38,'VIP Signups'!$A$5:$B$204,2,FALSE),D38,"Y")+1)*12),EDATE(D38,12)),"One-time","Used","Manual","Manual",D38)))</x:f>
       </x:c>
       <x:c r="F38" s="20" t="str">
         <x:f>IF(A38="","",IF(D38="","Yes",IF(E38="Manual","Manual",IF(E38="Used","No",IF(E38&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11276,7 +11288,7 @@
       <x:c r="C39" s="20"/>
       <x:c r="D39" s="21"/>
       <x:c r="E39" s="21" t="str">
-        <x:f>IF(A39="","",IF(D39="","Available",SWITCH(C39,"Daily",D39+1,"Weekly",D39+7,"Monthly",EDATE(D39,1),"Quarterly",EDATE(D39,3),"Yearly",EDATE(D39,12),"One-time","Used","Manual","Manual",D39)))</x:f>
+        <x:f>IF(A39="","",IF(D39="","Available",SWITCH(C39,"Daily",D39+1,"Weekly",IFERROR(VLOOKUP(A39,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D39-VLOOKUP(A39,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D39+7),"Monthly",IFERROR(EDATE(VLOOKUP(A39,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A39,'VIP Signups'!$A$5:$B$204,2,FALSE),D39,"M")+1),EDATE(D39,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A39,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A39,'VIP Signups'!$A$5:$B$204,2,FALSE),D39,"M")/3)+1)*3),EDATE(D39,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A39,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A39,'VIP Signups'!$A$5:$B$204,2,FALSE),D39,"Y")+1)*12),EDATE(D39,12)),"One-time","Used","Manual","Manual",D39)))</x:f>
       </x:c>
       <x:c r="F39" s="20" t="str">
         <x:f>IF(A39="","",IF(D39="","Yes",IF(E39="Manual","Manual",IF(E39="Used","No",IF(E39&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11299,7 +11311,7 @@
       <x:c r="C40" s="20"/>
       <x:c r="D40" s="21"/>
       <x:c r="E40" s="21" t="str">
-        <x:f>IF(A40="","",IF(D40="","Available",SWITCH(C40,"Daily",D40+1,"Weekly",D40+7,"Monthly",EDATE(D40,1),"Quarterly",EDATE(D40,3),"Yearly",EDATE(D40,12),"One-time","Used","Manual","Manual",D40)))</x:f>
+        <x:f>IF(A40="","",IF(D40="","Available",SWITCH(C40,"Daily",D40+1,"Weekly",IFERROR(VLOOKUP(A40,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D40-VLOOKUP(A40,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D40+7),"Monthly",IFERROR(EDATE(VLOOKUP(A40,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A40,'VIP Signups'!$A$5:$B$204,2,FALSE),D40,"M")+1),EDATE(D40,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A40,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A40,'VIP Signups'!$A$5:$B$204,2,FALSE),D40,"M")/3)+1)*3),EDATE(D40,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A40,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A40,'VIP Signups'!$A$5:$B$204,2,FALSE),D40,"Y")+1)*12),EDATE(D40,12)),"One-time","Used","Manual","Manual",D40)))</x:f>
       </x:c>
       <x:c r="F40" s="20" t="str">
         <x:f>IF(A40="","",IF(D40="","Yes",IF(E40="Manual","Manual",IF(E40="Used","No",IF(E40&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11322,7 +11334,7 @@
       <x:c r="C41" s="20"/>
       <x:c r="D41" s="21"/>
       <x:c r="E41" s="21" t="str">
-        <x:f>IF(A41="","",IF(D41="","Available",SWITCH(C41,"Daily",D41+1,"Weekly",D41+7,"Monthly",EDATE(D41,1),"Quarterly",EDATE(D41,3),"Yearly",EDATE(D41,12),"One-time","Used","Manual","Manual",D41)))</x:f>
+        <x:f>IF(A41="","",IF(D41="","Available",SWITCH(C41,"Daily",D41+1,"Weekly",IFERROR(VLOOKUP(A41,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D41-VLOOKUP(A41,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D41+7),"Monthly",IFERROR(EDATE(VLOOKUP(A41,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A41,'VIP Signups'!$A$5:$B$204,2,FALSE),D41,"M")+1),EDATE(D41,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A41,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A41,'VIP Signups'!$A$5:$B$204,2,FALSE),D41,"M")/3)+1)*3),EDATE(D41,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A41,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A41,'VIP Signups'!$A$5:$B$204,2,FALSE),D41,"Y")+1)*12),EDATE(D41,12)),"One-time","Used","Manual","Manual",D41)))</x:f>
       </x:c>
       <x:c r="F41" s="20" t="str">
         <x:f>IF(A41="","",IF(D41="","Yes",IF(E41="Manual","Manual",IF(E41="Used","No",IF(E41&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11345,7 +11357,7 @@
       <x:c r="C42" s="20"/>
       <x:c r="D42" s="21"/>
       <x:c r="E42" s="21" t="str">
-        <x:f>IF(A42="","",IF(D42="","Available",SWITCH(C42,"Daily",D42+1,"Weekly",D42+7,"Monthly",EDATE(D42,1),"Quarterly",EDATE(D42,3),"Yearly",EDATE(D42,12),"One-time","Used","Manual","Manual",D42)))</x:f>
+        <x:f>IF(A42="","",IF(D42="","Available",SWITCH(C42,"Daily",D42+1,"Weekly",IFERROR(VLOOKUP(A42,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D42-VLOOKUP(A42,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D42+7),"Monthly",IFERROR(EDATE(VLOOKUP(A42,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A42,'VIP Signups'!$A$5:$B$204,2,FALSE),D42,"M")+1),EDATE(D42,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A42,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A42,'VIP Signups'!$A$5:$B$204,2,FALSE),D42,"M")/3)+1)*3),EDATE(D42,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A42,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A42,'VIP Signups'!$A$5:$B$204,2,FALSE),D42,"Y")+1)*12),EDATE(D42,12)),"One-time","Used","Manual","Manual",D42)))</x:f>
       </x:c>
       <x:c r="F42" s="20" t="str">
         <x:f>IF(A42="","",IF(D42="","Yes",IF(E42="Manual","Manual",IF(E42="Used","No",IF(E42&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11368,7 +11380,7 @@
       <x:c r="C43" s="20"/>
       <x:c r="D43" s="21"/>
       <x:c r="E43" s="21" t="str">
-        <x:f>IF(A43="","",IF(D43="","Available",SWITCH(C43,"Daily",D43+1,"Weekly",D43+7,"Monthly",EDATE(D43,1),"Quarterly",EDATE(D43,3),"Yearly",EDATE(D43,12),"One-time","Used","Manual","Manual",D43)))</x:f>
+        <x:f>IF(A43="","",IF(D43="","Available",SWITCH(C43,"Daily",D43+1,"Weekly",IFERROR(VLOOKUP(A43,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D43-VLOOKUP(A43,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D43+7),"Monthly",IFERROR(EDATE(VLOOKUP(A43,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A43,'VIP Signups'!$A$5:$B$204,2,FALSE),D43,"M")+1),EDATE(D43,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A43,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A43,'VIP Signups'!$A$5:$B$204,2,FALSE),D43,"M")/3)+1)*3),EDATE(D43,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A43,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A43,'VIP Signups'!$A$5:$B$204,2,FALSE),D43,"Y")+1)*12),EDATE(D43,12)),"One-time","Used","Manual","Manual",D43)))</x:f>
       </x:c>
       <x:c r="F43" s="20" t="str">
         <x:f>IF(A43="","",IF(D43="","Yes",IF(E43="Manual","Manual",IF(E43="Used","No",IF(E43&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11391,7 +11403,7 @@
       <x:c r="C44" s="20"/>
       <x:c r="D44" s="21"/>
       <x:c r="E44" s="21" t="str">
-        <x:f>IF(A44="","",IF(D44="","Available",SWITCH(C44,"Daily",D44+1,"Weekly",D44+7,"Monthly",EDATE(D44,1),"Quarterly",EDATE(D44,3),"Yearly",EDATE(D44,12),"One-time","Used","Manual","Manual",D44)))</x:f>
+        <x:f>IF(A44="","",IF(D44="","Available",SWITCH(C44,"Daily",D44+1,"Weekly",IFERROR(VLOOKUP(A44,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D44-VLOOKUP(A44,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D44+7),"Monthly",IFERROR(EDATE(VLOOKUP(A44,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A44,'VIP Signups'!$A$5:$B$204,2,FALSE),D44,"M")+1),EDATE(D44,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A44,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A44,'VIP Signups'!$A$5:$B$204,2,FALSE),D44,"M")/3)+1)*3),EDATE(D44,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A44,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A44,'VIP Signups'!$A$5:$B$204,2,FALSE),D44,"Y")+1)*12),EDATE(D44,12)),"One-time","Used","Manual","Manual",D44)))</x:f>
       </x:c>
       <x:c r="F44" s="20" t="str">
         <x:f>IF(A44="","",IF(D44="","Yes",IF(E44="Manual","Manual",IF(E44="Used","No",IF(E44&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11414,7 +11426,7 @@
       <x:c r="C45" s="20"/>
       <x:c r="D45" s="21"/>
       <x:c r="E45" s="21" t="str">
-        <x:f>IF(A45="","",IF(D45="","Available",SWITCH(C45,"Daily",D45+1,"Weekly",D45+7,"Monthly",EDATE(D45,1),"Quarterly",EDATE(D45,3),"Yearly",EDATE(D45,12),"One-time","Used","Manual","Manual",D45)))</x:f>
+        <x:f>IF(A45="","",IF(D45="","Available",SWITCH(C45,"Daily",D45+1,"Weekly",IFERROR(VLOOKUP(A45,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D45-VLOOKUP(A45,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D45+7),"Monthly",IFERROR(EDATE(VLOOKUP(A45,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A45,'VIP Signups'!$A$5:$B$204,2,FALSE),D45,"M")+1),EDATE(D45,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A45,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A45,'VIP Signups'!$A$5:$B$204,2,FALSE),D45,"M")/3)+1)*3),EDATE(D45,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A45,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A45,'VIP Signups'!$A$5:$B$204,2,FALSE),D45,"Y")+1)*12),EDATE(D45,12)),"One-time","Used","Manual","Manual",D45)))</x:f>
       </x:c>
       <x:c r="F45" s="20" t="str">
         <x:f>IF(A45="","",IF(D45="","Yes",IF(E45="Manual","Manual",IF(E45="Used","No",IF(E45&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11437,7 +11449,7 @@
       <x:c r="C46" s="20"/>
       <x:c r="D46" s="21"/>
       <x:c r="E46" s="21" t="str">
-        <x:f>IF(A46="","",IF(D46="","Available",SWITCH(C46,"Daily",D46+1,"Weekly",D46+7,"Monthly",EDATE(D46,1),"Quarterly",EDATE(D46,3),"Yearly",EDATE(D46,12),"One-time","Used","Manual","Manual",D46)))</x:f>
+        <x:f>IF(A46="","",IF(D46="","Available",SWITCH(C46,"Daily",D46+1,"Weekly",IFERROR(VLOOKUP(A46,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D46-VLOOKUP(A46,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D46+7),"Monthly",IFERROR(EDATE(VLOOKUP(A46,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A46,'VIP Signups'!$A$5:$B$204,2,FALSE),D46,"M")+1),EDATE(D46,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A46,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A46,'VIP Signups'!$A$5:$B$204,2,FALSE),D46,"M")/3)+1)*3),EDATE(D46,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A46,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A46,'VIP Signups'!$A$5:$B$204,2,FALSE),D46,"Y")+1)*12),EDATE(D46,12)),"One-time","Used","Manual","Manual",D46)))</x:f>
       </x:c>
       <x:c r="F46" s="20" t="str">
         <x:f>IF(A46="","",IF(D46="","Yes",IF(E46="Manual","Manual",IF(E46="Used","No",IF(E46&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11460,7 +11472,7 @@
       <x:c r="C47" s="20"/>
       <x:c r="D47" s="21"/>
       <x:c r="E47" s="21" t="str">
-        <x:f>IF(A47="","",IF(D47="","Available",SWITCH(C47,"Daily",D47+1,"Weekly",D47+7,"Monthly",EDATE(D47,1),"Quarterly",EDATE(D47,3),"Yearly",EDATE(D47,12),"One-time","Used","Manual","Manual",D47)))</x:f>
+        <x:f>IF(A47="","",IF(D47="","Available",SWITCH(C47,"Daily",D47+1,"Weekly",IFERROR(VLOOKUP(A47,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D47-VLOOKUP(A47,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D47+7),"Monthly",IFERROR(EDATE(VLOOKUP(A47,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A47,'VIP Signups'!$A$5:$B$204,2,FALSE),D47,"M")+1),EDATE(D47,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A47,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A47,'VIP Signups'!$A$5:$B$204,2,FALSE),D47,"M")/3)+1)*3),EDATE(D47,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A47,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A47,'VIP Signups'!$A$5:$B$204,2,FALSE),D47,"Y")+1)*12),EDATE(D47,12)),"One-time","Used","Manual","Manual",D47)))</x:f>
       </x:c>
       <x:c r="F47" s="20" t="str">
         <x:f>IF(A47="","",IF(D47="","Yes",IF(E47="Manual","Manual",IF(E47="Used","No",IF(E47&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11483,7 +11495,7 @@
       <x:c r="C48" s="20"/>
       <x:c r="D48" s="21"/>
       <x:c r="E48" s="21" t="str">
-        <x:f>IF(A48="","",IF(D48="","Available",SWITCH(C48,"Daily",D48+1,"Weekly",D48+7,"Monthly",EDATE(D48,1),"Quarterly",EDATE(D48,3),"Yearly",EDATE(D48,12),"One-time","Used","Manual","Manual",D48)))</x:f>
+        <x:f>IF(A48="","",IF(D48="","Available",SWITCH(C48,"Daily",D48+1,"Weekly",IFERROR(VLOOKUP(A48,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D48-VLOOKUP(A48,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D48+7),"Monthly",IFERROR(EDATE(VLOOKUP(A48,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A48,'VIP Signups'!$A$5:$B$204,2,FALSE),D48,"M")+1),EDATE(D48,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A48,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A48,'VIP Signups'!$A$5:$B$204,2,FALSE),D48,"M")/3)+1)*3),EDATE(D48,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A48,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A48,'VIP Signups'!$A$5:$B$204,2,FALSE),D48,"Y")+1)*12),EDATE(D48,12)),"One-time","Used","Manual","Manual",D48)))</x:f>
       </x:c>
       <x:c r="F48" s="20" t="str">
         <x:f>IF(A48="","",IF(D48="","Yes",IF(E48="Manual","Manual",IF(E48="Used","No",IF(E48&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11506,7 +11518,7 @@
       <x:c r="C49" s="20"/>
       <x:c r="D49" s="21"/>
       <x:c r="E49" s="21" t="str">
-        <x:f>IF(A49="","",IF(D49="","Available",SWITCH(C49,"Daily",D49+1,"Weekly",D49+7,"Monthly",EDATE(D49,1),"Quarterly",EDATE(D49,3),"Yearly",EDATE(D49,12),"One-time","Used","Manual","Manual",D49)))</x:f>
+        <x:f>IF(A49="","",IF(D49="","Available",SWITCH(C49,"Daily",D49+1,"Weekly",IFERROR(VLOOKUP(A49,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D49-VLOOKUP(A49,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D49+7),"Monthly",IFERROR(EDATE(VLOOKUP(A49,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A49,'VIP Signups'!$A$5:$B$204,2,FALSE),D49,"M")+1),EDATE(D49,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A49,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A49,'VIP Signups'!$A$5:$B$204,2,FALSE),D49,"M")/3)+1)*3),EDATE(D49,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A49,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A49,'VIP Signups'!$A$5:$B$204,2,FALSE),D49,"Y")+1)*12),EDATE(D49,12)),"One-time","Used","Manual","Manual",D49)))</x:f>
       </x:c>
       <x:c r="F49" s="20" t="str">
         <x:f>IF(A49="","",IF(D49="","Yes",IF(E49="Manual","Manual",IF(E49="Used","No",IF(E49&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11529,7 +11541,7 @@
       <x:c r="C50" s="20"/>
       <x:c r="D50" s="21"/>
       <x:c r="E50" s="21" t="str">
-        <x:f>IF(A50="","",IF(D50="","Available",SWITCH(C50,"Daily",D50+1,"Weekly",D50+7,"Monthly",EDATE(D50,1),"Quarterly",EDATE(D50,3),"Yearly",EDATE(D50,12),"One-time","Used","Manual","Manual",D50)))</x:f>
+        <x:f>IF(A50="","",IF(D50="","Available",SWITCH(C50,"Daily",D50+1,"Weekly",IFERROR(VLOOKUP(A50,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D50-VLOOKUP(A50,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D50+7),"Monthly",IFERROR(EDATE(VLOOKUP(A50,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A50,'VIP Signups'!$A$5:$B$204,2,FALSE),D50,"M")+1),EDATE(D50,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A50,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A50,'VIP Signups'!$A$5:$B$204,2,FALSE),D50,"M")/3)+1)*3),EDATE(D50,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A50,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A50,'VIP Signups'!$A$5:$B$204,2,FALSE),D50,"Y")+1)*12),EDATE(D50,12)),"One-time","Used","Manual","Manual",D50)))</x:f>
       </x:c>
       <x:c r="F50" s="20" t="str">
         <x:f>IF(A50="","",IF(D50="","Yes",IF(E50="Manual","Manual",IF(E50="Used","No",IF(E50&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11552,7 +11564,7 @@
       <x:c r="C51" s="20"/>
       <x:c r="D51" s="21"/>
       <x:c r="E51" s="21" t="str">
-        <x:f>IF(A51="","",IF(D51="","Available",SWITCH(C51,"Daily",D51+1,"Weekly",D51+7,"Monthly",EDATE(D51,1),"Quarterly",EDATE(D51,3),"Yearly",EDATE(D51,12),"One-time","Used","Manual","Manual",D51)))</x:f>
+        <x:f>IF(A51="","",IF(D51="","Available",SWITCH(C51,"Daily",D51+1,"Weekly",IFERROR(VLOOKUP(A51,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D51-VLOOKUP(A51,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D51+7),"Monthly",IFERROR(EDATE(VLOOKUP(A51,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A51,'VIP Signups'!$A$5:$B$204,2,FALSE),D51,"M")+1),EDATE(D51,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A51,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A51,'VIP Signups'!$A$5:$B$204,2,FALSE),D51,"M")/3)+1)*3),EDATE(D51,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A51,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A51,'VIP Signups'!$A$5:$B$204,2,FALSE),D51,"Y")+1)*12),EDATE(D51,12)),"One-time","Used","Manual","Manual",D51)))</x:f>
       </x:c>
       <x:c r="F51" s="20" t="str">
         <x:f>IF(A51="","",IF(D51="","Yes",IF(E51="Manual","Manual",IF(E51="Used","No",IF(E51&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11575,7 +11587,7 @@
       <x:c r="C52" s="20"/>
       <x:c r="D52" s="21"/>
       <x:c r="E52" s="21" t="str">
-        <x:f>IF(A52="","",IF(D52="","Available",SWITCH(C52,"Daily",D52+1,"Weekly",D52+7,"Monthly",EDATE(D52,1),"Quarterly",EDATE(D52,3),"Yearly",EDATE(D52,12),"One-time","Used","Manual","Manual",D52)))</x:f>
+        <x:f>IF(A52="","",IF(D52="","Available",SWITCH(C52,"Daily",D52+1,"Weekly",IFERROR(VLOOKUP(A52,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D52-VLOOKUP(A52,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D52+7),"Monthly",IFERROR(EDATE(VLOOKUP(A52,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A52,'VIP Signups'!$A$5:$B$204,2,FALSE),D52,"M")+1),EDATE(D52,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A52,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A52,'VIP Signups'!$A$5:$B$204,2,FALSE),D52,"M")/3)+1)*3),EDATE(D52,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A52,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A52,'VIP Signups'!$A$5:$B$204,2,FALSE),D52,"Y")+1)*12),EDATE(D52,12)),"One-time","Used","Manual","Manual",D52)))</x:f>
       </x:c>
       <x:c r="F52" s="20" t="str">
         <x:f>IF(A52="","",IF(D52="","Yes",IF(E52="Manual","Manual",IF(E52="Used","No",IF(E52&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11598,7 +11610,7 @@
       <x:c r="C53" s="20"/>
       <x:c r="D53" s="21"/>
       <x:c r="E53" s="21" t="str">
-        <x:f>IF(A53="","",IF(D53="","Available",SWITCH(C53,"Daily",D53+1,"Weekly",D53+7,"Monthly",EDATE(D53,1),"Quarterly",EDATE(D53,3),"Yearly",EDATE(D53,12),"One-time","Used","Manual","Manual",D53)))</x:f>
+        <x:f>IF(A53="","",IF(D53="","Available",SWITCH(C53,"Daily",D53+1,"Weekly",IFERROR(VLOOKUP(A53,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D53-VLOOKUP(A53,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D53+7),"Monthly",IFERROR(EDATE(VLOOKUP(A53,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A53,'VIP Signups'!$A$5:$B$204,2,FALSE),D53,"M")+1),EDATE(D53,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A53,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A53,'VIP Signups'!$A$5:$B$204,2,FALSE),D53,"M")/3)+1)*3),EDATE(D53,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A53,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A53,'VIP Signups'!$A$5:$B$204,2,FALSE),D53,"Y")+1)*12),EDATE(D53,12)),"One-time","Used","Manual","Manual",D53)))</x:f>
       </x:c>
       <x:c r="F53" s="20" t="str">
         <x:f>IF(A53="","",IF(D53="","Yes",IF(E53="Manual","Manual",IF(E53="Used","No",IF(E53&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11621,7 +11633,7 @@
       <x:c r="C54" s="20"/>
       <x:c r="D54" s="21"/>
       <x:c r="E54" s="21" t="str">
-        <x:f>IF(A54="","",IF(D54="","Available",SWITCH(C54,"Daily",D54+1,"Weekly",D54+7,"Monthly",EDATE(D54,1),"Quarterly",EDATE(D54,3),"Yearly",EDATE(D54,12),"One-time","Used","Manual","Manual",D54)))</x:f>
+        <x:f>IF(A54="","",IF(D54="","Available",SWITCH(C54,"Daily",D54+1,"Weekly",IFERROR(VLOOKUP(A54,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D54-VLOOKUP(A54,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D54+7),"Monthly",IFERROR(EDATE(VLOOKUP(A54,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A54,'VIP Signups'!$A$5:$B$204,2,FALSE),D54,"M")+1),EDATE(D54,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A54,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A54,'VIP Signups'!$A$5:$B$204,2,FALSE),D54,"M")/3)+1)*3),EDATE(D54,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A54,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A54,'VIP Signups'!$A$5:$B$204,2,FALSE),D54,"Y")+1)*12),EDATE(D54,12)),"One-time","Used","Manual","Manual",D54)))</x:f>
       </x:c>
       <x:c r="F54" s="20" t="str">
         <x:f>IF(A54="","",IF(D54="","Yes",IF(E54="Manual","Manual",IF(E54="Used","No",IF(E54&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11644,7 +11656,7 @@
       <x:c r="C55" s="20"/>
       <x:c r="D55" s="21"/>
       <x:c r="E55" s="21" t="str">
-        <x:f>IF(A55="","",IF(D55="","Available",SWITCH(C55,"Daily",D55+1,"Weekly",D55+7,"Monthly",EDATE(D55,1),"Quarterly",EDATE(D55,3),"Yearly",EDATE(D55,12),"One-time","Used","Manual","Manual",D55)))</x:f>
+        <x:f>IF(A55="","",IF(D55="","Available",SWITCH(C55,"Daily",D55+1,"Weekly",IFERROR(VLOOKUP(A55,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D55-VLOOKUP(A55,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D55+7),"Monthly",IFERROR(EDATE(VLOOKUP(A55,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A55,'VIP Signups'!$A$5:$B$204,2,FALSE),D55,"M")+1),EDATE(D55,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A55,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A55,'VIP Signups'!$A$5:$B$204,2,FALSE),D55,"M")/3)+1)*3),EDATE(D55,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A55,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A55,'VIP Signups'!$A$5:$B$204,2,FALSE),D55,"Y")+1)*12),EDATE(D55,12)),"One-time","Used","Manual","Manual",D55)))</x:f>
       </x:c>
       <x:c r="F55" s="20" t="str">
         <x:f>IF(A55="","",IF(D55="","Yes",IF(E55="Manual","Manual",IF(E55="Used","No",IF(E55&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11667,7 +11679,7 @@
       <x:c r="C56" s="20"/>
       <x:c r="D56" s="21"/>
       <x:c r="E56" s="21" t="str">
-        <x:f>IF(A56="","",IF(D56="","Available",SWITCH(C56,"Daily",D56+1,"Weekly",D56+7,"Monthly",EDATE(D56,1),"Quarterly",EDATE(D56,3),"Yearly",EDATE(D56,12),"One-time","Used","Manual","Manual",D56)))</x:f>
+        <x:f>IF(A56="","",IF(D56="","Available",SWITCH(C56,"Daily",D56+1,"Weekly",IFERROR(VLOOKUP(A56,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D56-VLOOKUP(A56,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D56+7),"Monthly",IFERROR(EDATE(VLOOKUP(A56,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A56,'VIP Signups'!$A$5:$B$204,2,FALSE),D56,"M")+1),EDATE(D56,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A56,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A56,'VIP Signups'!$A$5:$B$204,2,FALSE),D56,"M")/3)+1)*3),EDATE(D56,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A56,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A56,'VIP Signups'!$A$5:$B$204,2,FALSE),D56,"Y")+1)*12),EDATE(D56,12)),"One-time","Used","Manual","Manual",D56)))</x:f>
       </x:c>
       <x:c r="F56" s="20" t="str">
         <x:f>IF(A56="","",IF(D56="","Yes",IF(E56="Manual","Manual",IF(E56="Used","No",IF(E56&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11690,7 +11702,7 @@
       <x:c r="C57" s="20"/>
       <x:c r="D57" s="21"/>
       <x:c r="E57" s="21" t="str">
-        <x:f>IF(A57="","",IF(D57="","Available",SWITCH(C57,"Daily",D57+1,"Weekly",D57+7,"Monthly",EDATE(D57,1),"Quarterly",EDATE(D57,3),"Yearly",EDATE(D57,12),"One-time","Used","Manual","Manual",D57)))</x:f>
+        <x:f>IF(A57="","",IF(D57="","Available",SWITCH(C57,"Daily",D57+1,"Weekly",IFERROR(VLOOKUP(A57,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D57-VLOOKUP(A57,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D57+7),"Monthly",IFERROR(EDATE(VLOOKUP(A57,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A57,'VIP Signups'!$A$5:$B$204,2,FALSE),D57,"M")+1),EDATE(D57,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A57,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A57,'VIP Signups'!$A$5:$B$204,2,FALSE),D57,"M")/3)+1)*3),EDATE(D57,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A57,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A57,'VIP Signups'!$A$5:$B$204,2,FALSE),D57,"Y")+1)*12),EDATE(D57,12)),"One-time","Used","Manual","Manual",D57)))</x:f>
       </x:c>
       <x:c r="F57" s="20" t="str">
         <x:f>IF(A57="","",IF(D57="","Yes",IF(E57="Manual","Manual",IF(E57="Used","No",IF(E57&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11713,7 +11725,7 @@
       <x:c r="C58" s="20"/>
       <x:c r="D58" s="21"/>
       <x:c r="E58" s="21" t="str">
-        <x:f>IF(A58="","",IF(D58="","Available",SWITCH(C58,"Daily",D58+1,"Weekly",D58+7,"Monthly",EDATE(D58,1),"Quarterly",EDATE(D58,3),"Yearly",EDATE(D58,12),"One-time","Used","Manual","Manual",D58)))</x:f>
+        <x:f>IF(A58="","",IF(D58="","Available",SWITCH(C58,"Daily",D58+1,"Weekly",IFERROR(VLOOKUP(A58,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D58-VLOOKUP(A58,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D58+7),"Monthly",IFERROR(EDATE(VLOOKUP(A58,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A58,'VIP Signups'!$A$5:$B$204,2,FALSE),D58,"M")+1),EDATE(D58,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A58,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A58,'VIP Signups'!$A$5:$B$204,2,FALSE),D58,"M")/3)+1)*3),EDATE(D58,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A58,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A58,'VIP Signups'!$A$5:$B$204,2,FALSE),D58,"Y")+1)*12),EDATE(D58,12)),"One-time","Used","Manual","Manual",D58)))</x:f>
       </x:c>
       <x:c r="F58" s="20" t="str">
         <x:f>IF(A58="","",IF(D58="","Yes",IF(E58="Manual","Manual",IF(E58="Used","No",IF(E58&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11736,7 +11748,7 @@
       <x:c r="C59" s="20"/>
       <x:c r="D59" s="21"/>
       <x:c r="E59" s="21" t="str">
-        <x:f>IF(A59="","",IF(D59="","Available",SWITCH(C59,"Daily",D59+1,"Weekly",D59+7,"Monthly",EDATE(D59,1),"Quarterly",EDATE(D59,3),"Yearly",EDATE(D59,12),"One-time","Used","Manual","Manual",D59)))</x:f>
+        <x:f>IF(A59="","",IF(D59="","Available",SWITCH(C59,"Daily",D59+1,"Weekly",IFERROR(VLOOKUP(A59,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D59-VLOOKUP(A59,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D59+7),"Monthly",IFERROR(EDATE(VLOOKUP(A59,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A59,'VIP Signups'!$A$5:$B$204,2,FALSE),D59,"M")+1),EDATE(D59,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A59,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A59,'VIP Signups'!$A$5:$B$204,2,FALSE),D59,"M")/3)+1)*3),EDATE(D59,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A59,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A59,'VIP Signups'!$A$5:$B$204,2,FALSE),D59,"Y")+1)*12),EDATE(D59,12)),"One-time","Used","Manual","Manual",D59)))</x:f>
       </x:c>
       <x:c r="F59" s="20" t="str">
         <x:f>IF(A59="","",IF(D59="","Yes",IF(E59="Manual","Manual",IF(E59="Used","No",IF(E59&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11759,7 +11771,7 @@
       <x:c r="C60" s="20"/>
       <x:c r="D60" s="21"/>
       <x:c r="E60" s="21" t="str">
-        <x:f>IF(A60="","",IF(D60="","Available",SWITCH(C60,"Daily",D60+1,"Weekly",D60+7,"Monthly",EDATE(D60,1),"Quarterly",EDATE(D60,3),"Yearly",EDATE(D60,12),"One-time","Used","Manual","Manual",D60)))</x:f>
+        <x:f>IF(A60="","",IF(D60="","Available",SWITCH(C60,"Daily",D60+1,"Weekly",IFERROR(VLOOKUP(A60,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D60-VLOOKUP(A60,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D60+7),"Monthly",IFERROR(EDATE(VLOOKUP(A60,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A60,'VIP Signups'!$A$5:$B$204,2,FALSE),D60,"M")+1),EDATE(D60,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A60,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A60,'VIP Signups'!$A$5:$B$204,2,FALSE),D60,"M")/3)+1)*3),EDATE(D60,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A60,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A60,'VIP Signups'!$A$5:$B$204,2,FALSE),D60,"Y")+1)*12),EDATE(D60,12)),"One-time","Used","Manual","Manual",D60)))</x:f>
       </x:c>
       <x:c r="F60" s="20" t="str">
         <x:f>IF(A60="","",IF(D60="","Yes",IF(E60="Manual","Manual",IF(E60="Used","No",IF(E60&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11782,7 +11794,7 @@
       <x:c r="C61" s="20"/>
       <x:c r="D61" s="21"/>
       <x:c r="E61" s="21" t="str">
-        <x:f>IF(A61="","",IF(D61="","Available",SWITCH(C61,"Daily",D61+1,"Weekly",D61+7,"Monthly",EDATE(D61,1),"Quarterly",EDATE(D61,3),"Yearly",EDATE(D61,12),"One-time","Used","Manual","Manual",D61)))</x:f>
+        <x:f>IF(A61="","",IF(D61="","Available",SWITCH(C61,"Daily",D61+1,"Weekly",IFERROR(VLOOKUP(A61,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D61-VLOOKUP(A61,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D61+7),"Monthly",IFERROR(EDATE(VLOOKUP(A61,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A61,'VIP Signups'!$A$5:$B$204,2,FALSE),D61,"M")+1),EDATE(D61,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A61,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A61,'VIP Signups'!$A$5:$B$204,2,FALSE),D61,"M")/3)+1)*3),EDATE(D61,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A61,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A61,'VIP Signups'!$A$5:$B$204,2,FALSE),D61,"Y")+1)*12),EDATE(D61,12)),"One-time","Used","Manual","Manual",D61)))</x:f>
       </x:c>
       <x:c r="F61" s="20" t="str">
         <x:f>IF(A61="","",IF(D61="","Yes",IF(E61="Manual","Manual",IF(E61="Used","No",IF(E61&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11805,7 +11817,7 @@
       <x:c r="C62" s="20"/>
       <x:c r="D62" s="21"/>
       <x:c r="E62" s="21" t="str">
-        <x:f>IF(A62="","",IF(D62="","Available",SWITCH(C62,"Daily",D62+1,"Weekly",D62+7,"Monthly",EDATE(D62,1),"Quarterly",EDATE(D62,3),"Yearly",EDATE(D62,12),"One-time","Used","Manual","Manual",D62)))</x:f>
+        <x:f>IF(A62="","",IF(D62="","Available",SWITCH(C62,"Daily",D62+1,"Weekly",IFERROR(VLOOKUP(A62,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D62-VLOOKUP(A62,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D62+7),"Monthly",IFERROR(EDATE(VLOOKUP(A62,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A62,'VIP Signups'!$A$5:$B$204,2,FALSE),D62,"M")+1),EDATE(D62,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A62,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A62,'VIP Signups'!$A$5:$B$204,2,FALSE),D62,"M")/3)+1)*3),EDATE(D62,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A62,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A62,'VIP Signups'!$A$5:$B$204,2,FALSE),D62,"Y")+1)*12),EDATE(D62,12)),"One-time","Used","Manual","Manual",D62)))</x:f>
       </x:c>
       <x:c r="F62" s="20" t="str">
         <x:f>IF(A62="","",IF(D62="","Yes",IF(E62="Manual","Manual",IF(E62="Used","No",IF(E62&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11828,7 +11840,7 @@
       <x:c r="C63" s="20"/>
       <x:c r="D63" s="21"/>
       <x:c r="E63" s="21" t="str">
-        <x:f>IF(A63="","",IF(D63="","Available",SWITCH(C63,"Daily",D63+1,"Weekly",D63+7,"Monthly",EDATE(D63,1),"Quarterly",EDATE(D63,3),"Yearly",EDATE(D63,12),"One-time","Used","Manual","Manual",D63)))</x:f>
+        <x:f>IF(A63="","",IF(D63="","Available",SWITCH(C63,"Daily",D63+1,"Weekly",IFERROR(VLOOKUP(A63,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D63-VLOOKUP(A63,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D63+7),"Monthly",IFERROR(EDATE(VLOOKUP(A63,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A63,'VIP Signups'!$A$5:$B$204,2,FALSE),D63,"M")+1),EDATE(D63,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A63,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A63,'VIP Signups'!$A$5:$B$204,2,FALSE),D63,"M")/3)+1)*3),EDATE(D63,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A63,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A63,'VIP Signups'!$A$5:$B$204,2,FALSE),D63,"Y")+1)*12),EDATE(D63,12)),"One-time","Used","Manual","Manual",D63)))</x:f>
       </x:c>
       <x:c r="F63" s="20" t="str">
         <x:f>IF(A63="","",IF(D63="","Yes",IF(E63="Manual","Manual",IF(E63="Used","No",IF(E63&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11851,7 +11863,7 @@
       <x:c r="C64" s="20"/>
       <x:c r="D64" s="21"/>
       <x:c r="E64" s="21" t="str">
-        <x:f>IF(A64="","",IF(D64="","Available",SWITCH(C64,"Daily",D64+1,"Weekly",D64+7,"Monthly",EDATE(D64,1),"Quarterly",EDATE(D64,3),"Yearly",EDATE(D64,12),"One-time","Used","Manual","Manual",D64)))</x:f>
+        <x:f>IF(A64="","",IF(D64="","Available",SWITCH(C64,"Daily",D64+1,"Weekly",IFERROR(VLOOKUP(A64,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D64-VLOOKUP(A64,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D64+7),"Monthly",IFERROR(EDATE(VLOOKUP(A64,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A64,'VIP Signups'!$A$5:$B$204,2,FALSE),D64,"M")+1),EDATE(D64,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A64,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A64,'VIP Signups'!$A$5:$B$204,2,FALSE),D64,"M")/3)+1)*3),EDATE(D64,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A64,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A64,'VIP Signups'!$A$5:$B$204,2,FALSE),D64,"Y")+1)*12),EDATE(D64,12)),"One-time","Used","Manual","Manual",D64)))</x:f>
       </x:c>
       <x:c r="F64" s="20" t="str">
         <x:f>IF(A64="","",IF(D64="","Yes",IF(E64="Manual","Manual",IF(E64="Used","No",IF(E64&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11874,7 +11886,7 @@
       <x:c r="C65" s="20"/>
       <x:c r="D65" s="21"/>
       <x:c r="E65" s="21" t="str">
-        <x:f>IF(A65="","",IF(D65="","Available",SWITCH(C65,"Daily",D65+1,"Weekly",D65+7,"Monthly",EDATE(D65,1),"Quarterly",EDATE(D65,3),"Yearly",EDATE(D65,12),"One-time","Used","Manual","Manual",D65)))</x:f>
+        <x:f>IF(A65="","",IF(D65="","Available",SWITCH(C65,"Daily",D65+1,"Weekly",IFERROR(VLOOKUP(A65,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D65-VLOOKUP(A65,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D65+7),"Monthly",IFERROR(EDATE(VLOOKUP(A65,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A65,'VIP Signups'!$A$5:$B$204,2,FALSE),D65,"M")+1),EDATE(D65,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A65,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A65,'VIP Signups'!$A$5:$B$204,2,FALSE),D65,"M")/3)+1)*3),EDATE(D65,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A65,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A65,'VIP Signups'!$A$5:$B$204,2,FALSE),D65,"Y")+1)*12),EDATE(D65,12)),"One-time","Used","Manual","Manual",D65)))</x:f>
       </x:c>
       <x:c r="F65" s="20" t="str">
         <x:f>IF(A65="","",IF(D65="","Yes",IF(E65="Manual","Manual",IF(E65="Used","No",IF(E65&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11897,7 +11909,7 @@
       <x:c r="C66" s="20"/>
       <x:c r="D66" s="21"/>
       <x:c r="E66" s="21" t="str">
-        <x:f>IF(A66="","",IF(D66="","Available",SWITCH(C66,"Daily",D66+1,"Weekly",D66+7,"Monthly",EDATE(D66,1),"Quarterly",EDATE(D66,3),"Yearly",EDATE(D66,12),"One-time","Used","Manual","Manual",D66)))</x:f>
+        <x:f>IF(A66="","",IF(D66="","Available",SWITCH(C66,"Daily",D66+1,"Weekly",IFERROR(VLOOKUP(A66,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D66-VLOOKUP(A66,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D66+7),"Monthly",IFERROR(EDATE(VLOOKUP(A66,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A66,'VIP Signups'!$A$5:$B$204,2,FALSE),D66,"M")+1),EDATE(D66,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A66,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A66,'VIP Signups'!$A$5:$B$204,2,FALSE),D66,"M")/3)+1)*3),EDATE(D66,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A66,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A66,'VIP Signups'!$A$5:$B$204,2,FALSE),D66,"Y")+1)*12),EDATE(D66,12)),"One-time","Used","Manual","Manual",D66)))</x:f>
       </x:c>
       <x:c r="F66" s="20" t="str">
         <x:f>IF(A66="","",IF(D66="","Yes",IF(E66="Manual","Manual",IF(E66="Used","No",IF(E66&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11920,7 +11932,7 @@
       <x:c r="C67" s="20"/>
       <x:c r="D67" s="21"/>
       <x:c r="E67" s="21" t="str">
-        <x:f>IF(A67="","",IF(D67="","Available",SWITCH(C67,"Daily",D67+1,"Weekly",D67+7,"Monthly",EDATE(D67,1),"Quarterly",EDATE(D67,3),"Yearly",EDATE(D67,12),"One-time","Used","Manual","Manual",D67)))</x:f>
+        <x:f>IF(A67="","",IF(D67="","Available",SWITCH(C67,"Daily",D67+1,"Weekly",IFERROR(VLOOKUP(A67,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D67-VLOOKUP(A67,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D67+7),"Monthly",IFERROR(EDATE(VLOOKUP(A67,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A67,'VIP Signups'!$A$5:$B$204,2,FALSE),D67,"M")+1),EDATE(D67,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A67,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A67,'VIP Signups'!$A$5:$B$204,2,FALSE),D67,"M")/3)+1)*3),EDATE(D67,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A67,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A67,'VIP Signups'!$A$5:$B$204,2,FALSE),D67,"Y")+1)*12),EDATE(D67,12)),"One-time","Used","Manual","Manual",D67)))</x:f>
       </x:c>
       <x:c r="F67" s="20" t="str">
         <x:f>IF(A67="","",IF(D67="","Yes",IF(E67="Manual","Manual",IF(E67="Used","No",IF(E67&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11943,7 +11955,7 @@
       <x:c r="C68" s="20"/>
       <x:c r="D68" s="21"/>
       <x:c r="E68" s="21" t="str">
-        <x:f>IF(A68="","",IF(D68="","Available",SWITCH(C68,"Daily",D68+1,"Weekly",D68+7,"Monthly",EDATE(D68,1),"Quarterly",EDATE(D68,3),"Yearly",EDATE(D68,12),"One-time","Used","Manual","Manual",D68)))</x:f>
+        <x:f>IF(A68="","",IF(D68="","Available",SWITCH(C68,"Daily",D68+1,"Weekly",IFERROR(VLOOKUP(A68,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D68-VLOOKUP(A68,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D68+7),"Monthly",IFERROR(EDATE(VLOOKUP(A68,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A68,'VIP Signups'!$A$5:$B$204,2,FALSE),D68,"M")+1),EDATE(D68,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A68,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A68,'VIP Signups'!$A$5:$B$204,2,FALSE),D68,"M")/3)+1)*3),EDATE(D68,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A68,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A68,'VIP Signups'!$A$5:$B$204,2,FALSE),D68,"Y")+1)*12),EDATE(D68,12)),"One-time","Used","Manual","Manual",D68)))</x:f>
       </x:c>
       <x:c r="F68" s="20" t="str">
         <x:f>IF(A68="","",IF(D68="","Yes",IF(E68="Manual","Manual",IF(E68="Used","No",IF(E68&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11966,7 +11978,7 @@
       <x:c r="C69" s="20"/>
       <x:c r="D69" s="21"/>
       <x:c r="E69" s="21" t="str">
-        <x:f>IF(A69="","",IF(D69="","Available",SWITCH(C69,"Daily",D69+1,"Weekly",D69+7,"Monthly",EDATE(D69,1),"Quarterly",EDATE(D69,3),"Yearly",EDATE(D69,12),"One-time","Used","Manual","Manual",D69)))</x:f>
+        <x:f>IF(A69="","",IF(D69="","Available",SWITCH(C69,"Daily",D69+1,"Weekly",IFERROR(VLOOKUP(A69,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D69-VLOOKUP(A69,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D69+7),"Monthly",IFERROR(EDATE(VLOOKUP(A69,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A69,'VIP Signups'!$A$5:$B$204,2,FALSE),D69,"M")+1),EDATE(D69,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A69,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A69,'VIP Signups'!$A$5:$B$204,2,FALSE),D69,"M")/3)+1)*3),EDATE(D69,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A69,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A69,'VIP Signups'!$A$5:$B$204,2,FALSE),D69,"Y")+1)*12),EDATE(D69,12)),"One-time","Used","Manual","Manual",D69)))</x:f>
       </x:c>
       <x:c r="F69" s="20" t="str">
         <x:f>IF(A69="","",IF(D69="","Yes",IF(E69="Manual","Manual",IF(E69="Used","No",IF(E69&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -11989,7 +12001,7 @@
       <x:c r="C70" s="20"/>
       <x:c r="D70" s="21"/>
       <x:c r="E70" s="21" t="str">
-        <x:f>IF(A70="","",IF(D70="","Available",SWITCH(C70,"Daily",D70+1,"Weekly",D70+7,"Monthly",EDATE(D70,1),"Quarterly",EDATE(D70,3),"Yearly",EDATE(D70,12),"One-time","Used","Manual","Manual",D70)))</x:f>
+        <x:f>IF(A70="","",IF(D70="","Available",SWITCH(C70,"Daily",D70+1,"Weekly",IFERROR(VLOOKUP(A70,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D70-VLOOKUP(A70,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D70+7),"Monthly",IFERROR(EDATE(VLOOKUP(A70,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A70,'VIP Signups'!$A$5:$B$204,2,FALSE),D70,"M")+1),EDATE(D70,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A70,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A70,'VIP Signups'!$A$5:$B$204,2,FALSE),D70,"M")/3)+1)*3),EDATE(D70,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A70,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A70,'VIP Signups'!$A$5:$B$204,2,FALSE),D70,"Y")+1)*12),EDATE(D70,12)),"One-time","Used","Manual","Manual",D70)))</x:f>
       </x:c>
       <x:c r="F70" s="20" t="str">
         <x:f>IF(A70="","",IF(D70="","Yes",IF(E70="Manual","Manual",IF(E70="Used","No",IF(E70&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12012,7 +12024,7 @@
       <x:c r="C71" s="20"/>
       <x:c r="D71" s="21"/>
       <x:c r="E71" s="21" t="str">
-        <x:f>IF(A71="","",IF(D71="","Available",SWITCH(C71,"Daily",D71+1,"Weekly",D71+7,"Monthly",EDATE(D71,1),"Quarterly",EDATE(D71,3),"Yearly",EDATE(D71,12),"One-time","Used","Manual","Manual",D71)))</x:f>
+        <x:f>IF(A71="","",IF(D71="","Available",SWITCH(C71,"Daily",D71+1,"Weekly",IFERROR(VLOOKUP(A71,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D71-VLOOKUP(A71,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D71+7),"Monthly",IFERROR(EDATE(VLOOKUP(A71,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A71,'VIP Signups'!$A$5:$B$204,2,FALSE),D71,"M")+1),EDATE(D71,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A71,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A71,'VIP Signups'!$A$5:$B$204,2,FALSE),D71,"M")/3)+1)*3),EDATE(D71,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A71,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A71,'VIP Signups'!$A$5:$B$204,2,FALSE),D71,"Y")+1)*12),EDATE(D71,12)),"One-time","Used","Manual","Manual",D71)))</x:f>
       </x:c>
       <x:c r="F71" s="20" t="str">
         <x:f>IF(A71="","",IF(D71="","Yes",IF(E71="Manual","Manual",IF(E71="Used","No",IF(E71&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12035,7 +12047,7 @@
       <x:c r="C72" s="20"/>
       <x:c r="D72" s="21"/>
       <x:c r="E72" s="21" t="str">
-        <x:f>IF(A72="","",IF(D72="","Available",SWITCH(C72,"Daily",D72+1,"Weekly",D72+7,"Monthly",EDATE(D72,1),"Quarterly",EDATE(D72,3),"Yearly",EDATE(D72,12),"One-time","Used","Manual","Manual",D72)))</x:f>
+        <x:f>IF(A72="","",IF(D72="","Available",SWITCH(C72,"Daily",D72+1,"Weekly",IFERROR(VLOOKUP(A72,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D72-VLOOKUP(A72,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D72+7),"Monthly",IFERROR(EDATE(VLOOKUP(A72,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A72,'VIP Signups'!$A$5:$B$204,2,FALSE),D72,"M")+1),EDATE(D72,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A72,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A72,'VIP Signups'!$A$5:$B$204,2,FALSE),D72,"M")/3)+1)*3),EDATE(D72,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A72,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A72,'VIP Signups'!$A$5:$B$204,2,FALSE),D72,"Y")+1)*12),EDATE(D72,12)),"One-time","Used","Manual","Manual",D72)))</x:f>
       </x:c>
       <x:c r="F72" s="20" t="str">
         <x:f>IF(A72="","",IF(D72="","Yes",IF(E72="Manual","Manual",IF(E72="Used","No",IF(E72&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12058,7 +12070,7 @@
       <x:c r="C73" s="20"/>
       <x:c r="D73" s="21"/>
       <x:c r="E73" s="21" t="str">
-        <x:f>IF(A73="","",IF(D73="","Available",SWITCH(C73,"Daily",D73+1,"Weekly",D73+7,"Monthly",EDATE(D73,1),"Quarterly",EDATE(D73,3),"Yearly",EDATE(D73,12),"One-time","Used","Manual","Manual",D73)))</x:f>
+        <x:f>IF(A73="","",IF(D73="","Available",SWITCH(C73,"Daily",D73+1,"Weekly",IFERROR(VLOOKUP(A73,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D73-VLOOKUP(A73,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D73+7),"Monthly",IFERROR(EDATE(VLOOKUP(A73,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A73,'VIP Signups'!$A$5:$B$204,2,FALSE),D73,"M")+1),EDATE(D73,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A73,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A73,'VIP Signups'!$A$5:$B$204,2,FALSE),D73,"M")/3)+1)*3),EDATE(D73,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A73,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A73,'VIP Signups'!$A$5:$B$204,2,FALSE),D73,"Y")+1)*12),EDATE(D73,12)),"One-time","Used","Manual","Manual",D73)))</x:f>
       </x:c>
       <x:c r="F73" s="20" t="str">
         <x:f>IF(A73="","",IF(D73="","Yes",IF(E73="Manual","Manual",IF(E73="Used","No",IF(E73&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12081,7 +12093,7 @@
       <x:c r="C74" s="20"/>
       <x:c r="D74" s="21"/>
       <x:c r="E74" s="21" t="str">
-        <x:f>IF(A74="","",IF(D74="","Available",SWITCH(C74,"Daily",D74+1,"Weekly",D74+7,"Monthly",EDATE(D74,1),"Quarterly",EDATE(D74,3),"Yearly",EDATE(D74,12),"One-time","Used","Manual","Manual",D74)))</x:f>
+        <x:f>IF(A74="","",IF(D74="","Available",SWITCH(C74,"Daily",D74+1,"Weekly",IFERROR(VLOOKUP(A74,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D74-VLOOKUP(A74,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D74+7),"Monthly",IFERROR(EDATE(VLOOKUP(A74,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A74,'VIP Signups'!$A$5:$B$204,2,FALSE),D74,"M")+1),EDATE(D74,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A74,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A74,'VIP Signups'!$A$5:$B$204,2,FALSE),D74,"M")/3)+1)*3),EDATE(D74,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A74,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A74,'VIP Signups'!$A$5:$B$204,2,FALSE),D74,"Y")+1)*12),EDATE(D74,12)),"One-time","Used","Manual","Manual",D74)))</x:f>
       </x:c>
       <x:c r="F74" s="20" t="str">
         <x:f>IF(A74="","",IF(D74="","Yes",IF(E74="Manual","Manual",IF(E74="Used","No",IF(E74&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12104,7 +12116,7 @@
       <x:c r="C75" s="20"/>
       <x:c r="D75" s="21"/>
       <x:c r="E75" s="21" t="str">
-        <x:f>IF(A75="","",IF(D75="","Available",SWITCH(C75,"Daily",D75+1,"Weekly",D75+7,"Monthly",EDATE(D75,1),"Quarterly",EDATE(D75,3),"Yearly",EDATE(D75,12),"One-time","Used","Manual","Manual",D75)))</x:f>
+        <x:f>IF(A75="","",IF(D75="","Available",SWITCH(C75,"Daily",D75+1,"Weekly",IFERROR(VLOOKUP(A75,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D75-VLOOKUP(A75,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D75+7),"Monthly",IFERROR(EDATE(VLOOKUP(A75,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A75,'VIP Signups'!$A$5:$B$204,2,FALSE),D75,"M")+1),EDATE(D75,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A75,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A75,'VIP Signups'!$A$5:$B$204,2,FALSE),D75,"M")/3)+1)*3),EDATE(D75,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A75,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A75,'VIP Signups'!$A$5:$B$204,2,FALSE),D75,"Y")+1)*12),EDATE(D75,12)),"One-time","Used","Manual","Manual",D75)))</x:f>
       </x:c>
       <x:c r="F75" s="20" t="str">
         <x:f>IF(A75="","",IF(D75="","Yes",IF(E75="Manual","Manual",IF(E75="Used","No",IF(E75&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12127,7 +12139,7 @@
       <x:c r="C76" s="20"/>
       <x:c r="D76" s="21"/>
       <x:c r="E76" s="21" t="str">
-        <x:f>IF(A76="","",IF(D76="","Available",SWITCH(C76,"Daily",D76+1,"Weekly",D76+7,"Monthly",EDATE(D76,1),"Quarterly",EDATE(D76,3),"Yearly",EDATE(D76,12),"One-time","Used","Manual","Manual",D76)))</x:f>
+        <x:f>IF(A76="","",IF(D76="","Available",SWITCH(C76,"Daily",D76+1,"Weekly",IFERROR(VLOOKUP(A76,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D76-VLOOKUP(A76,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D76+7),"Monthly",IFERROR(EDATE(VLOOKUP(A76,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A76,'VIP Signups'!$A$5:$B$204,2,FALSE),D76,"M")+1),EDATE(D76,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A76,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A76,'VIP Signups'!$A$5:$B$204,2,FALSE),D76,"M")/3)+1)*3),EDATE(D76,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A76,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A76,'VIP Signups'!$A$5:$B$204,2,FALSE),D76,"Y")+1)*12),EDATE(D76,12)),"One-time","Used","Manual","Manual",D76)))</x:f>
       </x:c>
       <x:c r="F76" s="20" t="str">
         <x:f>IF(A76="","",IF(D76="","Yes",IF(E76="Manual","Manual",IF(E76="Used","No",IF(E76&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12150,7 +12162,7 @@
       <x:c r="C77" s="20"/>
       <x:c r="D77" s="21"/>
       <x:c r="E77" s="21" t="str">
-        <x:f>IF(A77="","",IF(D77="","Available",SWITCH(C77,"Daily",D77+1,"Weekly",D77+7,"Monthly",EDATE(D77,1),"Quarterly",EDATE(D77,3),"Yearly",EDATE(D77,12),"One-time","Used","Manual","Manual",D77)))</x:f>
+        <x:f>IF(A77="","",IF(D77="","Available",SWITCH(C77,"Daily",D77+1,"Weekly",IFERROR(VLOOKUP(A77,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D77-VLOOKUP(A77,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D77+7),"Monthly",IFERROR(EDATE(VLOOKUP(A77,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A77,'VIP Signups'!$A$5:$B$204,2,FALSE),D77,"M")+1),EDATE(D77,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A77,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A77,'VIP Signups'!$A$5:$B$204,2,FALSE),D77,"M")/3)+1)*3),EDATE(D77,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A77,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A77,'VIP Signups'!$A$5:$B$204,2,FALSE),D77,"Y")+1)*12),EDATE(D77,12)),"One-time","Used","Manual","Manual",D77)))</x:f>
       </x:c>
       <x:c r="F77" s="20" t="str">
         <x:f>IF(A77="","",IF(D77="","Yes",IF(E77="Manual","Manual",IF(E77="Used","No",IF(E77&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12173,7 +12185,7 @@
       <x:c r="C78" s="20"/>
       <x:c r="D78" s="21"/>
       <x:c r="E78" s="21" t="str">
-        <x:f>IF(A78="","",IF(D78="","Available",SWITCH(C78,"Daily",D78+1,"Weekly",D78+7,"Monthly",EDATE(D78,1),"Quarterly",EDATE(D78,3),"Yearly",EDATE(D78,12),"One-time","Used","Manual","Manual",D78)))</x:f>
+        <x:f>IF(A78="","",IF(D78="","Available",SWITCH(C78,"Daily",D78+1,"Weekly",IFERROR(VLOOKUP(A78,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D78-VLOOKUP(A78,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D78+7),"Monthly",IFERROR(EDATE(VLOOKUP(A78,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A78,'VIP Signups'!$A$5:$B$204,2,FALSE),D78,"M")+1),EDATE(D78,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A78,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A78,'VIP Signups'!$A$5:$B$204,2,FALSE),D78,"M")/3)+1)*3),EDATE(D78,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A78,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A78,'VIP Signups'!$A$5:$B$204,2,FALSE),D78,"Y")+1)*12),EDATE(D78,12)),"One-time","Used","Manual","Manual",D78)))</x:f>
       </x:c>
       <x:c r="F78" s="20" t="str">
         <x:f>IF(A78="","",IF(D78="","Yes",IF(E78="Manual","Manual",IF(E78="Used","No",IF(E78&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12196,7 +12208,7 @@
       <x:c r="C79" s="20"/>
       <x:c r="D79" s="21"/>
       <x:c r="E79" s="21" t="str">
-        <x:f>IF(A79="","",IF(D79="","Available",SWITCH(C79,"Daily",D79+1,"Weekly",D79+7,"Monthly",EDATE(D79,1),"Quarterly",EDATE(D79,3),"Yearly",EDATE(D79,12),"One-time","Used","Manual","Manual",D79)))</x:f>
+        <x:f>IF(A79="","",IF(D79="","Available",SWITCH(C79,"Daily",D79+1,"Weekly",IFERROR(VLOOKUP(A79,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D79-VLOOKUP(A79,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D79+7),"Monthly",IFERROR(EDATE(VLOOKUP(A79,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A79,'VIP Signups'!$A$5:$B$204,2,FALSE),D79,"M")+1),EDATE(D79,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A79,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A79,'VIP Signups'!$A$5:$B$204,2,FALSE),D79,"M")/3)+1)*3),EDATE(D79,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A79,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A79,'VIP Signups'!$A$5:$B$204,2,FALSE),D79,"Y")+1)*12),EDATE(D79,12)),"One-time","Used","Manual","Manual",D79)))</x:f>
       </x:c>
       <x:c r="F79" s="20" t="str">
         <x:f>IF(A79="","",IF(D79="","Yes",IF(E79="Manual","Manual",IF(E79="Used","No",IF(E79&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12219,7 +12231,7 @@
       <x:c r="C80" s="20"/>
       <x:c r="D80" s="21"/>
       <x:c r="E80" s="21" t="str">
-        <x:f>IF(A80="","",IF(D80="","Available",SWITCH(C80,"Daily",D80+1,"Weekly",D80+7,"Monthly",EDATE(D80,1),"Quarterly",EDATE(D80,3),"Yearly",EDATE(D80,12),"One-time","Used","Manual","Manual",D80)))</x:f>
+        <x:f>IF(A80="","",IF(D80="","Available",SWITCH(C80,"Daily",D80+1,"Weekly",IFERROR(VLOOKUP(A80,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D80-VLOOKUP(A80,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D80+7),"Monthly",IFERROR(EDATE(VLOOKUP(A80,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A80,'VIP Signups'!$A$5:$B$204,2,FALSE),D80,"M")+1),EDATE(D80,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A80,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A80,'VIP Signups'!$A$5:$B$204,2,FALSE),D80,"M")/3)+1)*3),EDATE(D80,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A80,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A80,'VIP Signups'!$A$5:$B$204,2,FALSE),D80,"Y")+1)*12),EDATE(D80,12)),"One-time","Used","Manual","Manual",D80)))</x:f>
       </x:c>
       <x:c r="F80" s="20" t="str">
         <x:f>IF(A80="","",IF(D80="","Yes",IF(E80="Manual","Manual",IF(E80="Used","No",IF(E80&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12242,7 +12254,7 @@
       <x:c r="C81" s="20"/>
       <x:c r="D81" s="21"/>
       <x:c r="E81" s="21" t="str">
-        <x:f>IF(A81="","",IF(D81="","Available",SWITCH(C81,"Daily",D81+1,"Weekly",D81+7,"Monthly",EDATE(D81,1),"Quarterly",EDATE(D81,3),"Yearly",EDATE(D81,12),"One-time","Used","Manual","Manual",D81)))</x:f>
+        <x:f>IF(A81="","",IF(D81="","Available",SWITCH(C81,"Daily",D81+1,"Weekly",IFERROR(VLOOKUP(A81,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D81-VLOOKUP(A81,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D81+7),"Monthly",IFERROR(EDATE(VLOOKUP(A81,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A81,'VIP Signups'!$A$5:$B$204,2,FALSE),D81,"M")+1),EDATE(D81,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A81,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A81,'VIP Signups'!$A$5:$B$204,2,FALSE),D81,"M")/3)+1)*3),EDATE(D81,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A81,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A81,'VIP Signups'!$A$5:$B$204,2,FALSE),D81,"Y")+1)*12),EDATE(D81,12)),"One-time","Used","Manual","Manual",D81)))</x:f>
       </x:c>
       <x:c r="F81" s="20" t="str">
         <x:f>IF(A81="","",IF(D81="","Yes",IF(E81="Manual","Manual",IF(E81="Used","No",IF(E81&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12265,7 +12277,7 @@
       <x:c r="C82" s="20"/>
       <x:c r="D82" s="21"/>
       <x:c r="E82" s="21" t="str">
-        <x:f>IF(A82="","",IF(D82="","Available",SWITCH(C82,"Daily",D82+1,"Weekly",D82+7,"Monthly",EDATE(D82,1),"Quarterly",EDATE(D82,3),"Yearly",EDATE(D82,12),"One-time","Used","Manual","Manual",D82)))</x:f>
+        <x:f>IF(A82="","",IF(D82="","Available",SWITCH(C82,"Daily",D82+1,"Weekly",IFERROR(VLOOKUP(A82,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D82-VLOOKUP(A82,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D82+7),"Monthly",IFERROR(EDATE(VLOOKUP(A82,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A82,'VIP Signups'!$A$5:$B$204,2,FALSE),D82,"M")+1),EDATE(D82,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A82,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A82,'VIP Signups'!$A$5:$B$204,2,FALSE),D82,"M")/3)+1)*3),EDATE(D82,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A82,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A82,'VIP Signups'!$A$5:$B$204,2,FALSE),D82,"Y")+1)*12),EDATE(D82,12)),"One-time","Used","Manual","Manual",D82)))</x:f>
       </x:c>
       <x:c r="F82" s="20" t="str">
         <x:f>IF(A82="","",IF(D82="","Yes",IF(E82="Manual","Manual",IF(E82="Used","No",IF(E82&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12288,7 +12300,7 @@
       <x:c r="C83" s="20"/>
       <x:c r="D83" s="21"/>
       <x:c r="E83" s="21" t="str">
-        <x:f>IF(A83="","",IF(D83="","Available",SWITCH(C83,"Daily",D83+1,"Weekly",D83+7,"Monthly",EDATE(D83,1),"Quarterly",EDATE(D83,3),"Yearly",EDATE(D83,12),"One-time","Used","Manual","Manual",D83)))</x:f>
+        <x:f>IF(A83="","",IF(D83="","Available",SWITCH(C83,"Daily",D83+1,"Weekly",IFERROR(VLOOKUP(A83,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D83-VLOOKUP(A83,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D83+7),"Monthly",IFERROR(EDATE(VLOOKUP(A83,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A83,'VIP Signups'!$A$5:$B$204,2,FALSE),D83,"M")+1),EDATE(D83,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A83,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A83,'VIP Signups'!$A$5:$B$204,2,FALSE),D83,"M")/3)+1)*3),EDATE(D83,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A83,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A83,'VIP Signups'!$A$5:$B$204,2,FALSE),D83,"Y")+1)*12),EDATE(D83,12)),"One-time","Used","Manual","Manual",D83)))</x:f>
       </x:c>
       <x:c r="F83" s="20" t="str">
         <x:f>IF(A83="","",IF(D83="","Yes",IF(E83="Manual","Manual",IF(E83="Used","No",IF(E83&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12311,7 +12323,7 @@
       <x:c r="C84" s="20"/>
       <x:c r="D84" s="21"/>
       <x:c r="E84" s="21" t="str">
-        <x:f>IF(A84="","",IF(D84="","Available",SWITCH(C84,"Daily",D84+1,"Weekly",D84+7,"Monthly",EDATE(D84,1),"Quarterly",EDATE(D84,3),"Yearly",EDATE(D84,12),"One-time","Used","Manual","Manual",D84)))</x:f>
+        <x:f>IF(A84="","",IF(D84="","Available",SWITCH(C84,"Daily",D84+1,"Weekly",IFERROR(VLOOKUP(A84,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D84-VLOOKUP(A84,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D84+7),"Monthly",IFERROR(EDATE(VLOOKUP(A84,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A84,'VIP Signups'!$A$5:$B$204,2,FALSE),D84,"M")+1),EDATE(D84,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A84,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A84,'VIP Signups'!$A$5:$B$204,2,FALSE),D84,"M")/3)+1)*3),EDATE(D84,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A84,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A84,'VIP Signups'!$A$5:$B$204,2,FALSE),D84,"Y")+1)*12),EDATE(D84,12)),"One-time","Used","Manual","Manual",D84)))</x:f>
       </x:c>
       <x:c r="F84" s="20" t="str">
         <x:f>IF(A84="","",IF(D84="","Yes",IF(E84="Manual","Manual",IF(E84="Used","No",IF(E84&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12334,7 +12346,7 @@
       <x:c r="C85" s="20"/>
       <x:c r="D85" s="21"/>
       <x:c r="E85" s="21" t="str">
-        <x:f>IF(A85="","",IF(D85="","Available",SWITCH(C85,"Daily",D85+1,"Weekly",D85+7,"Monthly",EDATE(D85,1),"Quarterly",EDATE(D85,3),"Yearly",EDATE(D85,12),"One-time","Used","Manual","Manual",D85)))</x:f>
+        <x:f>IF(A85="","",IF(D85="","Available",SWITCH(C85,"Daily",D85+1,"Weekly",IFERROR(VLOOKUP(A85,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D85-VLOOKUP(A85,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D85+7),"Monthly",IFERROR(EDATE(VLOOKUP(A85,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A85,'VIP Signups'!$A$5:$B$204,2,FALSE),D85,"M")+1),EDATE(D85,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A85,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A85,'VIP Signups'!$A$5:$B$204,2,FALSE),D85,"M")/3)+1)*3),EDATE(D85,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A85,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A85,'VIP Signups'!$A$5:$B$204,2,FALSE),D85,"Y")+1)*12),EDATE(D85,12)),"One-time","Used","Manual","Manual",D85)))</x:f>
       </x:c>
       <x:c r="F85" s="20" t="str">
         <x:f>IF(A85="","",IF(D85="","Yes",IF(E85="Manual","Manual",IF(E85="Used","No",IF(E85&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12357,7 +12369,7 @@
       <x:c r="C86" s="20"/>
       <x:c r="D86" s="21"/>
       <x:c r="E86" s="21" t="str">
-        <x:f>IF(A86="","",IF(D86="","Available",SWITCH(C86,"Daily",D86+1,"Weekly",D86+7,"Monthly",EDATE(D86,1),"Quarterly",EDATE(D86,3),"Yearly",EDATE(D86,12),"One-time","Used","Manual","Manual",D86)))</x:f>
+        <x:f>IF(A86="","",IF(D86="","Available",SWITCH(C86,"Daily",D86+1,"Weekly",IFERROR(VLOOKUP(A86,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D86-VLOOKUP(A86,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D86+7),"Monthly",IFERROR(EDATE(VLOOKUP(A86,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A86,'VIP Signups'!$A$5:$B$204,2,FALSE),D86,"M")+1),EDATE(D86,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A86,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A86,'VIP Signups'!$A$5:$B$204,2,FALSE),D86,"M")/3)+1)*3),EDATE(D86,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A86,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A86,'VIP Signups'!$A$5:$B$204,2,FALSE),D86,"Y")+1)*12),EDATE(D86,12)),"One-time","Used","Manual","Manual",D86)))</x:f>
       </x:c>
       <x:c r="F86" s="20" t="str">
         <x:f>IF(A86="","",IF(D86="","Yes",IF(E86="Manual","Manual",IF(E86="Used","No",IF(E86&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12380,7 +12392,7 @@
       <x:c r="C87" s="20"/>
       <x:c r="D87" s="21"/>
       <x:c r="E87" s="21" t="str">
-        <x:f>IF(A87="","",IF(D87="","Available",SWITCH(C87,"Daily",D87+1,"Weekly",D87+7,"Monthly",EDATE(D87,1),"Quarterly",EDATE(D87,3),"Yearly",EDATE(D87,12),"One-time","Used","Manual","Manual",D87)))</x:f>
+        <x:f>IF(A87="","",IF(D87="","Available",SWITCH(C87,"Daily",D87+1,"Weekly",IFERROR(VLOOKUP(A87,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D87-VLOOKUP(A87,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D87+7),"Monthly",IFERROR(EDATE(VLOOKUP(A87,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A87,'VIP Signups'!$A$5:$B$204,2,FALSE),D87,"M")+1),EDATE(D87,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A87,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A87,'VIP Signups'!$A$5:$B$204,2,FALSE),D87,"M")/3)+1)*3),EDATE(D87,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A87,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A87,'VIP Signups'!$A$5:$B$204,2,FALSE),D87,"Y")+1)*12),EDATE(D87,12)),"One-time","Used","Manual","Manual",D87)))</x:f>
       </x:c>
       <x:c r="F87" s="20" t="str">
         <x:f>IF(A87="","",IF(D87="","Yes",IF(E87="Manual","Manual",IF(E87="Used","No",IF(E87&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12403,7 +12415,7 @@
       <x:c r="C88" s="20"/>
       <x:c r="D88" s="21"/>
       <x:c r="E88" s="21" t="str">
-        <x:f>IF(A88="","",IF(D88="","Available",SWITCH(C88,"Daily",D88+1,"Weekly",D88+7,"Monthly",EDATE(D88,1),"Quarterly",EDATE(D88,3),"Yearly",EDATE(D88,12),"One-time","Used","Manual","Manual",D88)))</x:f>
+        <x:f>IF(A88="","",IF(D88="","Available",SWITCH(C88,"Daily",D88+1,"Weekly",IFERROR(VLOOKUP(A88,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D88-VLOOKUP(A88,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D88+7),"Monthly",IFERROR(EDATE(VLOOKUP(A88,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A88,'VIP Signups'!$A$5:$B$204,2,FALSE),D88,"M")+1),EDATE(D88,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A88,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A88,'VIP Signups'!$A$5:$B$204,2,FALSE),D88,"M")/3)+1)*3),EDATE(D88,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A88,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A88,'VIP Signups'!$A$5:$B$204,2,FALSE),D88,"Y")+1)*12),EDATE(D88,12)),"One-time","Used","Manual","Manual",D88)))</x:f>
       </x:c>
       <x:c r="F88" s="20" t="str">
         <x:f>IF(A88="","",IF(D88="","Yes",IF(E88="Manual","Manual",IF(E88="Used","No",IF(E88&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12426,7 +12438,7 @@
       <x:c r="C89" s="20"/>
       <x:c r="D89" s="21"/>
       <x:c r="E89" s="21" t="str">
-        <x:f>IF(A89="","",IF(D89="","Available",SWITCH(C89,"Daily",D89+1,"Weekly",D89+7,"Monthly",EDATE(D89,1),"Quarterly",EDATE(D89,3),"Yearly",EDATE(D89,12),"One-time","Used","Manual","Manual",D89)))</x:f>
+        <x:f>IF(A89="","",IF(D89="","Available",SWITCH(C89,"Daily",D89+1,"Weekly",IFERROR(VLOOKUP(A89,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D89-VLOOKUP(A89,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D89+7),"Monthly",IFERROR(EDATE(VLOOKUP(A89,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A89,'VIP Signups'!$A$5:$B$204,2,FALSE),D89,"M")+1),EDATE(D89,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A89,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A89,'VIP Signups'!$A$5:$B$204,2,FALSE),D89,"M")/3)+1)*3),EDATE(D89,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A89,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A89,'VIP Signups'!$A$5:$B$204,2,FALSE),D89,"Y")+1)*12),EDATE(D89,12)),"One-time","Used","Manual","Manual",D89)))</x:f>
       </x:c>
       <x:c r="F89" s="20" t="str">
         <x:f>IF(A89="","",IF(D89="","Yes",IF(E89="Manual","Manual",IF(E89="Used","No",IF(E89&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12449,7 +12461,7 @@
       <x:c r="C90" s="20"/>
       <x:c r="D90" s="21"/>
       <x:c r="E90" s="21" t="str">
-        <x:f>IF(A90="","",IF(D90="","Available",SWITCH(C90,"Daily",D90+1,"Weekly",D90+7,"Monthly",EDATE(D90,1),"Quarterly",EDATE(D90,3),"Yearly",EDATE(D90,12),"One-time","Used","Manual","Manual",D90)))</x:f>
+        <x:f>IF(A90="","",IF(D90="","Available",SWITCH(C90,"Daily",D90+1,"Weekly",IFERROR(VLOOKUP(A90,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D90-VLOOKUP(A90,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D90+7),"Monthly",IFERROR(EDATE(VLOOKUP(A90,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A90,'VIP Signups'!$A$5:$B$204,2,FALSE),D90,"M")+1),EDATE(D90,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A90,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A90,'VIP Signups'!$A$5:$B$204,2,FALSE),D90,"M")/3)+1)*3),EDATE(D90,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A90,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A90,'VIP Signups'!$A$5:$B$204,2,FALSE),D90,"Y")+1)*12),EDATE(D90,12)),"One-time","Used","Manual","Manual",D90)))</x:f>
       </x:c>
       <x:c r="F90" s="20" t="str">
         <x:f>IF(A90="","",IF(D90="","Yes",IF(E90="Manual","Manual",IF(E90="Used","No",IF(E90&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12472,7 +12484,7 @@
       <x:c r="C91" s="20"/>
       <x:c r="D91" s="21"/>
       <x:c r="E91" s="21" t="str">
-        <x:f>IF(A91="","",IF(D91="","Available",SWITCH(C91,"Daily",D91+1,"Weekly",D91+7,"Monthly",EDATE(D91,1),"Quarterly",EDATE(D91,3),"Yearly",EDATE(D91,12),"One-time","Used","Manual","Manual",D91)))</x:f>
+        <x:f>IF(A91="","",IF(D91="","Available",SWITCH(C91,"Daily",D91+1,"Weekly",IFERROR(VLOOKUP(A91,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D91-VLOOKUP(A91,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D91+7),"Monthly",IFERROR(EDATE(VLOOKUP(A91,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A91,'VIP Signups'!$A$5:$B$204,2,FALSE),D91,"M")+1),EDATE(D91,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A91,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A91,'VIP Signups'!$A$5:$B$204,2,FALSE),D91,"M")/3)+1)*3),EDATE(D91,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A91,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A91,'VIP Signups'!$A$5:$B$204,2,FALSE),D91,"Y")+1)*12),EDATE(D91,12)),"One-time","Used","Manual","Manual",D91)))</x:f>
       </x:c>
       <x:c r="F91" s="20" t="str">
         <x:f>IF(A91="","",IF(D91="","Yes",IF(E91="Manual","Manual",IF(E91="Used","No",IF(E91&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12495,7 +12507,7 @@
       <x:c r="C92" s="20"/>
       <x:c r="D92" s="21"/>
       <x:c r="E92" s="21" t="str">
-        <x:f>IF(A92="","",IF(D92="","Available",SWITCH(C92,"Daily",D92+1,"Weekly",D92+7,"Monthly",EDATE(D92,1),"Quarterly",EDATE(D92,3),"Yearly",EDATE(D92,12),"One-time","Used","Manual","Manual",D92)))</x:f>
+        <x:f>IF(A92="","",IF(D92="","Available",SWITCH(C92,"Daily",D92+1,"Weekly",IFERROR(VLOOKUP(A92,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D92-VLOOKUP(A92,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D92+7),"Monthly",IFERROR(EDATE(VLOOKUP(A92,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A92,'VIP Signups'!$A$5:$B$204,2,FALSE),D92,"M")+1),EDATE(D92,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A92,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A92,'VIP Signups'!$A$5:$B$204,2,FALSE),D92,"M")/3)+1)*3),EDATE(D92,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A92,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A92,'VIP Signups'!$A$5:$B$204,2,FALSE),D92,"Y")+1)*12),EDATE(D92,12)),"One-time","Used","Manual","Manual",D92)))</x:f>
       </x:c>
       <x:c r="F92" s="20" t="str">
         <x:f>IF(A92="","",IF(D92="","Yes",IF(E92="Manual","Manual",IF(E92="Used","No",IF(E92&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12518,7 +12530,7 @@
       <x:c r="C93" s="20"/>
       <x:c r="D93" s="21"/>
       <x:c r="E93" s="21" t="str">
-        <x:f>IF(A93="","",IF(D93="","Available",SWITCH(C93,"Daily",D93+1,"Weekly",D93+7,"Monthly",EDATE(D93,1),"Quarterly",EDATE(D93,3),"Yearly",EDATE(D93,12),"One-time","Used","Manual","Manual",D93)))</x:f>
+        <x:f>IF(A93="","",IF(D93="","Available",SWITCH(C93,"Daily",D93+1,"Weekly",IFERROR(VLOOKUP(A93,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D93-VLOOKUP(A93,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D93+7),"Monthly",IFERROR(EDATE(VLOOKUP(A93,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A93,'VIP Signups'!$A$5:$B$204,2,FALSE),D93,"M")+1),EDATE(D93,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A93,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A93,'VIP Signups'!$A$5:$B$204,2,FALSE),D93,"M")/3)+1)*3),EDATE(D93,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A93,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A93,'VIP Signups'!$A$5:$B$204,2,FALSE),D93,"Y")+1)*12),EDATE(D93,12)),"One-time","Used","Manual","Manual",D93)))</x:f>
       </x:c>
       <x:c r="F93" s="20" t="str">
         <x:f>IF(A93="","",IF(D93="","Yes",IF(E93="Manual","Manual",IF(E93="Used","No",IF(E93&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12541,7 +12553,7 @@
       <x:c r="C94" s="20"/>
       <x:c r="D94" s="21"/>
       <x:c r="E94" s="21" t="str">
-        <x:f>IF(A94="","",IF(D94="","Available",SWITCH(C94,"Daily",D94+1,"Weekly",D94+7,"Monthly",EDATE(D94,1),"Quarterly",EDATE(D94,3),"Yearly",EDATE(D94,12),"One-time","Used","Manual","Manual",D94)))</x:f>
+        <x:f>IF(A94="","",IF(D94="","Available",SWITCH(C94,"Daily",D94+1,"Weekly",IFERROR(VLOOKUP(A94,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D94-VLOOKUP(A94,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D94+7),"Monthly",IFERROR(EDATE(VLOOKUP(A94,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A94,'VIP Signups'!$A$5:$B$204,2,FALSE),D94,"M")+1),EDATE(D94,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A94,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A94,'VIP Signups'!$A$5:$B$204,2,FALSE),D94,"M")/3)+1)*3),EDATE(D94,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A94,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A94,'VIP Signups'!$A$5:$B$204,2,FALSE),D94,"Y")+1)*12),EDATE(D94,12)),"One-time","Used","Manual","Manual",D94)))</x:f>
       </x:c>
       <x:c r="F94" s="20" t="str">
         <x:f>IF(A94="","",IF(D94="","Yes",IF(E94="Manual","Manual",IF(E94="Used","No",IF(E94&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12564,7 +12576,7 @@
       <x:c r="C95" s="20"/>
       <x:c r="D95" s="21"/>
       <x:c r="E95" s="21" t="str">
-        <x:f>IF(A95="","",IF(D95="","Available",SWITCH(C95,"Daily",D95+1,"Weekly",D95+7,"Monthly",EDATE(D95,1),"Quarterly",EDATE(D95,3),"Yearly",EDATE(D95,12),"One-time","Used","Manual","Manual",D95)))</x:f>
+        <x:f>IF(A95="","",IF(D95="","Available",SWITCH(C95,"Daily",D95+1,"Weekly",IFERROR(VLOOKUP(A95,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D95-VLOOKUP(A95,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D95+7),"Monthly",IFERROR(EDATE(VLOOKUP(A95,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A95,'VIP Signups'!$A$5:$B$204,2,FALSE),D95,"M")+1),EDATE(D95,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A95,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A95,'VIP Signups'!$A$5:$B$204,2,FALSE),D95,"M")/3)+1)*3),EDATE(D95,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A95,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A95,'VIP Signups'!$A$5:$B$204,2,FALSE),D95,"Y")+1)*12),EDATE(D95,12)),"One-time","Used","Manual","Manual",D95)))</x:f>
       </x:c>
       <x:c r="F95" s="20" t="str">
         <x:f>IF(A95="","",IF(D95="","Yes",IF(E95="Manual","Manual",IF(E95="Used","No",IF(E95&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12587,7 +12599,7 @@
       <x:c r="C96" s="20"/>
       <x:c r="D96" s="21"/>
       <x:c r="E96" s="21" t="str">
-        <x:f>IF(A96="","",IF(D96="","Available",SWITCH(C96,"Daily",D96+1,"Weekly",D96+7,"Monthly",EDATE(D96,1),"Quarterly",EDATE(D96,3),"Yearly",EDATE(D96,12),"One-time","Used","Manual","Manual",D96)))</x:f>
+        <x:f>IF(A96="","",IF(D96="","Available",SWITCH(C96,"Daily",D96+1,"Weekly",IFERROR(VLOOKUP(A96,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D96-VLOOKUP(A96,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D96+7),"Monthly",IFERROR(EDATE(VLOOKUP(A96,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A96,'VIP Signups'!$A$5:$B$204,2,FALSE),D96,"M")+1),EDATE(D96,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A96,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A96,'VIP Signups'!$A$5:$B$204,2,FALSE),D96,"M")/3)+1)*3),EDATE(D96,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A96,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A96,'VIP Signups'!$A$5:$B$204,2,FALSE),D96,"Y")+1)*12),EDATE(D96,12)),"One-time","Used","Manual","Manual",D96)))</x:f>
       </x:c>
       <x:c r="F96" s="20" t="str">
         <x:f>IF(A96="","",IF(D96="","Yes",IF(E96="Manual","Manual",IF(E96="Used","No",IF(E96&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12610,7 +12622,7 @@
       <x:c r="C97" s="20"/>
       <x:c r="D97" s="21"/>
       <x:c r="E97" s="21" t="str">
-        <x:f>IF(A97="","",IF(D97="","Available",SWITCH(C97,"Daily",D97+1,"Weekly",D97+7,"Monthly",EDATE(D97,1),"Quarterly",EDATE(D97,3),"Yearly",EDATE(D97,12),"One-time","Used","Manual","Manual",D97)))</x:f>
+        <x:f>IF(A97="","",IF(D97="","Available",SWITCH(C97,"Daily",D97+1,"Weekly",IFERROR(VLOOKUP(A97,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D97-VLOOKUP(A97,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D97+7),"Monthly",IFERROR(EDATE(VLOOKUP(A97,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A97,'VIP Signups'!$A$5:$B$204,2,FALSE),D97,"M")+1),EDATE(D97,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A97,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A97,'VIP Signups'!$A$5:$B$204,2,FALSE),D97,"M")/3)+1)*3),EDATE(D97,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A97,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A97,'VIP Signups'!$A$5:$B$204,2,FALSE),D97,"Y")+1)*12),EDATE(D97,12)),"One-time","Used","Manual","Manual",D97)))</x:f>
       </x:c>
       <x:c r="F97" s="20" t="str">
         <x:f>IF(A97="","",IF(D97="","Yes",IF(E97="Manual","Manual",IF(E97="Used","No",IF(E97&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12633,7 +12645,7 @@
       <x:c r="C98" s="20"/>
       <x:c r="D98" s="21"/>
       <x:c r="E98" s="21" t="str">
-        <x:f>IF(A98="","",IF(D98="","Available",SWITCH(C98,"Daily",D98+1,"Weekly",D98+7,"Monthly",EDATE(D98,1),"Quarterly",EDATE(D98,3),"Yearly",EDATE(D98,12),"One-time","Used","Manual","Manual",D98)))</x:f>
+        <x:f>IF(A98="","",IF(D98="","Available",SWITCH(C98,"Daily",D98+1,"Weekly",IFERROR(VLOOKUP(A98,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D98-VLOOKUP(A98,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D98+7),"Monthly",IFERROR(EDATE(VLOOKUP(A98,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A98,'VIP Signups'!$A$5:$B$204,2,FALSE),D98,"M")+1),EDATE(D98,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A98,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A98,'VIP Signups'!$A$5:$B$204,2,FALSE),D98,"M")/3)+1)*3),EDATE(D98,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A98,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A98,'VIP Signups'!$A$5:$B$204,2,FALSE),D98,"Y")+1)*12),EDATE(D98,12)),"One-time","Used","Manual","Manual",D98)))</x:f>
       </x:c>
       <x:c r="F98" s="20" t="str">
         <x:f>IF(A98="","",IF(D98="","Yes",IF(E98="Manual","Manual",IF(E98="Used","No",IF(E98&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12656,7 +12668,7 @@
       <x:c r="C99" s="20"/>
       <x:c r="D99" s="21"/>
       <x:c r="E99" s="21" t="str">
-        <x:f>IF(A99="","",IF(D99="","Available",SWITCH(C99,"Daily",D99+1,"Weekly",D99+7,"Monthly",EDATE(D99,1),"Quarterly",EDATE(D99,3),"Yearly",EDATE(D99,12),"One-time","Used","Manual","Manual",D99)))</x:f>
+        <x:f>IF(A99="","",IF(D99="","Available",SWITCH(C99,"Daily",D99+1,"Weekly",IFERROR(VLOOKUP(A99,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D99-VLOOKUP(A99,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D99+7),"Monthly",IFERROR(EDATE(VLOOKUP(A99,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A99,'VIP Signups'!$A$5:$B$204,2,FALSE),D99,"M")+1),EDATE(D99,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A99,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A99,'VIP Signups'!$A$5:$B$204,2,FALSE),D99,"M")/3)+1)*3),EDATE(D99,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A99,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A99,'VIP Signups'!$A$5:$B$204,2,FALSE),D99,"Y")+1)*12),EDATE(D99,12)),"One-time","Used","Manual","Manual",D99)))</x:f>
       </x:c>
       <x:c r="F99" s="20" t="str">
         <x:f>IF(A99="","",IF(D99="","Yes",IF(E99="Manual","Manual",IF(E99="Used","No",IF(E99&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12679,7 +12691,7 @@
       <x:c r="C100" s="20"/>
       <x:c r="D100" s="21"/>
       <x:c r="E100" s="21" t="str">
-        <x:f>IF(A100="","",IF(D100="","Available",SWITCH(C100,"Daily",D100+1,"Weekly",D100+7,"Monthly",EDATE(D100,1),"Quarterly",EDATE(D100,3),"Yearly",EDATE(D100,12),"One-time","Used","Manual","Manual",D100)))</x:f>
+        <x:f>IF(A100="","",IF(D100="","Available",SWITCH(C100,"Daily",D100+1,"Weekly",IFERROR(VLOOKUP(A100,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D100-VLOOKUP(A100,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D100+7),"Monthly",IFERROR(EDATE(VLOOKUP(A100,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A100,'VIP Signups'!$A$5:$B$204,2,FALSE),D100,"M")+1),EDATE(D100,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A100,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A100,'VIP Signups'!$A$5:$B$204,2,FALSE),D100,"M")/3)+1)*3),EDATE(D100,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A100,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A100,'VIP Signups'!$A$5:$B$204,2,FALSE),D100,"Y")+1)*12),EDATE(D100,12)),"One-time","Used","Manual","Manual",D100)))</x:f>
       </x:c>
       <x:c r="F100" s="20" t="str">
         <x:f>IF(A100="","",IF(D100="","Yes",IF(E100="Manual","Manual",IF(E100="Used","No",IF(E100&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12702,7 +12714,7 @@
       <x:c r="C101" s="20"/>
       <x:c r="D101" s="21"/>
       <x:c r="E101" s="21" t="str">
-        <x:f>IF(A101="","",IF(D101="","Available",SWITCH(C101,"Daily",D101+1,"Weekly",D101+7,"Monthly",EDATE(D101,1),"Quarterly",EDATE(D101,3),"Yearly",EDATE(D101,12),"One-time","Used","Manual","Manual",D101)))</x:f>
+        <x:f>IF(A101="","",IF(D101="","Available",SWITCH(C101,"Daily",D101+1,"Weekly",IFERROR(VLOOKUP(A101,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D101-VLOOKUP(A101,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D101+7),"Monthly",IFERROR(EDATE(VLOOKUP(A101,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A101,'VIP Signups'!$A$5:$B$204,2,FALSE),D101,"M")+1),EDATE(D101,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A101,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A101,'VIP Signups'!$A$5:$B$204,2,FALSE),D101,"M")/3)+1)*3),EDATE(D101,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A101,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A101,'VIP Signups'!$A$5:$B$204,2,FALSE),D101,"Y")+1)*12),EDATE(D101,12)),"One-time","Used","Manual","Manual",D101)))</x:f>
       </x:c>
       <x:c r="F101" s="20" t="str">
         <x:f>IF(A101="","",IF(D101="","Yes",IF(E101="Manual","Manual",IF(E101="Used","No",IF(E101&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12725,7 +12737,7 @@
       <x:c r="C102" s="20"/>
       <x:c r="D102" s="21"/>
       <x:c r="E102" s="21" t="str">
-        <x:f>IF(A102="","",IF(D102="","Available",SWITCH(C102,"Daily",D102+1,"Weekly",D102+7,"Monthly",EDATE(D102,1),"Quarterly",EDATE(D102,3),"Yearly",EDATE(D102,12),"One-time","Used","Manual","Manual",D102)))</x:f>
+        <x:f>IF(A102="","",IF(D102="","Available",SWITCH(C102,"Daily",D102+1,"Weekly",IFERROR(VLOOKUP(A102,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D102-VLOOKUP(A102,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D102+7),"Monthly",IFERROR(EDATE(VLOOKUP(A102,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A102,'VIP Signups'!$A$5:$B$204,2,FALSE),D102,"M")+1),EDATE(D102,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A102,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A102,'VIP Signups'!$A$5:$B$204,2,FALSE),D102,"M")/3)+1)*3),EDATE(D102,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A102,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A102,'VIP Signups'!$A$5:$B$204,2,FALSE),D102,"Y")+1)*12),EDATE(D102,12)),"One-time","Used","Manual","Manual",D102)))</x:f>
       </x:c>
       <x:c r="F102" s="20" t="str">
         <x:f>IF(A102="","",IF(D102="","Yes",IF(E102="Manual","Manual",IF(E102="Used","No",IF(E102&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12748,7 +12760,7 @@
       <x:c r="C103" s="20"/>
       <x:c r="D103" s="21"/>
       <x:c r="E103" s="21" t="str">
-        <x:f>IF(A103="","",IF(D103="","Available",SWITCH(C103,"Daily",D103+1,"Weekly",D103+7,"Monthly",EDATE(D103,1),"Quarterly",EDATE(D103,3),"Yearly",EDATE(D103,12),"One-time","Used","Manual","Manual",D103)))</x:f>
+        <x:f>IF(A103="","",IF(D103="","Available",SWITCH(C103,"Daily",D103+1,"Weekly",IFERROR(VLOOKUP(A103,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D103-VLOOKUP(A103,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D103+7),"Monthly",IFERROR(EDATE(VLOOKUP(A103,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A103,'VIP Signups'!$A$5:$B$204,2,FALSE),D103,"M")+1),EDATE(D103,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A103,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A103,'VIP Signups'!$A$5:$B$204,2,FALSE),D103,"M")/3)+1)*3),EDATE(D103,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A103,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A103,'VIP Signups'!$A$5:$B$204,2,FALSE),D103,"Y")+1)*12),EDATE(D103,12)),"One-time","Used","Manual","Manual",D103)))</x:f>
       </x:c>
       <x:c r="F103" s="20" t="str">
         <x:f>IF(A103="","",IF(D103="","Yes",IF(E103="Manual","Manual",IF(E103="Used","No",IF(E103&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12771,7 +12783,7 @@
       <x:c r="C104" s="20"/>
       <x:c r="D104" s="21"/>
       <x:c r="E104" s="21" t="str">
-        <x:f>IF(A104="","",IF(D104="","Available",SWITCH(C104,"Daily",D104+1,"Weekly",D104+7,"Monthly",EDATE(D104,1),"Quarterly",EDATE(D104,3),"Yearly",EDATE(D104,12),"One-time","Used","Manual","Manual",D104)))</x:f>
+        <x:f>IF(A104="","",IF(D104="","Available",SWITCH(C104,"Daily",D104+1,"Weekly",IFERROR(VLOOKUP(A104,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D104-VLOOKUP(A104,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D104+7),"Monthly",IFERROR(EDATE(VLOOKUP(A104,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A104,'VIP Signups'!$A$5:$B$204,2,FALSE),D104,"M")+1),EDATE(D104,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A104,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A104,'VIP Signups'!$A$5:$B$204,2,FALSE),D104,"M")/3)+1)*3),EDATE(D104,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A104,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A104,'VIP Signups'!$A$5:$B$204,2,FALSE),D104,"Y")+1)*12),EDATE(D104,12)),"One-time","Used","Manual","Manual",D104)))</x:f>
       </x:c>
       <x:c r="F104" s="20" t="str">
         <x:f>IF(A104="","",IF(D104="","Yes",IF(E104="Manual","Manual",IF(E104="Used","No",IF(E104&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12794,7 +12806,7 @@
       <x:c r="C105" s="20"/>
       <x:c r="D105" s="21"/>
       <x:c r="E105" s="21" t="str">
-        <x:f>IF(A105="","",IF(D105="","Available",SWITCH(C105,"Daily",D105+1,"Weekly",D105+7,"Monthly",EDATE(D105,1),"Quarterly",EDATE(D105,3),"Yearly",EDATE(D105,12),"One-time","Used","Manual","Manual",D105)))</x:f>
+        <x:f>IF(A105="","",IF(D105="","Available",SWITCH(C105,"Daily",D105+1,"Weekly",IFERROR(VLOOKUP(A105,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D105-VLOOKUP(A105,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D105+7),"Monthly",IFERROR(EDATE(VLOOKUP(A105,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A105,'VIP Signups'!$A$5:$B$204,2,FALSE),D105,"M")+1),EDATE(D105,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A105,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A105,'VIP Signups'!$A$5:$B$204,2,FALSE),D105,"M")/3)+1)*3),EDATE(D105,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A105,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A105,'VIP Signups'!$A$5:$B$204,2,FALSE),D105,"Y")+1)*12),EDATE(D105,12)),"One-time","Used","Manual","Manual",D105)))</x:f>
       </x:c>
       <x:c r="F105" s="20" t="str">
         <x:f>IF(A105="","",IF(D105="","Yes",IF(E105="Manual","Manual",IF(E105="Used","No",IF(E105&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12817,7 +12829,7 @@
       <x:c r="C106" s="20"/>
       <x:c r="D106" s="21"/>
       <x:c r="E106" s="21" t="str">
-        <x:f>IF(A106="","",IF(D106="","Available",SWITCH(C106,"Daily",D106+1,"Weekly",D106+7,"Monthly",EDATE(D106,1),"Quarterly",EDATE(D106,3),"Yearly",EDATE(D106,12),"One-time","Used","Manual","Manual",D106)))</x:f>
+        <x:f>IF(A106="","",IF(D106="","Available",SWITCH(C106,"Daily",D106+1,"Weekly",IFERROR(VLOOKUP(A106,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D106-VLOOKUP(A106,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D106+7),"Monthly",IFERROR(EDATE(VLOOKUP(A106,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A106,'VIP Signups'!$A$5:$B$204,2,FALSE),D106,"M")+1),EDATE(D106,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A106,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A106,'VIP Signups'!$A$5:$B$204,2,FALSE),D106,"M")/3)+1)*3),EDATE(D106,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A106,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A106,'VIP Signups'!$A$5:$B$204,2,FALSE),D106,"Y")+1)*12),EDATE(D106,12)),"One-time","Used","Manual","Manual",D106)))</x:f>
       </x:c>
       <x:c r="F106" s="20" t="str">
         <x:f>IF(A106="","",IF(D106="","Yes",IF(E106="Manual","Manual",IF(E106="Used","No",IF(E106&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12840,7 +12852,7 @@
       <x:c r="C107" s="20"/>
       <x:c r="D107" s="21"/>
       <x:c r="E107" s="21" t="str">
-        <x:f>IF(A107="","",IF(D107="","Available",SWITCH(C107,"Daily",D107+1,"Weekly",D107+7,"Monthly",EDATE(D107,1),"Quarterly",EDATE(D107,3),"Yearly",EDATE(D107,12),"One-time","Used","Manual","Manual",D107)))</x:f>
+        <x:f>IF(A107="","",IF(D107="","Available",SWITCH(C107,"Daily",D107+1,"Weekly",IFERROR(VLOOKUP(A107,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D107-VLOOKUP(A107,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D107+7),"Monthly",IFERROR(EDATE(VLOOKUP(A107,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A107,'VIP Signups'!$A$5:$B$204,2,FALSE),D107,"M")+1),EDATE(D107,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A107,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A107,'VIP Signups'!$A$5:$B$204,2,FALSE),D107,"M")/3)+1)*3),EDATE(D107,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A107,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A107,'VIP Signups'!$A$5:$B$204,2,FALSE),D107,"Y")+1)*12),EDATE(D107,12)),"One-time","Used","Manual","Manual",D107)))</x:f>
       </x:c>
       <x:c r="F107" s="20" t="str">
         <x:f>IF(A107="","",IF(D107="","Yes",IF(E107="Manual","Manual",IF(E107="Used","No",IF(E107&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12863,7 +12875,7 @@
       <x:c r="C108" s="20"/>
       <x:c r="D108" s="21"/>
       <x:c r="E108" s="21" t="str">
-        <x:f>IF(A108="","",IF(D108="","Available",SWITCH(C108,"Daily",D108+1,"Weekly",D108+7,"Monthly",EDATE(D108,1),"Quarterly",EDATE(D108,3),"Yearly",EDATE(D108,12),"One-time","Used","Manual","Manual",D108)))</x:f>
+        <x:f>IF(A108="","",IF(D108="","Available",SWITCH(C108,"Daily",D108+1,"Weekly",IFERROR(VLOOKUP(A108,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D108-VLOOKUP(A108,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D108+7),"Monthly",IFERROR(EDATE(VLOOKUP(A108,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A108,'VIP Signups'!$A$5:$B$204,2,FALSE),D108,"M")+1),EDATE(D108,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A108,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A108,'VIP Signups'!$A$5:$B$204,2,FALSE),D108,"M")/3)+1)*3),EDATE(D108,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A108,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A108,'VIP Signups'!$A$5:$B$204,2,FALSE),D108,"Y")+1)*12),EDATE(D108,12)),"One-time","Used","Manual","Manual",D108)))</x:f>
       </x:c>
       <x:c r="F108" s="20" t="str">
         <x:f>IF(A108="","",IF(D108="","Yes",IF(E108="Manual","Manual",IF(E108="Used","No",IF(E108&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12886,7 +12898,7 @@
       <x:c r="C109" s="20"/>
       <x:c r="D109" s="21"/>
       <x:c r="E109" s="21" t="str">
-        <x:f>IF(A109="","",IF(D109="","Available",SWITCH(C109,"Daily",D109+1,"Weekly",D109+7,"Monthly",EDATE(D109,1),"Quarterly",EDATE(D109,3),"Yearly",EDATE(D109,12),"One-time","Used","Manual","Manual",D109)))</x:f>
+        <x:f>IF(A109="","",IF(D109="","Available",SWITCH(C109,"Daily",D109+1,"Weekly",IFERROR(VLOOKUP(A109,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D109-VLOOKUP(A109,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D109+7),"Monthly",IFERROR(EDATE(VLOOKUP(A109,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A109,'VIP Signups'!$A$5:$B$204,2,FALSE),D109,"M")+1),EDATE(D109,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A109,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A109,'VIP Signups'!$A$5:$B$204,2,FALSE),D109,"M")/3)+1)*3),EDATE(D109,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A109,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A109,'VIP Signups'!$A$5:$B$204,2,FALSE),D109,"Y")+1)*12),EDATE(D109,12)),"One-time","Used","Manual","Manual",D109)))</x:f>
       </x:c>
       <x:c r="F109" s="20" t="str">
         <x:f>IF(A109="","",IF(D109="","Yes",IF(E109="Manual","Manual",IF(E109="Used","No",IF(E109&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12909,7 +12921,7 @@
       <x:c r="C110" s="20"/>
       <x:c r="D110" s="21"/>
       <x:c r="E110" s="21" t="str">
-        <x:f>IF(A110="","",IF(D110="","Available",SWITCH(C110,"Daily",D110+1,"Weekly",D110+7,"Monthly",EDATE(D110,1),"Quarterly",EDATE(D110,3),"Yearly",EDATE(D110,12),"One-time","Used","Manual","Manual",D110)))</x:f>
+        <x:f>IF(A110="","",IF(D110="","Available",SWITCH(C110,"Daily",D110+1,"Weekly",IFERROR(VLOOKUP(A110,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D110-VLOOKUP(A110,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D110+7),"Monthly",IFERROR(EDATE(VLOOKUP(A110,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A110,'VIP Signups'!$A$5:$B$204,2,FALSE),D110,"M")+1),EDATE(D110,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A110,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A110,'VIP Signups'!$A$5:$B$204,2,FALSE),D110,"M")/3)+1)*3),EDATE(D110,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A110,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A110,'VIP Signups'!$A$5:$B$204,2,FALSE),D110,"Y")+1)*12),EDATE(D110,12)),"One-time","Used","Manual","Manual",D110)))</x:f>
       </x:c>
       <x:c r="F110" s="20" t="str">
         <x:f>IF(A110="","",IF(D110="","Yes",IF(E110="Manual","Manual",IF(E110="Used","No",IF(E110&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12932,7 +12944,7 @@
       <x:c r="C111" s="20"/>
       <x:c r="D111" s="21"/>
       <x:c r="E111" s="21" t="str">
-        <x:f>IF(A111="","",IF(D111="","Available",SWITCH(C111,"Daily",D111+1,"Weekly",D111+7,"Monthly",EDATE(D111,1),"Quarterly",EDATE(D111,3),"Yearly",EDATE(D111,12),"One-time","Used","Manual","Manual",D111)))</x:f>
+        <x:f>IF(A111="","",IF(D111="","Available",SWITCH(C111,"Daily",D111+1,"Weekly",IFERROR(VLOOKUP(A111,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D111-VLOOKUP(A111,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D111+7),"Monthly",IFERROR(EDATE(VLOOKUP(A111,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A111,'VIP Signups'!$A$5:$B$204,2,FALSE),D111,"M")+1),EDATE(D111,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A111,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A111,'VIP Signups'!$A$5:$B$204,2,FALSE),D111,"M")/3)+1)*3),EDATE(D111,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A111,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A111,'VIP Signups'!$A$5:$B$204,2,FALSE),D111,"Y")+1)*12),EDATE(D111,12)),"One-time","Used","Manual","Manual",D111)))</x:f>
       </x:c>
       <x:c r="F111" s="20" t="str">
         <x:f>IF(A111="","",IF(D111="","Yes",IF(E111="Manual","Manual",IF(E111="Used","No",IF(E111&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12955,7 +12967,7 @@
       <x:c r="C112" s="20"/>
       <x:c r="D112" s="21"/>
       <x:c r="E112" s="21" t="str">
-        <x:f>IF(A112="","",IF(D112="","Available",SWITCH(C112,"Daily",D112+1,"Weekly",D112+7,"Monthly",EDATE(D112,1),"Quarterly",EDATE(D112,3),"Yearly",EDATE(D112,12),"One-time","Used","Manual","Manual",D112)))</x:f>
+        <x:f>IF(A112="","",IF(D112="","Available",SWITCH(C112,"Daily",D112+1,"Weekly",IFERROR(VLOOKUP(A112,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D112-VLOOKUP(A112,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D112+7),"Monthly",IFERROR(EDATE(VLOOKUP(A112,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A112,'VIP Signups'!$A$5:$B$204,2,FALSE),D112,"M")+1),EDATE(D112,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A112,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A112,'VIP Signups'!$A$5:$B$204,2,FALSE),D112,"M")/3)+1)*3),EDATE(D112,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A112,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A112,'VIP Signups'!$A$5:$B$204,2,FALSE),D112,"Y")+1)*12),EDATE(D112,12)),"One-time","Used","Manual","Manual",D112)))</x:f>
       </x:c>
       <x:c r="F112" s="20" t="str">
         <x:f>IF(A112="","",IF(D112="","Yes",IF(E112="Manual","Manual",IF(E112="Used","No",IF(E112&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -12978,7 +12990,7 @@
       <x:c r="C113" s="20"/>
       <x:c r="D113" s="21"/>
       <x:c r="E113" s="21" t="str">
-        <x:f>IF(A113="","",IF(D113="","Available",SWITCH(C113,"Daily",D113+1,"Weekly",D113+7,"Monthly",EDATE(D113,1),"Quarterly",EDATE(D113,3),"Yearly",EDATE(D113,12),"One-time","Used","Manual","Manual",D113)))</x:f>
+        <x:f>IF(A113="","",IF(D113="","Available",SWITCH(C113,"Daily",D113+1,"Weekly",IFERROR(VLOOKUP(A113,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D113-VLOOKUP(A113,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D113+7),"Monthly",IFERROR(EDATE(VLOOKUP(A113,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A113,'VIP Signups'!$A$5:$B$204,2,FALSE),D113,"M")+1),EDATE(D113,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A113,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A113,'VIP Signups'!$A$5:$B$204,2,FALSE),D113,"M")/3)+1)*3),EDATE(D113,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A113,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A113,'VIP Signups'!$A$5:$B$204,2,FALSE),D113,"Y")+1)*12),EDATE(D113,12)),"One-time","Used","Manual","Manual",D113)))</x:f>
       </x:c>
       <x:c r="F113" s="20" t="str">
         <x:f>IF(A113="","",IF(D113="","Yes",IF(E113="Manual","Manual",IF(E113="Used","No",IF(E113&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13001,7 +13013,7 @@
       <x:c r="C114" s="20"/>
       <x:c r="D114" s="21"/>
       <x:c r="E114" s="21" t="str">
-        <x:f>IF(A114="","",IF(D114="","Available",SWITCH(C114,"Daily",D114+1,"Weekly",D114+7,"Monthly",EDATE(D114,1),"Quarterly",EDATE(D114,3),"Yearly",EDATE(D114,12),"One-time","Used","Manual","Manual",D114)))</x:f>
+        <x:f>IF(A114="","",IF(D114="","Available",SWITCH(C114,"Daily",D114+1,"Weekly",IFERROR(VLOOKUP(A114,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D114-VLOOKUP(A114,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D114+7),"Monthly",IFERROR(EDATE(VLOOKUP(A114,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A114,'VIP Signups'!$A$5:$B$204,2,FALSE),D114,"M")+1),EDATE(D114,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A114,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A114,'VIP Signups'!$A$5:$B$204,2,FALSE),D114,"M")/3)+1)*3),EDATE(D114,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A114,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A114,'VIP Signups'!$A$5:$B$204,2,FALSE),D114,"Y")+1)*12),EDATE(D114,12)),"One-time","Used","Manual","Manual",D114)))</x:f>
       </x:c>
       <x:c r="F114" s="20" t="str">
         <x:f>IF(A114="","",IF(D114="","Yes",IF(E114="Manual","Manual",IF(E114="Used","No",IF(E114&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13024,7 +13036,7 @@
       <x:c r="C115" s="20"/>
       <x:c r="D115" s="21"/>
       <x:c r="E115" s="21" t="str">
-        <x:f>IF(A115="","",IF(D115="","Available",SWITCH(C115,"Daily",D115+1,"Weekly",D115+7,"Monthly",EDATE(D115,1),"Quarterly",EDATE(D115,3),"Yearly",EDATE(D115,12),"One-time","Used","Manual","Manual",D115)))</x:f>
+        <x:f>IF(A115="","",IF(D115="","Available",SWITCH(C115,"Daily",D115+1,"Weekly",IFERROR(VLOOKUP(A115,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D115-VLOOKUP(A115,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D115+7),"Monthly",IFERROR(EDATE(VLOOKUP(A115,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A115,'VIP Signups'!$A$5:$B$204,2,FALSE),D115,"M")+1),EDATE(D115,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A115,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A115,'VIP Signups'!$A$5:$B$204,2,FALSE),D115,"M")/3)+1)*3),EDATE(D115,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A115,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A115,'VIP Signups'!$A$5:$B$204,2,FALSE),D115,"Y")+1)*12),EDATE(D115,12)),"One-time","Used","Manual","Manual",D115)))</x:f>
       </x:c>
       <x:c r="F115" s="20" t="str">
         <x:f>IF(A115="","",IF(D115="","Yes",IF(E115="Manual","Manual",IF(E115="Used","No",IF(E115&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13047,7 +13059,7 @@
       <x:c r="C116" s="20"/>
       <x:c r="D116" s="21"/>
       <x:c r="E116" s="21" t="str">
-        <x:f>IF(A116="","",IF(D116="","Available",SWITCH(C116,"Daily",D116+1,"Weekly",D116+7,"Monthly",EDATE(D116,1),"Quarterly",EDATE(D116,3),"Yearly",EDATE(D116,12),"One-time","Used","Manual","Manual",D116)))</x:f>
+        <x:f>IF(A116="","",IF(D116="","Available",SWITCH(C116,"Daily",D116+1,"Weekly",IFERROR(VLOOKUP(A116,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D116-VLOOKUP(A116,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D116+7),"Monthly",IFERROR(EDATE(VLOOKUP(A116,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A116,'VIP Signups'!$A$5:$B$204,2,FALSE),D116,"M")+1),EDATE(D116,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A116,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A116,'VIP Signups'!$A$5:$B$204,2,FALSE),D116,"M")/3)+1)*3),EDATE(D116,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A116,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A116,'VIP Signups'!$A$5:$B$204,2,FALSE),D116,"Y")+1)*12),EDATE(D116,12)),"One-time","Used","Manual","Manual",D116)))</x:f>
       </x:c>
       <x:c r="F116" s="20" t="str">
         <x:f>IF(A116="","",IF(D116="","Yes",IF(E116="Manual","Manual",IF(E116="Used","No",IF(E116&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13070,7 +13082,7 @@
       <x:c r="C117" s="20"/>
       <x:c r="D117" s="21"/>
       <x:c r="E117" s="21" t="str">
-        <x:f>IF(A117="","",IF(D117="","Available",SWITCH(C117,"Daily",D117+1,"Weekly",D117+7,"Monthly",EDATE(D117,1),"Quarterly",EDATE(D117,3),"Yearly",EDATE(D117,12),"One-time","Used","Manual","Manual",D117)))</x:f>
+        <x:f>IF(A117="","",IF(D117="","Available",SWITCH(C117,"Daily",D117+1,"Weekly",IFERROR(VLOOKUP(A117,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D117-VLOOKUP(A117,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D117+7),"Monthly",IFERROR(EDATE(VLOOKUP(A117,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A117,'VIP Signups'!$A$5:$B$204,2,FALSE),D117,"M")+1),EDATE(D117,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A117,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A117,'VIP Signups'!$A$5:$B$204,2,FALSE),D117,"M")/3)+1)*3),EDATE(D117,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A117,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A117,'VIP Signups'!$A$5:$B$204,2,FALSE),D117,"Y")+1)*12),EDATE(D117,12)),"One-time","Used","Manual","Manual",D117)))</x:f>
       </x:c>
       <x:c r="F117" s="20" t="str">
         <x:f>IF(A117="","",IF(D117="","Yes",IF(E117="Manual","Manual",IF(E117="Used","No",IF(E117&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13093,7 +13105,7 @@
       <x:c r="C118" s="20"/>
       <x:c r="D118" s="21"/>
       <x:c r="E118" s="21" t="str">
-        <x:f>IF(A118="","",IF(D118="","Available",SWITCH(C118,"Daily",D118+1,"Weekly",D118+7,"Monthly",EDATE(D118,1),"Quarterly",EDATE(D118,3),"Yearly",EDATE(D118,12),"One-time","Used","Manual","Manual",D118)))</x:f>
+        <x:f>IF(A118="","",IF(D118="","Available",SWITCH(C118,"Daily",D118+1,"Weekly",IFERROR(VLOOKUP(A118,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D118-VLOOKUP(A118,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D118+7),"Monthly",IFERROR(EDATE(VLOOKUP(A118,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A118,'VIP Signups'!$A$5:$B$204,2,FALSE),D118,"M")+1),EDATE(D118,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A118,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A118,'VIP Signups'!$A$5:$B$204,2,FALSE),D118,"M")/3)+1)*3),EDATE(D118,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A118,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A118,'VIP Signups'!$A$5:$B$204,2,FALSE),D118,"Y")+1)*12),EDATE(D118,12)),"One-time","Used","Manual","Manual",D118)))</x:f>
       </x:c>
       <x:c r="F118" s="20" t="str">
         <x:f>IF(A118="","",IF(D118="","Yes",IF(E118="Manual","Manual",IF(E118="Used","No",IF(E118&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13116,7 +13128,7 @@
       <x:c r="C119" s="20"/>
       <x:c r="D119" s="21"/>
       <x:c r="E119" s="21" t="str">
-        <x:f>IF(A119="","",IF(D119="","Available",SWITCH(C119,"Daily",D119+1,"Weekly",D119+7,"Monthly",EDATE(D119,1),"Quarterly",EDATE(D119,3),"Yearly",EDATE(D119,12),"One-time","Used","Manual","Manual",D119)))</x:f>
+        <x:f>IF(A119="","",IF(D119="","Available",SWITCH(C119,"Daily",D119+1,"Weekly",IFERROR(VLOOKUP(A119,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D119-VLOOKUP(A119,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D119+7),"Monthly",IFERROR(EDATE(VLOOKUP(A119,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A119,'VIP Signups'!$A$5:$B$204,2,FALSE),D119,"M")+1),EDATE(D119,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A119,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A119,'VIP Signups'!$A$5:$B$204,2,FALSE),D119,"M")/3)+1)*3),EDATE(D119,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A119,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A119,'VIP Signups'!$A$5:$B$204,2,FALSE),D119,"Y")+1)*12),EDATE(D119,12)),"One-time","Used","Manual","Manual",D119)))</x:f>
       </x:c>
       <x:c r="F119" s="20" t="str">
         <x:f>IF(A119="","",IF(D119="","Yes",IF(E119="Manual","Manual",IF(E119="Used","No",IF(E119&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13139,7 +13151,7 @@
       <x:c r="C120" s="20"/>
       <x:c r="D120" s="21"/>
       <x:c r="E120" s="21" t="str">
-        <x:f>IF(A120="","",IF(D120="","Available",SWITCH(C120,"Daily",D120+1,"Weekly",D120+7,"Monthly",EDATE(D120,1),"Quarterly",EDATE(D120,3),"Yearly",EDATE(D120,12),"One-time","Used","Manual","Manual",D120)))</x:f>
+        <x:f>IF(A120="","",IF(D120="","Available",SWITCH(C120,"Daily",D120+1,"Weekly",IFERROR(VLOOKUP(A120,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D120-VLOOKUP(A120,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D120+7),"Monthly",IFERROR(EDATE(VLOOKUP(A120,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A120,'VIP Signups'!$A$5:$B$204,2,FALSE),D120,"M")+1),EDATE(D120,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A120,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A120,'VIP Signups'!$A$5:$B$204,2,FALSE),D120,"M")/3)+1)*3),EDATE(D120,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A120,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A120,'VIP Signups'!$A$5:$B$204,2,FALSE),D120,"Y")+1)*12),EDATE(D120,12)),"One-time","Used","Manual","Manual",D120)))</x:f>
       </x:c>
       <x:c r="F120" s="20" t="str">
         <x:f>IF(A120="","",IF(D120="","Yes",IF(E120="Manual","Manual",IF(E120="Used","No",IF(E120&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13162,7 +13174,7 @@
       <x:c r="C121" s="20"/>
       <x:c r="D121" s="21"/>
       <x:c r="E121" s="21" t="str">
-        <x:f>IF(A121="","",IF(D121="","Available",SWITCH(C121,"Daily",D121+1,"Weekly",D121+7,"Monthly",EDATE(D121,1),"Quarterly",EDATE(D121,3),"Yearly",EDATE(D121,12),"One-time","Used","Manual","Manual",D121)))</x:f>
+        <x:f>IF(A121="","",IF(D121="","Available",SWITCH(C121,"Daily",D121+1,"Weekly",IFERROR(VLOOKUP(A121,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D121-VLOOKUP(A121,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D121+7),"Monthly",IFERROR(EDATE(VLOOKUP(A121,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A121,'VIP Signups'!$A$5:$B$204,2,FALSE),D121,"M")+1),EDATE(D121,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A121,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A121,'VIP Signups'!$A$5:$B$204,2,FALSE),D121,"M")/3)+1)*3),EDATE(D121,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A121,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A121,'VIP Signups'!$A$5:$B$204,2,FALSE),D121,"Y")+1)*12),EDATE(D121,12)),"One-time","Used","Manual","Manual",D121)))</x:f>
       </x:c>
       <x:c r="F121" s="20" t="str">
         <x:f>IF(A121="","",IF(D121="","Yes",IF(E121="Manual","Manual",IF(E121="Used","No",IF(E121&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13185,7 +13197,7 @@
       <x:c r="C122" s="20"/>
       <x:c r="D122" s="21"/>
       <x:c r="E122" s="21" t="str">
-        <x:f>IF(A122="","",IF(D122="","Available",SWITCH(C122,"Daily",D122+1,"Weekly",D122+7,"Monthly",EDATE(D122,1),"Quarterly",EDATE(D122,3),"Yearly",EDATE(D122,12),"One-time","Used","Manual","Manual",D122)))</x:f>
+        <x:f>IF(A122="","",IF(D122="","Available",SWITCH(C122,"Daily",D122+1,"Weekly",IFERROR(VLOOKUP(A122,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D122-VLOOKUP(A122,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D122+7),"Monthly",IFERROR(EDATE(VLOOKUP(A122,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A122,'VIP Signups'!$A$5:$B$204,2,FALSE),D122,"M")+1),EDATE(D122,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A122,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A122,'VIP Signups'!$A$5:$B$204,2,FALSE),D122,"M")/3)+1)*3),EDATE(D122,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A122,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A122,'VIP Signups'!$A$5:$B$204,2,FALSE),D122,"Y")+1)*12),EDATE(D122,12)),"One-time","Used","Manual","Manual",D122)))</x:f>
       </x:c>
       <x:c r="F122" s="20" t="str">
         <x:f>IF(A122="","",IF(D122="","Yes",IF(E122="Manual","Manual",IF(E122="Used","No",IF(E122&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13208,7 +13220,7 @@
       <x:c r="C123" s="20"/>
       <x:c r="D123" s="21"/>
       <x:c r="E123" s="21" t="str">
-        <x:f>IF(A123="","",IF(D123="","Available",SWITCH(C123,"Daily",D123+1,"Weekly",D123+7,"Monthly",EDATE(D123,1),"Quarterly",EDATE(D123,3),"Yearly",EDATE(D123,12),"One-time","Used","Manual","Manual",D123)))</x:f>
+        <x:f>IF(A123="","",IF(D123="","Available",SWITCH(C123,"Daily",D123+1,"Weekly",IFERROR(VLOOKUP(A123,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D123-VLOOKUP(A123,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D123+7),"Monthly",IFERROR(EDATE(VLOOKUP(A123,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A123,'VIP Signups'!$A$5:$B$204,2,FALSE),D123,"M")+1),EDATE(D123,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A123,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A123,'VIP Signups'!$A$5:$B$204,2,FALSE),D123,"M")/3)+1)*3),EDATE(D123,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A123,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A123,'VIP Signups'!$A$5:$B$204,2,FALSE),D123,"Y")+1)*12),EDATE(D123,12)),"One-time","Used","Manual","Manual",D123)))</x:f>
       </x:c>
       <x:c r="F123" s="20" t="str">
         <x:f>IF(A123="","",IF(D123="","Yes",IF(E123="Manual","Manual",IF(E123="Used","No",IF(E123&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13231,7 +13243,7 @@
       <x:c r="C124" s="20"/>
       <x:c r="D124" s="21"/>
       <x:c r="E124" s="21" t="str">
-        <x:f>IF(A124="","",IF(D124="","Available",SWITCH(C124,"Daily",D124+1,"Weekly",D124+7,"Monthly",EDATE(D124,1),"Quarterly",EDATE(D124,3),"Yearly",EDATE(D124,12),"One-time","Used","Manual","Manual",D124)))</x:f>
+        <x:f>IF(A124="","",IF(D124="","Available",SWITCH(C124,"Daily",D124+1,"Weekly",IFERROR(VLOOKUP(A124,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D124-VLOOKUP(A124,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D124+7),"Monthly",IFERROR(EDATE(VLOOKUP(A124,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A124,'VIP Signups'!$A$5:$B$204,2,FALSE),D124,"M")+1),EDATE(D124,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A124,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A124,'VIP Signups'!$A$5:$B$204,2,FALSE),D124,"M")/3)+1)*3),EDATE(D124,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A124,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A124,'VIP Signups'!$A$5:$B$204,2,FALSE),D124,"Y")+1)*12),EDATE(D124,12)),"One-time","Used","Manual","Manual",D124)))</x:f>
       </x:c>
       <x:c r="F124" s="20" t="str">
         <x:f>IF(A124="","",IF(D124="","Yes",IF(E124="Manual","Manual",IF(E124="Used","No",IF(E124&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13254,7 +13266,7 @@
       <x:c r="C125" s="20"/>
       <x:c r="D125" s="21"/>
       <x:c r="E125" s="21" t="str">
-        <x:f>IF(A125="","",IF(D125="","Available",SWITCH(C125,"Daily",D125+1,"Weekly",D125+7,"Monthly",EDATE(D125,1),"Quarterly",EDATE(D125,3),"Yearly",EDATE(D125,12),"One-time","Used","Manual","Manual",D125)))</x:f>
+        <x:f>IF(A125="","",IF(D125="","Available",SWITCH(C125,"Daily",D125+1,"Weekly",IFERROR(VLOOKUP(A125,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D125-VLOOKUP(A125,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D125+7),"Monthly",IFERROR(EDATE(VLOOKUP(A125,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A125,'VIP Signups'!$A$5:$B$204,2,FALSE),D125,"M")+1),EDATE(D125,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A125,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A125,'VIP Signups'!$A$5:$B$204,2,FALSE),D125,"M")/3)+1)*3),EDATE(D125,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A125,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A125,'VIP Signups'!$A$5:$B$204,2,FALSE),D125,"Y")+1)*12),EDATE(D125,12)),"One-time","Used","Manual","Manual",D125)))</x:f>
       </x:c>
       <x:c r="F125" s="20" t="str">
         <x:f>IF(A125="","",IF(D125="","Yes",IF(E125="Manual","Manual",IF(E125="Used","No",IF(E125&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13277,7 +13289,7 @@
       <x:c r="C126" s="20"/>
       <x:c r="D126" s="21"/>
       <x:c r="E126" s="21" t="str">
-        <x:f>IF(A126="","",IF(D126="","Available",SWITCH(C126,"Daily",D126+1,"Weekly",D126+7,"Monthly",EDATE(D126,1),"Quarterly",EDATE(D126,3),"Yearly",EDATE(D126,12),"One-time","Used","Manual","Manual",D126)))</x:f>
+        <x:f>IF(A126="","",IF(D126="","Available",SWITCH(C126,"Daily",D126+1,"Weekly",IFERROR(VLOOKUP(A126,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D126-VLOOKUP(A126,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D126+7),"Monthly",IFERROR(EDATE(VLOOKUP(A126,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A126,'VIP Signups'!$A$5:$B$204,2,FALSE),D126,"M")+1),EDATE(D126,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A126,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A126,'VIP Signups'!$A$5:$B$204,2,FALSE),D126,"M")/3)+1)*3),EDATE(D126,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A126,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A126,'VIP Signups'!$A$5:$B$204,2,FALSE),D126,"Y")+1)*12),EDATE(D126,12)),"One-time","Used","Manual","Manual",D126)))</x:f>
       </x:c>
       <x:c r="F126" s="20" t="str">
         <x:f>IF(A126="","",IF(D126="","Yes",IF(E126="Manual","Manual",IF(E126="Used","No",IF(E126&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13300,7 +13312,7 @@
       <x:c r="C127" s="20"/>
       <x:c r="D127" s="21"/>
       <x:c r="E127" s="21" t="str">
-        <x:f>IF(A127="","",IF(D127="","Available",SWITCH(C127,"Daily",D127+1,"Weekly",D127+7,"Monthly",EDATE(D127,1),"Quarterly",EDATE(D127,3),"Yearly",EDATE(D127,12),"One-time","Used","Manual","Manual",D127)))</x:f>
+        <x:f>IF(A127="","",IF(D127="","Available",SWITCH(C127,"Daily",D127+1,"Weekly",IFERROR(VLOOKUP(A127,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D127-VLOOKUP(A127,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D127+7),"Monthly",IFERROR(EDATE(VLOOKUP(A127,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A127,'VIP Signups'!$A$5:$B$204,2,FALSE),D127,"M")+1),EDATE(D127,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A127,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A127,'VIP Signups'!$A$5:$B$204,2,FALSE),D127,"M")/3)+1)*3),EDATE(D127,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A127,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A127,'VIP Signups'!$A$5:$B$204,2,FALSE),D127,"Y")+1)*12),EDATE(D127,12)),"One-time","Used","Manual","Manual",D127)))</x:f>
       </x:c>
       <x:c r="F127" s="20" t="str">
         <x:f>IF(A127="","",IF(D127="","Yes",IF(E127="Manual","Manual",IF(E127="Used","No",IF(E127&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13323,7 +13335,7 @@
       <x:c r="C128" s="20"/>
       <x:c r="D128" s="21"/>
       <x:c r="E128" s="21" t="str">
-        <x:f>IF(A128="","",IF(D128="","Available",SWITCH(C128,"Daily",D128+1,"Weekly",D128+7,"Monthly",EDATE(D128,1),"Quarterly",EDATE(D128,3),"Yearly",EDATE(D128,12),"One-time","Used","Manual","Manual",D128)))</x:f>
+        <x:f>IF(A128="","",IF(D128="","Available",SWITCH(C128,"Daily",D128+1,"Weekly",IFERROR(VLOOKUP(A128,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D128-VLOOKUP(A128,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D128+7),"Monthly",IFERROR(EDATE(VLOOKUP(A128,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A128,'VIP Signups'!$A$5:$B$204,2,FALSE),D128,"M")+1),EDATE(D128,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A128,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A128,'VIP Signups'!$A$5:$B$204,2,FALSE),D128,"M")/3)+1)*3),EDATE(D128,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A128,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A128,'VIP Signups'!$A$5:$B$204,2,FALSE),D128,"Y")+1)*12),EDATE(D128,12)),"One-time","Used","Manual","Manual",D128)))</x:f>
       </x:c>
       <x:c r="F128" s="20" t="str">
         <x:f>IF(A128="","",IF(D128="","Yes",IF(E128="Manual","Manual",IF(E128="Used","No",IF(E128&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13346,7 +13358,7 @@
       <x:c r="C129" s="20"/>
       <x:c r="D129" s="21"/>
       <x:c r="E129" s="21" t="str">
-        <x:f>IF(A129="","",IF(D129="","Available",SWITCH(C129,"Daily",D129+1,"Weekly",D129+7,"Monthly",EDATE(D129,1),"Quarterly",EDATE(D129,3),"Yearly",EDATE(D129,12),"One-time","Used","Manual","Manual",D129)))</x:f>
+        <x:f>IF(A129="","",IF(D129="","Available",SWITCH(C129,"Daily",D129+1,"Weekly",IFERROR(VLOOKUP(A129,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D129-VLOOKUP(A129,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D129+7),"Monthly",IFERROR(EDATE(VLOOKUP(A129,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A129,'VIP Signups'!$A$5:$B$204,2,FALSE),D129,"M")+1),EDATE(D129,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A129,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A129,'VIP Signups'!$A$5:$B$204,2,FALSE),D129,"M")/3)+1)*3),EDATE(D129,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A129,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A129,'VIP Signups'!$A$5:$B$204,2,FALSE),D129,"Y")+1)*12),EDATE(D129,12)),"One-time","Used","Manual","Manual",D129)))</x:f>
       </x:c>
       <x:c r="F129" s="20" t="str">
         <x:f>IF(A129="","",IF(D129="","Yes",IF(E129="Manual","Manual",IF(E129="Used","No",IF(E129&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13369,7 +13381,7 @@
       <x:c r="C130" s="20"/>
       <x:c r="D130" s="21"/>
       <x:c r="E130" s="21" t="str">
-        <x:f>IF(A130="","",IF(D130="","Available",SWITCH(C130,"Daily",D130+1,"Weekly",D130+7,"Monthly",EDATE(D130,1),"Quarterly",EDATE(D130,3),"Yearly",EDATE(D130,12),"One-time","Used","Manual","Manual",D130)))</x:f>
+        <x:f>IF(A130="","",IF(D130="","Available",SWITCH(C130,"Daily",D130+1,"Weekly",IFERROR(VLOOKUP(A130,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D130-VLOOKUP(A130,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D130+7),"Monthly",IFERROR(EDATE(VLOOKUP(A130,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A130,'VIP Signups'!$A$5:$B$204,2,FALSE),D130,"M")+1),EDATE(D130,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A130,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A130,'VIP Signups'!$A$5:$B$204,2,FALSE),D130,"M")/3)+1)*3),EDATE(D130,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A130,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A130,'VIP Signups'!$A$5:$B$204,2,FALSE),D130,"Y")+1)*12),EDATE(D130,12)),"One-time","Used","Manual","Manual",D130)))</x:f>
       </x:c>
       <x:c r="F130" s="20" t="str">
         <x:f>IF(A130="","",IF(D130="","Yes",IF(E130="Manual","Manual",IF(E130="Used","No",IF(E130&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13392,7 +13404,7 @@
       <x:c r="C131" s="20"/>
       <x:c r="D131" s="21"/>
       <x:c r="E131" s="21" t="str">
-        <x:f>IF(A131="","",IF(D131="","Available",SWITCH(C131,"Daily",D131+1,"Weekly",D131+7,"Monthly",EDATE(D131,1),"Quarterly",EDATE(D131,3),"Yearly",EDATE(D131,12),"One-time","Used","Manual","Manual",D131)))</x:f>
+        <x:f>IF(A131="","",IF(D131="","Available",SWITCH(C131,"Daily",D131+1,"Weekly",IFERROR(VLOOKUP(A131,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D131-VLOOKUP(A131,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D131+7),"Monthly",IFERROR(EDATE(VLOOKUP(A131,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A131,'VIP Signups'!$A$5:$B$204,2,FALSE),D131,"M")+1),EDATE(D131,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A131,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A131,'VIP Signups'!$A$5:$B$204,2,FALSE),D131,"M")/3)+1)*3),EDATE(D131,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A131,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A131,'VIP Signups'!$A$5:$B$204,2,FALSE),D131,"Y")+1)*12),EDATE(D131,12)),"One-time","Used","Manual","Manual",D131)))</x:f>
       </x:c>
       <x:c r="F131" s="20" t="str">
         <x:f>IF(A131="","",IF(D131="","Yes",IF(E131="Manual","Manual",IF(E131="Used","No",IF(E131&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13415,7 +13427,7 @@
       <x:c r="C132" s="20"/>
       <x:c r="D132" s="21"/>
       <x:c r="E132" s="21" t="str">
-        <x:f>IF(A132="","",IF(D132="","Available",SWITCH(C132,"Daily",D132+1,"Weekly",D132+7,"Monthly",EDATE(D132,1),"Quarterly",EDATE(D132,3),"Yearly",EDATE(D132,12),"One-time","Used","Manual","Manual",D132)))</x:f>
+        <x:f>IF(A132="","",IF(D132="","Available",SWITCH(C132,"Daily",D132+1,"Weekly",IFERROR(VLOOKUP(A132,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D132-VLOOKUP(A132,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D132+7),"Monthly",IFERROR(EDATE(VLOOKUP(A132,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A132,'VIP Signups'!$A$5:$B$204,2,FALSE),D132,"M")+1),EDATE(D132,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A132,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A132,'VIP Signups'!$A$5:$B$204,2,FALSE),D132,"M")/3)+1)*3),EDATE(D132,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A132,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A132,'VIP Signups'!$A$5:$B$204,2,FALSE),D132,"Y")+1)*12),EDATE(D132,12)),"One-time","Used","Manual","Manual",D132)))</x:f>
       </x:c>
       <x:c r="F132" s="20" t="str">
         <x:f>IF(A132="","",IF(D132="","Yes",IF(E132="Manual","Manual",IF(E132="Used","No",IF(E132&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13438,7 +13450,7 @@
       <x:c r="C133" s="20"/>
       <x:c r="D133" s="21"/>
       <x:c r="E133" s="21" t="str">
-        <x:f>IF(A133="","",IF(D133="","Available",SWITCH(C133,"Daily",D133+1,"Weekly",D133+7,"Monthly",EDATE(D133,1),"Quarterly",EDATE(D133,3),"Yearly",EDATE(D133,12),"One-time","Used","Manual","Manual",D133)))</x:f>
+        <x:f>IF(A133="","",IF(D133="","Available",SWITCH(C133,"Daily",D133+1,"Weekly",IFERROR(VLOOKUP(A133,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D133-VLOOKUP(A133,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D133+7),"Monthly",IFERROR(EDATE(VLOOKUP(A133,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A133,'VIP Signups'!$A$5:$B$204,2,FALSE),D133,"M")+1),EDATE(D133,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A133,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A133,'VIP Signups'!$A$5:$B$204,2,FALSE),D133,"M")/3)+1)*3),EDATE(D133,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A133,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A133,'VIP Signups'!$A$5:$B$204,2,FALSE),D133,"Y")+1)*12),EDATE(D133,12)),"One-time","Used","Manual","Manual",D133)))</x:f>
       </x:c>
       <x:c r="F133" s="20" t="str">
         <x:f>IF(A133="","",IF(D133="","Yes",IF(E133="Manual","Manual",IF(E133="Used","No",IF(E133&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13461,7 +13473,7 @@
       <x:c r="C134" s="20"/>
       <x:c r="D134" s="21"/>
       <x:c r="E134" s="21" t="str">
-        <x:f>IF(A134="","",IF(D134="","Available",SWITCH(C134,"Daily",D134+1,"Weekly",D134+7,"Monthly",EDATE(D134,1),"Quarterly",EDATE(D134,3),"Yearly",EDATE(D134,12),"One-time","Used","Manual","Manual",D134)))</x:f>
+        <x:f>IF(A134="","",IF(D134="","Available",SWITCH(C134,"Daily",D134+1,"Weekly",IFERROR(VLOOKUP(A134,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D134-VLOOKUP(A134,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D134+7),"Monthly",IFERROR(EDATE(VLOOKUP(A134,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A134,'VIP Signups'!$A$5:$B$204,2,FALSE),D134,"M")+1),EDATE(D134,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A134,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A134,'VIP Signups'!$A$5:$B$204,2,FALSE),D134,"M")/3)+1)*3),EDATE(D134,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A134,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A134,'VIP Signups'!$A$5:$B$204,2,FALSE),D134,"Y")+1)*12),EDATE(D134,12)),"One-time","Used","Manual","Manual",D134)))</x:f>
       </x:c>
       <x:c r="F134" s="20" t="str">
         <x:f>IF(A134="","",IF(D134="","Yes",IF(E134="Manual","Manual",IF(E134="Used","No",IF(E134&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13484,7 +13496,7 @@
       <x:c r="C135" s="20"/>
       <x:c r="D135" s="21"/>
       <x:c r="E135" s="21" t="str">
-        <x:f>IF(A135="","",IF(D135="","Available",SWITCH(C135,"Daily",D135+1,"Weekly",D135+7,"Monthly",EDATE(D135,1),"Quarterly",EDATE(D135,3),"Yearly",EDATE(D135,12),"One-time","Used","Manual","Manual",D135)))</x:f>
+        <x:f>IF(A135="","",IF(D135="","Available",SWITCH(C135,"Daily",D135+1,"Weekly",IFERROR(VLOOKUP(A135,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D135-VLOOKUP(A135,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D135+7),"Monthly",IFERROR(EDATE(VLOOKUP(A135,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A135,'VIP Signups'!$A$5:$B$204,2,FALSE),D135,"M")+1),EDATE(D135,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A135,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A135,'VIP Signups'!$A$5:$B$204,2,FALSE),D135,"M")/3)+1)*3),EDATE(D135,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A135,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A135,'VIP Signups'!$A$5:$B$204,2,FALSE),D135,"Y")+1)*12),EDATE(D135,12)),"One-time","Used","Manual","Manual",D135)))</x:f>
       </x:c>
       <x:c r="F135" s="20" t="str">
         <x:f>IF(A135="","",IF(D135="","Yes",IF(E135="Manual","Manual",IF(E135="Used","No",IF(E135&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13507,7 +13519,7 @@
       <x:c r="C136" s="20"/>
       <x:c r="D136" s="21"/>
       <x:c r="E136" s="21" t="str">
-        <x:f>IF(A136="","",IF(D136="","Available",SWITCH(C136,"Daily",D136+1,"Weekly",D136+7,"Monthly",EDATE(D136,1),"Quarterly",EDATE(D136,3),"Yearly",EDATE(D136,12),"One-time","Used","Manual","Manual",D136)))</x:f>
+        <x:f>IF(A136="","",IF(D136="","Available",SWITCH(C136,"Daily",D136+1,"Weekly",IFERROR(VLOOKUP(A136,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D136-VLOOKUP(A136,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D136+7),"Monthly",IFERROR(EDATE(VLOOKUP(A136,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A136,'VIP Signups'!$A$5:$B$204,2,FALSE),D136,"M")+1),EDATE(D136,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A136,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A136,'VIP Signups'!$A$5:$B$204,2,FALSE),D136,"M")/3)+1)*3),EDATE(D136,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A136,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A136,'VIP Signups'!$A$5:$B$204,2,FALSE),D136,"Y")+1)*12),EDATE(D136,12)),"One-time","Used","Manual","Manual",D136)))</x:f>
       </x:c>
       <x:c r="F136" s="20" t="str">
         <x:f>IF(A136="","",IF(D136="","Yes",IF(E136="Manual","Manual",IF(E136="Used","No",IF(E136&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13530,7 +13542,7 @@
       <x:c r="C137" s="20"/>
       <x:c r="D137" s="21"/>
       <x:c r="E137" s="21" t="str">
-        <x:f>IF(A137="","",IF(D137="","Available",SWITCH(C137,"Daily",D137+1,"Weekly",D137+7,"Monthly",EDATE(D137,1),"Quarterly",EDATE(D137,3),"Yearly",EDATE(D137,12),"One-time","Used","Manual","Manual",D137)))</x:f>
+        <x:f>IF(A137="","",IF(D137="","Available",SWITCH(C137,"Daily",D137+1,"Weekly",IFERROR(VLOOKUP(A137,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D137-VLOOKUP(A137,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D137+7),"Monthly",IFERROR(EDATE(VLOOKUP(A137,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A137,'VIP Signups'!$A$5:$B$204,2,FALSE),D137,"M")+1),EDATE(D137,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A137,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A137,'VIP Signups'!$A$5:$B$204,2,FALSE),D137,"M")/3)+1)*3),EDATE(D137,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A137,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A137,'VIP Signups'!$A$5:$B$204,2,FALSE),D137,"Y")+1)*12),EDATE(D137,12)),"One-time","Used","Manual","Manual",D137)))</x:f>
       </x:c>
       <x:c r="F137" s="20" t="str">
         <x:f>IF(A137="","",IF(D137="","Yes",IF(E137="Manual","Manual",IF(E137="Used","No",IF(E137&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13553,7 +13565,7 @@
       <x:c r="C138" s="20"/>
       <x:c r="D138" s="21"/>
       <x:c r="E138" s="21" t="str">
-        <x:f>IF(A138="","",IF(D138="","Available",SWITCH(C138,"Daily",D138+1,"Weekly",D138+7,"Monthly",EDATE(D138,1),"Quarterly",EDATE(D138,3),"Yearly",EDATE(D138,12),"One-time","Used","Manual","Manual",D138)))</x:f>
+        <x:f>IF(A138="","",IF(D138="","Available",SWITCH(C138,"Daily",D138+1,"Weekly",IFERROR(VLOOKUP(A138,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D138-VLOOKUP(A138,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D138+7),"Monthly",IFERROR(EDATE(VLOOKUP(A138,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A138,'VIP Signups'!$A$5:$B$204,2,FALSE),D138,"M")+1),EDATE(D138,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A138,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A138,'VIP Signups'!$A$5:$B$204,2,FALSE),D138,"M")/3)+1)*3),EDATE(D138,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A138,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A138,'VIP Signups'!$A$5:$B$204,2,FALSE),D138,"Y")+1)*12),EDATE(D138,12)),"One-time","Used","Manual","Manual",D138)))</x:f>
       </x:c>
       <x:c r="F138" s="20" t="str">
         <x:f>IF(A138="","",IF(D138="","Yes",IF(E138="Manual","Manual",IF(E138="Used","No",IF(E138&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13576,7 +13588,7 @@
       <x:c r="C139" s="20"/>
       <x:c r="D139" s="21"/>
       <x:c r="E139" s="21" t="str">
-        <x:f>IF(A139="","",IF(D139="","Available",SWITCH(C139,"Daily",D139+1,"Weekly",D139+7,"Monthly",EDATE(D139,1),"Quarterly",EDATE(D139,3),"Yearly",EDATE(D139,12),"One-time","Used","Manual","Manual",D139)))</x:f>
+        <x:f>IF(A139="","",IF(D139="","Available",SWITCH(C139,"Daily",D139+1,"Weekly",IFERROR(VLOOKUP(A139,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D139-VLOOKUP(A139,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D139+7),"Monthly",IFERROR(EDATE(VLOOKUP(A139,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A139,'VIP Signups'!$A$5:$B$204,2,FALSE),D139,"M")+1),EDATE(D139,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A139,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A139,'VIP Signups'!$A$5:$B$204,2,FALSE),D139,"M")/3)+1)*3),EDATE(D139,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A139,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A139,'VIP Signups'!$A$5:$B$204,2,FALSE),D139,"Y")+1)*12),EDATE(D139,12)),"One-time","Used","Manual","Manual",D139)))</x:f>
       </x:c>
       <x:c r="F139" s="20" t="str">
         <x:f>IF(A139="","",IF(D139="","Yes",IF(E139="Manual","Manual",IF(E139="Used","No",IF(E139&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13599,7 +13611,7 @@
       <x:c r="C140" s="20"/>
       <x:c r="D140" s="21"/>
       <x:c r="E140" s="21" t="str">
-        <x:f>IF(A140="","",IF(D140="","Available",SWITCH(C140,"Daily",D140+1,"Weekly",D140+7,"Monthly",EDATE(D140,1),"Quarterly",EDATE(D140,3),"Yearly",EDATE(D140,12),"One-time","Used","Manual","Manual",D140)))</x:f>
+        <x:f>IF(A140="","",IF(D140="","Available",SWITCH(C140,"Daily",D140+1,"Weekly",IFERROR(VLOOKUP(A140,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D140-VLOOKUP(A140,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D140+7),"Monthly",IFERROR(EDATE(VLOOKUP(A140,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A140,'VIP Signups'!$A$5:$B$204,2,FALSE),D140,"M")+1),EDATE(D140,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A140,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A140,'VIP Signups'!$A$5:$B$204,2,FALSE),D140,"M")/3)+1)*3),EDATE(D140,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A140,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A140,'VIP Signups'!$A$5:$B$204,2,FALSE),D140,"Y")+1)*12),EDATE(D140,12)),"One-time","Used","Manual","Manual",D140)))</x:f>
       </x:c>
       <x:c r="F140" s="20" t="str">
         <x:f>IF(A140="","",IF(D140="","Yes",IF(E140="Manual","Manual",IF(E140="Used","No",IF(E140&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13622,7 +13634,7 @@
       <x:c r="C141" s="20"/>
       <x:c r="D141" s="21"/>
       <x:c r="E141" s="21" t="str">
-        <x:f>IF(A141="","",IF(D141="","Available",SWITCH(C141,"Daily",D141+1,"Weekly",D141+7,"Monthly",EDATE(D141,1),"Quarterly",EDATE(D141,3),"Yearly",EDATE(D141,12),"One-time","Used","Manual","Manual",D141)))</x:f>
+        <x:f>IF(A141="","",IF(D141="","Available",SWITCH(C141,"Daily",D141+1,"Weekly",IFERROR(VLOOKUP(A141,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D141-VLOOKUP(A141,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D141+7),"Monthly",IFERROR(EDATE(VLOOKUP(A141,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A141,'VIP Signups'!$A$5:$B$204,2,FALSE),D141,"M")+1),EDATE(D141,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A141,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A141,'VIP Signups'!$A$5:$B$204,2,FALSE),D141,"M")/3)+1)*3),EDATE(D141,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A141,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A141,'VIP Signups'!$A$5:$B$204,2,FALSE),D141,"Y")+1)*12),EDATE(D141,12)),"One-time","Used","Manual","Manual",D141)))</x:f>
       </x:c>
       <x:c r="F141" s="20" t="str">
         <x:f>IF(A141="","",IF(D141="","Yes",IF(E141="Manual","Manual",IF(E141="Used","No",IF(E141&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13645,7 +13657,7 @@
       <x:c r="C142" s="20"/>
       <x:c r="D142" s="21"/>
       <x:c r="E142" s="21" t="str">
-        <x:f>IF(A142="","",IF(D142="","Available",SWITCH(C142,"Daily",D142+1,"Weekly",D142+7,"Monthly",EDATE(D142,1),"Quarterly",EDATE(D142,3),"Yearly",EDATE(D142,12),"One-time","Used","Manual","Manual",D142)))</x:f>
+        <x:f>IF(A142="","",IF(D142="","Available",SWITCH(C142,"Daily",D142+1,"Weekly",IFERROR(VLOOKUP(A142,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D142-VLOOKUP(A142,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D142+7),"Monthly",IFERROR(EDATE(VLOOKUP(A142,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A142,'VIP Signups'!$A$5:$B$204,2,FALSE),D142,"M")+1),EDATE(D142,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A142,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A142,'VIP Signups'!$A$5:$B$204,2,FALSE),D142,"M")/3)+1)*3),EDATE(D142,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A142,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A142,'VIP Signups'!$A$5:$B$204,2,FALSE),D142,"Y")+1)*12),EDATE(D142,12)),"One-time","Used","Manual","Manual",D142)))</x:f>
       </x:c>
       <x:c r="F142" s="20" t="str">
         <x:f>IF(A142="","",IF(D142="","Yes",IF(E142="Manual","Manual",IF(E142="Used","No",IF(E142&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13668,7 +13680,7 @@
       <x:c r="C143" s="20"/>
       <x:c r="D143" s="21"/>
       <x:c r="E143" s="21" t="str">
-        <x:f>IF(A143="","",IF(D143="","Available",SWITCH(C143,"Daily",D143+1,"Weekly",D143+7,"Monthly",EDATE(D143,1),"Quarterly",EDATE(D143,3),"Yearly",EDATE(D143,12),"One-time","Used","Manual","Manual",D143)))</x:f>
+        <x:f>IF(A143="","",IF(D143="","Available",SWITCH(C143,"Daily",D143+1,"Weekly",IFERROR(VLOOKUP(A143,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D143-VLOOKUP(A143,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D143+7),"Monthly",IFERROR(EDATE(VLOOKUP(A143,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A143,'VIP Signups'!$A$5:$B$204,2,FALSE),D143,"M")+1),EDATE(D143,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A143,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A143,'VIP Signups'!$A$5:$B$204,2,FALSE),D143,"M")/3)+1)*3),EDATE(D143,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A143,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A143,'VIP Signups'!$A$5:$B$204,2,FALSE),D143,"Y")+1)*12),EDATE(D143,12)),"One-time","Used","Manual","Manual",D143)))</x:f>
       </x:c>
       <x:c r="F143" s="20" t="str">
         <x:f>IF(A143="","",IF(D143="","Yes",IF(E143="Manual","Manual",IF(E143="Used","No",IF(E143&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13691,7 +13703,7 @@
       <x:c r="C144" s="20"/>
       <x:c r="D144" s="21"/>
       <x:c r="E144" s="21" t="str">
-        <x:f>IF(A144="","",IF(D144="","Available",SWITCH(C144,"Daily",D144+1,"Weekly",D144+7,"Monthly",EDATE(D144,1),"Quarterly",EDATE(D144,3),"Yearly",EDATE(D144,12),"One-time","Used","Manual","Manual",D144)))</x:f>
+        <x:f>IF(A144="","",IF(D144="","Available",SWITCH(C144,"Daily",D144+1,"Weekly",IFERROR(VLOOKUP(A144,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D144-VLOOKUP(A144,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D144+7),"Monthly",IFERROR(EDATE(VLOOKUP(A144,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A144,'VIP Signups'!$A$5:$B$204,2,FALSE),D144,"M")+1),EDATE(D144,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A144,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A144,'VIP Signups'!$A$5:$B$204,2,FALSE),D144,"M")/3)+1)*3),EDATE(D144,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A144,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A144,'VIP Signups'!$A$5:$B$204,2,FALSE),D144,"Y")+1)*12),EDATE(D144,12)),"One-time","Used","Manual","Manual",D144)))</x:f>
       </x:c>
       <x:c r="F144" s="20" t="str">
         <x:f>IF(A144="","",IF(D144="","Yes",IF(E144="Manual","Manual",IF(E144="Used","No",IF(E144&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13714,7 +13726,7 @@
       <x:c r="C145" s="20"/>
       <x:c r="D145" s="21"/>
       <x:c r="E145" s="21" t="str">
-        <x:f>IF(A145="","",IF(D145="","Available",SWITCH(C145,"Daily",D145+1,"Weekly",D145+7,"Monthly",EDATE(D145,1),"Quarterly",EDATE(D145,3),"Yearly",EDATE(D145,12),"One-time","Used","Manual","Manual",D145)))</x:f>
+        <x:f>IF(A145="","",IF(D145="","Available",SWITCH(C145,"Daily",D145+1,"Weekly",IFERROR(VLOOKUP(A145,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D145-VLOOKUP(A145,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D145+7),"Monthly",IFERROR(EDATE(VLOOKUP(A145,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A145,'VIP Signups'!$A$5:$B$204,2,FALSE),D145,"M")+1),EDATE(D145,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A145,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A145,'VIP Signups'!$A$5:$B$204,2,FALSE),D145,"M")/3)+1)*3),EDATE(D145,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A145,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A145,'VIP Signups'!$A$5:$B$204,2,FALSE),D145,"Y")+1)*12),EDATE(D145,12)),"One-time","Used","Manual","Manual",D145)))</x:f>
       </x:c>
       <x:c r="F145" s="20" t="str">
         <x:f>IF(A145="","",IF(D145="","Yes",IF(E145="Manual","Manual",IF(E145="Used","No",IF(E145&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13737,7 +13749,7 @@
       <x:c r="C146" s="20"/>
       <x:c r="D146" s="21"/>
       <x:c r="E146" s="21" t="str">
-        <x:f>IF(A146="","",IF(D146="","Available",SWITCH(C146,"Daily",D146+1,"Weekly",D146+7,"Monthly",EDATE(D146,1),"Quarterly",EDATE(D146,3),"Yearly",EDATE(D146,12),"One-time","Used","Manual","Manual",D146)))</x:f>
+        <x:f>IF(A146="","",IF(D146="","Available",SWITCH(C146,"Daily",D146+1,"Weekly",IFERROR(VLOOKUP(A146,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D146-VLOOKUP(A146,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D146+7),"Monthly",IFERROR(EDATE(VLOOKUP(A146,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A146,'VIP Signups'!$A$5:$B$204,2,FALSE),D146,"M")+1),EDATE(D146,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A146,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A146,'VIP Signups'!$A$5:$B$204,2,FALSE),D146,"M")/3)+1)*3),EDATE(D146,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A146,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A146,'VIP Signups'!$A$5:$B$204,2,FALSE),D146,"Y")+1)*12),EDATE(D146,12)),"One-time","Used","Manual","Manual",D146)))</x:f>
       </x:c>
       <x:c r="F146" s="20" t="str">
         <x:f>IF(A146="","",IF(D146="","Yes",IF(E146="Manual","Manual",IF(E146="Used","No",IF(E146&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13760,7 +13772,7 @@
       <x:c r="C147" s="20"/>
       <x:c r="D147" s="21"/>
       <x:c r="E147" s="21" t="str">
-        <x:f>IF(A147="","",IF(D147="","Available",SWITCH(C147,"Daily",D147+1,"Weekly",D147+7,"Monthly",EDATE(D147,1),"Quarterly",EDATE(D147,3),"Yearly",EDATE(D147,12),"One-time","Used","Manual","Manual",D147)))</x:f>
+        <x:f>IF(A147="","",IF(D147="","Available",SWITCH(C147,"Daily",D147+1,"Weekly",IFERROR(VLOOKUP(A147,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D147-VLOOKUP(A147,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D147+7),"Monthly",IFERROR(EDATE(VLOOKUP(A147,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A147,'VIP Signups'!$A$5:$B$204,2,FALSE),D147,"M")+1),EDATE(D147,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A147,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A147,'VIP Signups'!$A$5:$B$204,2,FALSE),D147,"M")/3)+1)*3),EDATE(D147,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A147,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A147,'VIP Signups'!$A$5:$B$204,2,FALSE),D147,"Y")+1)*12),EDATE(D147,12)),"One-time","Used","Manual","Manual",D147)))</x:f>
       </x:c>
       <x:c r="F147" s="20" t="str">
         <x:f>IF(A147="","",IF(D147="","Yes",IF(E147="Manual","Manual",IF(E147="Used","No",IF(E147&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13783,7 +13795,7 @@
       <x:c r="C148" s="20"/>
       <x:c r="D148" s="21"/>
       <x:c r="E148" s="21" t="str">
-        <x:f>IF(A148="","",IF(D148="","Available",SWITCH(C148,"Daily",D148+1,"Weekly",D148+7,"Monthly",EDATE(D148,1),"Quarterly",EDATE(D148,3),"Yearly",EDATE(D148,12),"One-time","Used","Manual","Manual",D148)))</x:f>
+        <x:f>IF(A148="","",IF(D148="","Available",SWITCH(C148,"Daily",D148+1,"Weekly",IFERROR(VLOOKUP(A148,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D148-VLOOKUP(A148,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D148+7),"Monthly",IFERROR(EDATE(VLOOKUP(A148,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A148,'VIP Signups'!$A$5:$B$204,2,FALSE),D148,"M")+1),EDATE(D148,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A148,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A148,'VIP Signups'!$A$5:$B$204,2,FALSE),D148,"M")/3)+1)*3),EDATE(D148,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A148,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A148,'VIP Signups'!$A$5:$B$204,2,FALSE),D148,"Y")+1)*12),EDATE(D148,12)),"One-time","Used","Manual","Manual",D148)))</x:f>
       </x:c>
       <x:c r="F148" s="20" t="str">
         <x:f>IF(A148="","",IF(D148="","Yes",IF(E148="Manual","Manual",IF(E148="Used","No",IF(E148&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13806,7 +13818,7 @@
       <x:c r="C149" s="20"/>
       <x:c r="D149" s="21"/>
       <x:c r="E149" s="21" t="str">
-        <x:f>IF(A149="","",IF(D149="","Available",SWITCH(C149,"Daily",D149+1,"Weekly",D149+7,"Monthly",EDATE(D149,1),"Quarterly",EDATE(D149,3),"Yearly",EDATE(D149,12),"One-time","Used","Manual","Manual",D149)))</x:f>
+        <x:f>IF(A149="","",IF(D149="","Available",SWITCH(C149,"Daily",D149+1,"Weekly",IFERROR(VLOOKUP(A149,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D149-VLOOKUP(A149,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D149+7),"Monthly",IFERROR(EDATE(VLOOKUP(A149,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A149,'VIP Signups'!$A$5:$B$204,2,FALSE),D149,"M")+1),EDATE(D149,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A149,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A149,'VIP Signups'!$A$5:$B$204,2,FALSE),D149,"M")/3)+1)*3),EDATE(D149,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A149,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A149,'VIP Signups'!$A$5:$B$204,2,FALSE),D149,"Y")+1)*12),EDATE(D149,12)),"One-time","Used","Manual","Manual",D149)))</x:f>
       </x:c>
       <x:c r="F149" s="20" t="str">
         <x:f>IF(A149="","",IF(D149="","Yes",IF(E149="Manual","Manual",IF(E149="Used","No",IF(E149&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13829,7 +13841,7 @@
       <x:c r="C150" s="20"/>
       <x:c r="D150" s="21"/>
       <x:c r="E150" s="21" t="str">
-        <x:f>IF(A150="","",IF(D150="","Available",SWITCH(C150,"Daily",D150+1,"Weekly",D150+7,"Monthly",EDATE(D150,1),"Quarterly",EDATE(D150,3),"Yearly",EDATE(D150,12),"One-time","Used","Manual","Manual",D150)))</x:f>
+        <x:f>IF(A150="","",IF(D150="","Available",SWITCH(C150,"Daily",D150+1,"Weekly",IFERROR(VLOOKUP(A150,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D150-VLOOKUP(A150,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D150+7),"Monthly",IFERROR(EDATE(VLOOKUP(A150,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A150,'VIP Signups'!$A$5:$B$204,2,FALSE),D150,"M")+1),EDATE(D150,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A150,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A150,'VIP Signups'!$A$5:$B$204,2,FALSE),D150,"M")/3)+1)*3),EDATE(D150,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A150,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A150,'VIP Signups'!$A$5:$B$204,2,FALSE),D150,"Y")+1)*12),EDATE(D150,12)),"One-time","Used","Manual","Manual",D150)))</x:f>
       </x:c>
       <x:c r="F150" s="20" t="str">
         <x:f>IF(A150="","",IF(D150="","Yes",IF(E150="Manual","Manual",IF(E150="Used","No",IF(E150&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13852,7 +13864,7 @@
       <x:c r="C151" s="20"/>
       <x:c r="D151" s="21"/>
       <x:c r="E151" s="21" t="str">
-        <x:f>IF(A151="","",IF(D151="","Available",SWITCH(C151,"Daily",D151+1,"Weekly",D151+7,"Monthly",EDATE(D151,1),"Quarterly",EDATE(D151,3),"Yearly",EDATE(D151,12),"One-time","Used","Manual","Manual",D151)))</x:f>
+        <x:f>IF(A151="","",IF(D151="","Available",SWITCH(C151,"Daily",D151+1,"Weekly",IFERROR(VLOOKUP(A151,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D151-VLOOKUP(A151,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D151+7),"Monthly",IFERROR(EDATE(VLOOKUP(A151,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A151,'VIP Signups'!$A$5:$B$204,2,FALSE),D151,"M")+1),EDATE(D151,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A151,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A151,'VIP Signups'!$A$5:$B$204,2,FALSE),D151,"M")/3)+1)*3),EDATE(D151,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A151,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A151,'VIP Signups'!$A$5:$B$204,2,FALSE),D151,"Y")+1)*12),EDATE(D151,12)),"One-time","Used","Manual","Manual",D151)))</x:f>
       </x:c>
       <x:c r="F151" s="20" t="str">
         <x:f>IF(A151="","",IF(D151="","Yes",IF(E151="Manual","Manual",IF(E151="Used","No",IF(E151&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13875,7 +13887,7 @@
       <x:c r="C152" s="20"/>
       <x:c r="D152" s="21"/>
       <x:c r="E152" s="21" t="str">
-        <x:f>IF(A152="","",IF(D152="","Available",SWITCH(C152,"Daily",D152+1,"Weekly",D152+7,"Monthly",EDATE(D152,1),"Quarterly",EDATE(D152,3),"Yearly",EDATE(D152,12),"One-time","Used","Manual","Manual",D152)))</x:f>
+        <x:f>IF(A152="","",IF(D152="","Available",SWITCH(C152,"Daily",D152+1,"Weekly",IFERROR(VLOOKUP(A152,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D152-VLOOKUP(A152,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D152+7),"Monthly",IFERROR(EDATE(VLOOKUP(A152,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A152,'VIP Signups'!$A$5:$B$204,2,FALSE),D152,"M")+1),EDATE(D152,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A152,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A152,'VIP Signups'!$A$5:$B$204,2,FALSE),D152,"M")/3)+1)*3),EDATE(D152,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A152,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A152,'VIP Signups'!$A$5:$B$204,2,FALSE),D152,"Y")+1)*12),EDATE(D152,12)),"One-time","Used","Manual","Manual",D152)))</x:f>
       </x:c>
       <x:c r="F152" s="20" t="str">
         <x:f>IF(A152="","",IF(D152="","Yes",IF(E152="Manual","Manual",IF(E152="Used","No",IF(E152&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13898,7 +13910,7 @@
       <x:c r="C153" s="20"/>
       <x:c r="D153" s="21"/>
       <x:c r="E153" s="21" t="str">
-        <x:f>IF(A153="","",IF(D153="","Available",SWITCH(C153,"Daily",D153+1,"Weekly",D153+7,"Monthly",EDATE(D153,1),"Quarterly",EDATE(D153,3),"Yearly",EDATE(D153,12),"One-time","Used","Manual","Manual",D153)))</x:f>
+        <x:f>IF(A153="","",IF(D153="","Available",SWITCH(C153,"Daily",D153+1,"Weekly",IFERROR(VLOOKUP(A153,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D153-VLOOKUP(A153,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D153+7),"Monthly",IFERROR(EDATE(VLOOKUP(A153,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A153,'VIP Signups'!$A$5:$B$204,2,FALSE),D153,"M")+1),EDATE(D153,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A153,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A153,'VIP Signups'!$A$5:$B$204,2,FALSE),D153,"M")/3)+1)*3),EDATE(D153,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A153,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A153,'VIP Signups'!$A$5:$B$204,2,FALSE),D153,"Y")+1)*12),EDATE(D153,12)),"One-time","Used","Manual","Manual",D153)))</x:f>
       </x:c>
       <x:c r="F153" s="20" t="str">
         <x:f>IF(A153="","",IF(D153="","Yes",IF(E153="Manual","Manual",IF(E153="Used","No",IF(E153&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13921,7 +13933,7 @@
       <x:c r="C154" s="20"/>
       <x:c r="D154" s="21"/>
       <x:c r="E154" s="21" t="str">
-        <x:f>IF(A154="","",IF(D154="","Available",SWITCH(C154,"Daily",D154+1,"Weekly",D154+7,"Monthly",EDATE(D154,1),"Quarterly",EDATE(D154,3),"Yearly",EDATE(D154,12),"One-time","Used","Manual","Manual",D154)))</x:f>
+        <x:f>IF(A154="","",IF(D154="","Available",SWITCH(C154,"Daily",D154+1,"Weekly",IFERROR(VLOOKUP(A154,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D154-VLOOKUP(A154,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D154+7),"Monthly",IFERROR(EDATE(VLOOKUP(A154,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A154,'VIP Signups'!$A$5:$B$204,2,FALSE),D154,"M")+1),EDATE(D154,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A154,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A154,'VIP Signups'!$A$5:$B$204,2,FALSE),D154,"M")/3)+1)*3),EDATE(D154,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A154,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A154,'VIP Signups'!$A$5:$B$204,2,FALSE),D154,"Y")+1)*12),EDATE(D154,12)),"One-time","Used","Manual","Manual",D154)))</x:f>
       </x:c>
       <x:c r="F154" s="20" t="str">
         <x:f>IF(A154="","",IF(D154="","Yes",IF(E154="Manual","Manual",IF(E154="Used","No",IF(E154&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13944,7 +13956,7 @@
       <x:c r="C155" s="20"/>
       <x:c r="D155" s="21"/>
       <x:c r="E155" s="21" t="str">
-        <x:f>IF(A155="","",IF(D155="","Available",SWITCH(C155,"Daily",D155+1,"Weekly",D155+7,"Monthly",EDATE(D155,1),"Quarterly",EDATE(D155,3),"Yearly",EDATE(D155,12),"One-time","Used","Manual","Manual",D155)))</x:f>
+        <x:f>IF(A155="","",IF(D155="","Available",SWITCH(C155,"Daily",D155+1,"Weekly",IFERROR(VLOOKUP(A155,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D155-VLOOKUP(A155,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D155+7),"Monthly",IFERROR(EDATE(VLOOKUP(A155,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A155,'VIP Signups'!$A$5:$B$204,2,FALSE),D155,"M")+1),EDATE(D155,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A155,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A155,'VIP Signups'!$A$5:$B$204,2,FALSE),D155,"M")/3)+1)*3),EDATE(D155,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A155,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A155,'VIP Signups'!$A$5:$B$204,2,FALSE),D155,"Y")+1)*12),EDATE(D155,12)),"One-time","Used","Manual","Manual",D155)))</x:f>
       </x:c>
       <x:c r="F155" s="20" t="str">
         <x:f>IF(A155="","",IF(D155="","Yes",IF(E155="Manual","Manual",IF(E155="Used","No",IF(E155&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13967,7 +13979,7 @@
       <x:c r="C156" s="20"/>
       <x:c r="D156" s="21"/>
       <x:c r="E156" s="21" t="str">
-        <x:f>IF(A156="","",IF(D156="","Available",SWITCH(C156,"Daily",D156+1,"Weekly",D156+7,"Monthly",EDATE(D156,1),"Quarterly",EDATE(D156,3),"Yearly",EDATE(D156,12),"One-time","Used","Manual","Manual",D156)))</x:f>
+        <x:f>IF(A156="","",IF(D156="","Available",SWITCH(C156,"Daily",D156+1,"Weekly",IFERROR(VLOOKUP(A156,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D156-VLOOKUP(A156,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D156+7),"Monthly",IFERROR(EDATE(VLOOKUP(A156,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A156,'VIP Signups'!$A$5:$B$204,2,FALSE),D156,"M")+1),EDATE(D156,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A156,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A156,'VIP Signups'!$A$5:$B$204,2,FALSE),D156,"M")/3)+1)*3),EDATE(D156,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A156,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A156,'VIP Signups'!$A$5:$B$204,2,FALSE),D156,"Y")+1)*12),EDATE(D156,12)),"One-time","Used","Manual","Manual",D156)))</x:f>
       </x:c>
       <x:c r="F156" s="20" t="str">
         <x:f>IF(A156="","",IF(D156="","Yes",IF(E156="Manual","Manual",IF(E156="Used","No",IF(E156&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -13990,7 +14002,7 @@
       <x:c r="C157" s="20"/>
       <x:c r="D157" s="21"/>
       <x:c r="E157" s="21" t="str">
-        <x:f>IF(A157="","",IF(D157="","Available",SWITCH(C157,"Daily",D157+1,"Weekly",D157+7,"Monthly",EDATE(D157,1),"Quarterly",EDATE(D157,3),"Yearly",EDATE(D157,12),"One-time","Used","Manual","Manual",D157)))</x:f>
+        <x:f>IF(A157="","",IF(D157="","Available",SWITCH(C157,"Daily",D157+1,"Weekly",IFERROR(VLOOKUP(A157,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D157-VLOOKUP(A157,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D157+7),"Monthly",IFERROR(EDATE(VLOOKUP(A157,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A157,'VIP Signups'!$A$5:$B$204,2,FALSE),D157,"M")+1),EDATE(D157,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A157,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A157,'VIP Signups'!$A$5:$B$204,2,FALSE),D157,"M")/3)+1)*3),EDATE(D157,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A157,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A157,'VIP Signups'!$A$5:$B$204,2,FALSE),D157,"Y")+1)*12),EDATE(D157,12)),"One-time","Used","Manual","Manual",D157)))</x:f>
       </x:c>
       <x:c r="F157" s="20" t="str">
         <x:f>IF(A157="","",IF(D157="","Yes",IF(E157="Manual","Manual",IF(E157="Used","No",IF(E157&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14013,7 +14025,7 @@
       <x:c r="C158" s="20"/>
       <x:c r="D158" s="21"/>
       <x:c r="E158" s="21" t="str">
-        <x:f>IF(A158="","",IF(D158="","Available",SWITCH(C158,"Daily",D158+1,"Weekly",D158+7,"Monthly",EDATE(D158,1),"Quarterly",EDATE(D158,3),"Yearly",EDATE(D158,12),"One-time","Used","Manual","Manual",D158)))</x:f>
+        <x:f>IF(A158="","",IF(D158="","Available",SWITCH(C158,"Daily",D158+1,"Weekly",IFERROR(VLOOKUP(A158,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D158-VLOOKUP(A158,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D158+7),"Monthly",IFERROR(EDATE(VLOOKUP(A158,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A158,'VIP Signups'!$A$5:$B$204,2,FALSE),D158,"M")+1),EDATE(D158,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A158,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A158,'VIP Signups'!$A$5:$B$204,2,FALSE),D158,"M")/3)+1)*3),EDATE(D158,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A158,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A158,'VIP Signups'!$A$5:$B$204,2,FALSE),D158,"Y")+1)*12),EDATE(D158,12)),"One-time","Used","Manual","Manual",D158)))</x:f>
       </x:c>
       <x:c r="F158" s="20" t="str">
         <x:f>IF(A158="","",IF(D158="","Yes",IF(E158="Manual","Manual",IF(E158="Used","No",IF(E158&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14036,7 +14048,7 @@
       <x:c r="C159" s="20"/>
       <x:c r="D159" s="21"/>
       <x:c r="E159" s="21" t="str">
-        <x:f>IF(A159="","",IF(D159="","Available",SWITCH(C159,"Daily",D159+1,"Weekly",D159+7,"Monthly",EDATE(D159,1),"Quarterly",EDATE(D159,3),"Yearly",EDATE(D159,12),"One-time","Used","Manual","Manual",D159)))</x:f>
+        <x:f>IF(A159="","",IF(D159="","Available",SWITCH(C159,"Daily",D159+1,"Weekly",IFERROR(VLOOKUP(A159,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D159-VLOOKUP(A159,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D159+7),"Monthly",IFERROR(EDATE(VLOOKUP(A159,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A159,'VIP Signups'!$A$5:$B$204,2,FALSE),D159,"M")+1),EDATE(D159,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A159,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A159,'VIP Signups'!$A$5:$B$204,2,FALSE),D159,"M")/3)+1)*3),EDATE(D159,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A159,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A159,'VIP Signups'!$A$5:$B$204,2,FALSE),D159,"Y")+1)*12),EDATE(D159,12)),"One-time","Used","Manual","Manual",D159)))</x:f>
       </x:c>
       <x:c r="F159" s="20" t="str">
         <x:f>IF(A159="","",IF(D159="","Yes",IF(E159="Manual","Manual",IF(E159="Used","No",IF(E159&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14059,7 +14071,7 @@
       <x:c r="C160" s="20"/>
       <x:c r="D160" s="21"/>
       <x:c r="E160" s="21" t="str">
-        <x:f>IF(A160="","",IF(D160="","Available",SWITCH(C160,"Daily",D160+1,"Weekly",D160+7,"Monthly",EDATE(D160,1),"Quarterly",EDATE(D160,3),"Yearly",EDATE(D160,12),"One-time","Used","Manual","Manual",D160)))</x:f>
+        <x:f>IF(A160="","",IF(D160="","Available",SWITCH(C160,"Daily",D160+1,"Weekly",IFERROR(VLOOKUP(A160,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D160-VLOOKUP(A160,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D160+7),"Monthly",IFERROR(EDATE(VLOOKUP(A160,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A160,'VIP Signups'!$A$5:$B$204,2,FALSE),D160,"M")+1),EDATE(D160,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A160,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A160,'VIP Signups'!$A$5:$B$204,2,FALSE),D160,"M")/3)+1)*3),EDATE(D160,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A160,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A160,'VIP Signups'!$A$5:$B$204,2,FALSE),D160,"Y")+1)*12),EDATE(D160,12)),"One-time","Used","Manual","Manual",D160)))</x:f>
       </x:c>
       <x:c r="F160" s="20" t="str">
         <x:f>IF(A160="","",IF(D160="","Yes",IF(E160="Manual","Manual",IF(E160="Used","No",IF(E160&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14082,7 +14094,7 @@
       <x:c r="C161" s="20"/>
       <x:c r="D161" s="21"/>
       <x:c r="E161" s="21" t="str">
-        <x:f>IF(A161="","",IF(D161="","Available",SWITCH(C161,"Daily",D161+1,"Weekly",D161+7,"Monthly",EDATE(D161,1),"Quarterly",EDATE(D161,3),"Yearly",EDATE(D161,12),"One-time","Used","Manual","Manual",D161)))</x:f>
+        <x:f>IF(A161="","",IF(D161="","Available",SWITCH(C161,"Daily",D161+1,"Weekly",IFERROR(VLOOKUP(A161,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D161-VLOOKUP(A161,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D161+7),"Monthly",IFERROR(EDATE(VLOOKUP(A161,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A161,'VIP Signups'!$A$5:$B$204,2,FALSE),D161,"M")+1),EDATE(D161,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A161,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A161,'VIP Signups'!$A$5:$B$204,2,FALSE),D161,"M")/3)+1)*3),EDATE(D161,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A161,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A161,'VIP Signups'!$A$5:$B$204,2,FALSE),D161,"Y")+1)*12),EDATE(D161,12)),"One-time","Used","Manual","Manual",D161)))</x:f>
       </x:c>
       <x:c r="F161" s="20" t="str">
         <x:f>IF(A161="","",IF(D161="","Yes",IF(E161="Manual","Manual",IF(E161="Used","No",IF(E161&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14105,7 +14117,7 @@
       <x:c r="C162" s="20"/>
       <x:c r="D162" s="21"/>
       <x:c r="E162" s="21" t="str">
-        <x:f>IF(A162="","",IF(D162="","Available",SWITCH(C162,"Daily",D162+1,"Weekly",D162+7,"Monthly",EDATE(D162,1),"Quarterly",EDATE(D162,3),"Yearly",EDATE(D162,12),"One-time","Used","Manual","Manual",D162)))</x:f>
+        <x:f>IF(A162="","",IF(D162="","Available",SWITCH(C162,"Daily",D162+1,"Weekly",IFERROR(VLOOKUP(A162,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D162-VLOOKUP(A162,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D162+7),"Monthly",IFERROR(EDATE(VLOOKUP(A162,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A162,'VIP Signups'!$A$5:$B$204,2,FALSE),D162,"M")+1),EDATE(D162,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A162,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A162,'VIP Signups'!$A$5:$B$204,2,FALSE),D162,"M")/3)+1)*3),EDATE(D162,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A162,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A162,'VIP Signups'!$A$5:$B$204,2,FALSE),D162,"Y")+1)*12),EDATE(D162,12)),"One-time","Used","Manual","Manual",D162)))</x:f>
       </x:c>
       <x:c r="F162" s="20" t="str">
         <x:f>IF(A162="","",IF(D162="","Yes",IF(E162="Manual","Manual",IF(E162="Used","No",IF(E162&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14128,7 +14140,7 @@
       <x:c r="C163" s="20"/>
       <x:c r="D163" s="21"/>
       <x:c r="E163" s="21" t="str">
-        <x:f>IF(A163="","",IF(D163="","Available",SWITCH(C163,"Daily",D163+1,"Weekly",D163+7,"Monthly",EDATE(D163,1),"Quarterly",EDATE(D163,3),"Yearly",EDATE(D163,12),"One-time","Used","Manual","Manual",D163)))</x:f>
+        <x:f>IF(A163="","",IF(D163="","Available",SWITCH(C163,"Daily",D163+1,"Weekly",IFERROR(VLOOKUP(A163,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D163-VLOOKUP(A163,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D163+7),"Monthly",IFERROR(EDATE(VLOOKUP(A163,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A163,'VIP Signups'!$A$5:$B$204,2,FALSE),D163,"M")+1),EDATE(D163,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A163,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A163,'VIP Signups'!$A$5:$B$204,2,FALSE),D163,"M")/3)+1)*3),EDATE(D163,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A163,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A163,'VIP Signups'!$A$5:$B$204,2,FALSE),D163,"Y")+1)*12),EDATE(D163,12)),"One-time","Used","Manual","Manual",D163)))</x:f>
       </x:c>
       <x:c r="F163" s="20" t="str">
         <x:f>IF(A163="","",IF(D163="","Yes",IF(E163="Manual","Manual",IF(E163="Used","No",IF(E163&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14151,7 +14163,7 @@
       <x:c r="C164" s="20"/>
       <x:c r="D164" s="21"/>
       <x:c r="E164" s="21" t="str">
-        <x:f>IF(A164="","",IF(D164="","Available",SWITCH(C164,"Daily",D164+1,"Weekly",D164+7,"Monthly",EDATE(D164,1),"Quarterly",EDATE(D164,3),"Yearly",EDATE(D164,12),"One-time","Used","Manual","Manual",D164)))</x:f>
+        <x:f>IF(A164="","",IF(D164="","Available",SWITCH(C164,"Daily",D164+1,"Weekly",IFERROR(VLOOKUP(A164,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D164-VLOOKUP(A164,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D164+7),"Monthly",IFERROR(EDATE(VLOOKUP(A164,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A164,'VIP Signups'!$A$5:$B$204,2,FALSE),D164,"M")+1),EDATE(D164,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A164,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A164,'VIP Signups'!$A$5:$B$204,2,FALSE),D164,"M")/3)+1)*3),EDATE(D164,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A164,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A164,'VIP Signups'!$A$5:$B$204,2,FALSE),D164,"Y")+1)*12),EDATE(D164,12)),"One-time","Used","Manual","Manual",D164)))</x:f>
       </x:c>
       <x:c r="F164" s="20" t="str">
         <x:f>IF(A164="","",IF(D164="","Yes",IF(E164="Manual","Manual",IF(E164="Used","No",IF(E164&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14174,7 +14186,7 @@
       <x:c r="C165" s="20"/>
       <x:c r="D165" s="21"/>
       <x:c r="E165" s="21" t="str">
-        <x:f>IF(A165="","",IF(D165="","Available",SWITCH(C165,"Daily",D165+1,"Weekly",D165+7,"Monthly",EDATE(D165,1),"Quarterly",EDATE(D165,3),"Yearly",EDATE(D165,12),"One-time","Used","Manual","Manual",D165)))</x:f>
+        <x:f>IF(A165="","",IF(D165="","Available",SWITCH(C165,"Daily",D165+1,"Weekly",IFERROR(VLOOKUP(A165,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D165-VLOOKUP(A165,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D165+7),"Monthly",IFERROR(EDATE(VLOOKUP(A165,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A165,'VIP Signups'!$A$5:$B$204,2,FALSE),D165,"M")+1),EDATE(D165,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A165,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A165,'VIP Signups'!$A$5:$B$204,2,FALSE),D165,"M")/3)+1)*3),EDATE(D165,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A165,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A165,'VIP Signups'!$A$5:$B$204,2,FALSE),D165,"Y")+1)*12),EDATE(D165,12)),"One-time","Used","Manual","Manual",D165)))</x:f>
       </x:c>
       <x:c r="F165" s="20" t="str">
         <x:f>IF(A165="","",IF(D165="","Yes",IF(E165="Manual","Manual",IF(E165="Used","No",IF(E165&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14197,7 +14209,7 @@
       <x:c r="C166" s="20"/>
       <x:c r="D166" s="21"/>
       <x:c r="E166" s="21" t="str">
-        <x:f>IF(A166="","",IF(D166="","Available",SWITCH(C166,"Daily",D166+1,"Weekly",D166+7,"Monthly",EDATE(D166,1),"Quarterly",EDATE(D166,3),"Yearly",EDATE(D166,12),"One-time","Used","Manual","Manual",D166)))</x:f>
+        <x:f>IF(A166="","",IF(D166="","Available",SWITCH(C166,"Daily",D166+1,"Weekly",IFERROR(VLOOKUP(A166,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D166-VLOOKUP(A166,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D166+7),"Monthly",IFERROR(EDATE(VLOOKUP(A166,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A166,'VIP Signups'!$A$5:$B$204,2,FALSE),D166,"M")+1),EDATE(D166,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A166,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A166,'VIP Signups'!$A$5:$B$204,2,FALSE),D166,"M")/3)+1)*3),EDATE(D166,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A166,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A166,'VIP Signups'!$A$5:$B$204,2,FALSE),D166,"Y")+1)*12),EDATE(D166,12)),"One-time","Used","Manual","Manual",D166)))</x:f>
       </x:c>
       <x:c r="F166" s="20" t="str">
         <x:f>IF(A166="","",IF(D166="","Yes",IF(E166="Manual","Manual",IF(E166="Used","No",IF(E166&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14220,7 +14232,7 @@
       <x:c r="C167" s="20"/>
       <x:c r="D167" s="21"/>
       <x:c r="E167" s="21" t="str">
-        <x:f>IF(A167="","",IF(D167="","Available",SWITCH(C167,"Daily",D167+1,"Weekly",D167+7,"Monthly",EDATE(D167,1),"Quarterly",EDATE(D167,3),"Yearly",EDATE(D167,12),"One-time","Used","Manual","Manual",D167)))</x:f>
+        <x:f>IF(A167="","",IF(D167="","Available",SWITCH(C167,"Daily",D167+1,"Weekly",IFERROR(VLOOKUP(A167,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D167-VLOOKUP(A167,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D167+7),"Monthly",IFERROR(EDATE(VLOOKUP(A167,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A167,'VIP Signups'!$A$5:$B$204,2,FALSE),D167,"M")+1),EDATE(D167,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A167,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A167,'VIP Signups'!$A$5:$B$204,2,FALSE),D167,"M")/3)+1)*3),EDATE(D167,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A167,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A167,'VIP Signups'!$A$5:$B$204,2,FALSE),D167,"Y")+1)*12),EDATE(D167,12)),"One-time","Used","Manual","Manual",D167)))</x:f>
       </x:c>
       <x:c r="F167" s="20" t="str">
         <x:f>IF(A167="","",IF(D167="","Yes",IF(E167="Manual","Manual",IF(E167="Used","No",IF(E167&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14243,7 +14255,7 @@
       <x:c r="C168" s="20"/>
       <x:c r="D168" s="21"/>
       <x:c r="E168" s="21" t="str">
-        <x:f>IF(A168="","",IF(D168="","Available",SWITCH(C168,"Daily",D168+1,"Weekly",D168+7,"Monthly",EDATE(D168,1),"Quarterly",EDATE(D168,3),"Yearly",EDATE(D168,12),"One-time","Used","Manual","Manual",D168)))</x:f>
+        <x:f>IF(A168="","",IF(D168="","Available",SWITCH(C168,"Daily",D168+1,"Weekly",IFERROR(VLOOKUP(A168,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D168-VLOOKUP(A168,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D168+7),"Monthly",IFERROR(EDATE(VLOOKUP(A168,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A168,'VIP Signups'!$A$5:$B$204,2,FALSE),D168,"M")+1),EDATE(D168,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A168,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A168,'VIP Signups'!$A$5:$B$204,2,FALSE),D168,"M")/3)+1)*3),EDATE(D168,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A168,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A168,'VIP Signups'!$A$5:$B$204,2,FALSE),D168,"Y")+1)*12),EDATE(D168,12)),"One-time","Used","Manual","Manual",D168)))</x:f>
       </x:c>
       <x:c r="F168" s="20" t="str">
         <x:f>IF(A168="","",IF(D168="","Yes",IF(E168="Manual","Manual",IF(E168="Used","No",IF(E168&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14266,7 +14278,7 @@
       <x:c r="C169" s="20"/>
       <x:c r="D169" s="21"/>
       <x:c r="E169" s="21" t="str">
-        <x:f>IF(A169="","",IF(D169="","Available",SWITCH(C169,"Daily",D169+1,"Weekly",D169+7,"Monthly",EDATE(D169,1),"Quarterly",EDATE(D169,3),"Yearly",EDATE(D169,12),"One-time","Used","Manual","Manual",D169)))</x:f>
+        <x:f>IF(A169="","",IF(D169="","Available",SWITCH(C169,"Daily",D169+1,"Weekly",IFERROR(VLOOKUP(A169,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D169-VLOOKUP(A169,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D169+7),"Monthly",IFERROR(EDATE(VLOOKUP(A169,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A169,'VIP Signups'!$A$5:$B$204,2,FALSE),D169,"M")+1),EDATE(D169,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A169,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A169,'VIP Signups'!$A$5:$B$204,2,FALSE),D169,"M")/3)+1)*3),EDATE(D169,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A169,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A169,'VIP Signups'!$A$5:$B$204,2,FALSE),D169,"Y")+1)*12),EDATE(D169,12)),"One-time","Used","Manual","Manual",D169)))</x:f>
       </x:c>
       <x:c r="F169" s="20" t="str">
         <x:f>IF(A169="","",IF(D169="","Yes",IF(E169="Manual","Manual",IF(E169="Used","No",IF(E169&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14289,7 +14301,7 @@
       <x:c r="C170" s="20"/>
       <x:c r="D170" s="21"/>
       <x:c r="E170" s="21" t="str">
-        <x:f>IF(A170="","",IF(D170="","Available",SWITCH(C170,"Daily",D170+1,"Weekly",D170+7,"Monthly",EDATE(D170,1),"Quarterly",EDATE(D170,3),"Yearly",EDATE(D170,12),"One-time","Used","Manual","Manual",D170)))</x:f>
+        <x:f>IF(A170="","",IF(D170="","Available",SWITCH(C170,"Daily",D170+1,"Weekly",IFERROR(VLOOKUP(A170,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D170-VLOOKUP(A170,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D170+7),"Monthly",IFERROR(EDATE(VLOOKUP(A170,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A170,'VIP Signups'!$A$5:$B$204,2,FALSE),D170,"M")+1),EDATE(D170,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A170,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A170,'VIP Signups'!$A$5:$B$204,2,FALSE),D170,"M")/3)+1)*3),EDATE(D170,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A170,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A170,'VIP Signups'!$A$5:$B$204,2,FALSE),D170,"Y")+1)*12),EDATE(D170,12)),"One-time","Used","Manual","Manual",D170)))</x:f>
       </x:c>
       <x:c r="F170" s="20" t="str">
         <x:f>IF(A170="","",IF(D170="","Yes",IF(E170="Manual","Manual",IF(E170="Used","No",IF(E170&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14312,7 +14324,7 @@
       <x:c r="C171" s="20"/>
       <x:c r="D171" s="21"/>
       <x:c r="E171" s="21" t="str">
-        <x:f>IF(A171="","",IF(D171="","Available",SWITCH(C171,"Daily",D171+1,"Weekly",D171+7,"Monthly",EDATE(D171,1),"Quarterly",EDATE(D171,3),"Yearly",EDATE(D171,12),"One-time","Used","Manual","Manual",D171)))</x:f>
+        <x:f>IF(A171="","",IF(D171="","Available",SWITCH(C171,"Daily",D171+1,"Weekly",IFERROR(VLOOKUP(A171,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D171-VLOOKUP(A171,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D171+7),"Monthly",IFERROR(EDATE(VLOOKUP(A171,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A171,'VIP Signups'!$A$5:$B$204,2,FALSE),D171,"M")+1),EDATE(D171,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A171,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A171,'VIP Signups'!$A$5:$B$204,2,FALSE),D171,"M")/3)+1)*3),EDATE(D171,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A171,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A171,'VIP Signups'!$A$5:$B$204,2,FALSE),D171,"Y")+1)*12),EDATE(D171,12)),"One-time","Used","Manual","Manual",D171)))</x:f>
       </x:c>
       <x:c r="F171" s="20" t="str">
         <x:f>IF(A171="","",IF(D171="","Yes",IF(E171="Manual","Manual",IF(E171="Used","No",IF(E171&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14335,7 +14347,7 @@
       <x:c r="C172" s="20"/>
       <x:c r="D172" s="21"/>
       <x:c r="E172" s="21" t="str">
-        <x:f>IF(A172="","",IF(D172="","Available",SWITCH(C172,"Daily",D172+1,"Weekly",D172+7,"Monthly",EDATE(D172,1),"Quarterly",EDATE(D172,3),"Yearly",EDATE(D172,12),"One-time","Used","Manual","Manual",D172)))</x:f>
+        <x:f>IF(A172="","",IF(D172="","Available",SWITCH(C172,"Daily",D172+1,"Weekly",IFERROR(VLOOKUP(A172,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D172-VLOOKUP(A172,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D172+7),"Monthly",IFERROR(EDATE(VLOOKUP(A172,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A172,'VIP Signups'!$A$5:$B$204,2,FALSE),D172,"M")+1),EDATE(D172,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A172,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A172,'VIP Signups'!$A$5:$B$204,2,FALSE),D172,"M")/3)+1)*3),EDATE(D172,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A172,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A172,'VIP Signups'!$A$5:$B$204,2,FALSE),D172,"Y")+1)*12),EDATE(D172,12)),"One-time","Used","Manual","Manual",D172)))</x:f>
       </x:c>
       <x:c r="F172" s="20" t="str">
         <x:f>IF(A172="","",IF(D172="","Yes",IF(E172="Manual","Manual",IF(E172="Used","No",IF(E172&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14358,7 +14370,7 @@
       <x:c r="C173" s="20"/>
       <x:c r="D173" s="21"/>
       <x:c r="E173" s="21" t="str">
-        <x:f>IF(A173="","",IF(D173="","Available",SWITCH(C173,"Daily",D173+1,"Weekly",D173+7,"Monthly",EDATE(D173,1),"Quarterly",EDATE(D173,3),"Yearly",EDATE(D173,12),"One-time","Used","Manual","Manual",D173)))</x:f>
+        <x:f>IF(A173="","",IF(D173="","Available",SWITCH(C173,"Daily",D173+1,"Weekly",IFERROR(VLOOKUP(A173,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D173-VLOOKUP(A173,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D173+7),"Monthly",IFERROR(EDATE(VLOOKUP(A173,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A173,'VIP Signups'!$A$5:$B$204,2,FALSE),D173,"M")+1),EDATE(D173,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A173,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A173,'VIP Signups'!$A$5:$B$204,2,FALSE),D173,"M")/3)+1)*3),EDATE(D173,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A173,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A173,'VIP Signups'!$A$5:$B$204,2,FALSE),D173,"Y")+1)*12),EDATE(D173,12)),"One-time","Used","Manual","Manual",D173)))</x:f>
       </x:c>
       <x:c r="F173" s="20" t="str">
         <x:f>IF(A173="","",IF(D173="","Yes",IF(E173="Manual","Manual",IF(E173="Used","No",IF(E173&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14381,7 +14393,7 @@
       <x:c r="C174" s="20"/>
       <x:c r="D174" s="21"/>
       <x:c r="E174" s="21" t="str">
-        <x:f>IF(A174="","",IF(D174="","Available",SWITCH(C174,"Daily",D174+1,"Weekly",D174+7,"Monthly",EDATE(D174,1),"Quarterly",EDATE(D174,3),"Yearly",EDATE(D174,12),"One-time","Used","Manual","Manual",D174)))</x:f>
+        <x:f>IF(A174="","",IF(D174="","Available",SWITCH(C174,"Daily",D174+1,"Weekly",IFERROR(VLOOKUP(A174,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D174-VLOOKUP(A174,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D174+7),"Monthly",IFERROR(EDATE(VLOOKUP(A174,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A174,'VIP Signups'!$A$5:$B$204,2,FALSE),D174,"M")+1),EDATE(D174,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A174,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A174,'VIP Signups'!$A$5:$B$204,2,FALSE),D174,"M")/3)+1)*3),EDATE(D174,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A174,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A174,'VIP Signups'!$A$5:$B$204,2,FALSE),D174,"Y")+1)*12),EDATE(D174,12)),"One-time","Used","Manual","Manual",D174)))</x:f>
       </x:c>
       <x:c r="F174" s="20" t="str">
         <x:f>IF(A174="","",IF(D174="","Yes",IF(E174="Manual","Manual",IF(E174="Used","No",IF(E174&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14404,7 +14416,7 @@
       <x:c r="C175" s="20"/>
       <x:c r="D175" s="21"/>
       <x:c r="E175" s="21" t="str">
-        <x:f>IF(A175="","",IF(D175="","Available",SWITCH(C175,"Daily",D175+1,"Weekly",D175+7,"Monthly",EDATE(D175,1),"Quarterly",EDATE(D175,3),"Yearly",EDATE(D175,12),"One-time","Used","Manual","Manual",D175)))</x:f>
+        <x:f>IF(A175="","",IF(D175="","Available",SWITCH(C175,"Daily",D175+1,"Weekly",IFERROR(VLOOKUP(A175,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D175-VLOOKUP(A175,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D175+7),"Monthly",IFERROR(EDATE(VLOOKUP(A175,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A175,'VIP Signups'!$A$5:$B$204,2,FALSE),D175,"M")+1),EDATE(D175,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A175,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A175,'VIP Signups'!$A$5:$B$204,2,FALSE),D175,"M")/3)+1)*3),EDATE(D175,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A175,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A175,'VIP Signups'!$A$5:$B$204,2,FALSE),D175,"Y")+1)*12),EDATE(D175,12)),"One-time","Used","Manual","Manual",D175)))</x:f>
       </x:c>
       <x:c r="F175" s="20" t="str">
         <x:f>IF(A175="","",IF(D175="","Yes",IF(E175="Manual","Manual",IF(E175="Used","No",IF(E175&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14427,7 +14439,7 @@
       <x:c r="C176" s="20"/>
       <x:c r="D176" s="21"/>
       <x:c r="E176" s="21" t="str">
-        <x:f>IF(A176="","",IF(D176="","Available",SWITCH(C176,"Daily",D176+1,"Weekly",D176+7,"Monthly",EDATE(D176,1),"Quarterly",EDATE(D176,3),"Yearly",EDATE(D176,12),"One-time","Used","Manual","Manual",D176)))</x:f>
+        <x:f>IF(A176="","",IF(D176="","Available",SWITCH(C176,"Daily",D176+1,"Weekly",IFERROR(VLOOKUP(A176,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D176-VLOOKUP(A176,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D176+7),"Monthly",IFERROR(EDATE(VLOOKUP(A176,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A176,'VIP Signups'!$A$5:$B$204,2,FALSE),D176,"M")+1),EDATE(D176,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A176,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A176,'VIP Signups'!$A$5:$B$204,2,FALSE),D176,"M")/3)+1)*3),EDATE(D176,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A176,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A176,'VIP Signups'!$A$5:$B$204,2,FALSE),D176,"Y")+1)*12),EDATE(D176,12)),"One-time","Used","Manual","Manual",D176)))</x:f>
       </x:c>
       <x:c r="F176" s="20" t="str">
         <x:f>IF(A176="","",IF(D176="","Yes",IF(E176="Manual","Manual",IF(E176="Used","No",IF(E176&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14450,7 +14462,7 @@
       <x:c r="C177" s="20"/>
       <x:c r="D177" s="21"/>
       <x:c r="E177" s="21" t="str">
-        <x:f>IF(A177="","",IF(D177="","Available",SWITCH(C177,"Daily",D177+1,"Weekly",D177+7,"Monthly",EDATE(D177,1),"Quarterly",EDATE(D177,3),"Yearly",EDATE(D177,12),"One-time","Used","Manual","Manual",D177)))</x:f>
+        <x:f>IF(A177="","",IF(D177="","Available",SWITCH(C177,"Daily",D177+1,"Weekly",IFERROR(VLOOKUP(A177,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D177-VLOOKUP(A177,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D177+7),"Monthly",IFERROR(EDATE(VLOOKUP(A177,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A177,'VIP Signups'!$A$5:$B$204,2,FALSE),D177,"M")+1),EDATE(D177,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A177,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A177,'VIP Signups'!$A$5:$B$204,2,FALSE),D177,"M")/3)+1)*3),EDATE(D177,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A177,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A177,'VIP Signups'!$A$5:$B$204,2,FALSE),D177,"Y")+1)*12),EDATE(D177,12)),"One-time","Used","Manual","Manual",D177)))</x:f>
       </x:c>
       <x:c r="F177" s="20" t="str">
         <x:f>IF(A177="","",IF(D177="","Yes",IF(E177="Manual","Manual",IF(E177="Used","No",IF(E177&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14473,7 +14485,7 @@
       <x:c r="C178" s="20"/>
       <x:c r="D178" s="21"/>
       <x:c r="E178" s="21" t="str">
-        <x:f>IF(A178="","",IF(D178="","Available",SWITCH(C178,"Daily",D178+1,"Weekly",D178+7,"Monthly",EDATE(D178,1),"Quarterly",EDATE(D178,3),"Yearly",EDATE(D178,12),"One-time","Used","Manual","Manual",D178)))</x:f>
+        <x:f>IF(A178="","",IF(D178="","Available",SWITCH(C178,"Daily",D178+1,"Weekly",IFERROR(VLOOKUP(A178,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D178-VLOOKUP(A178,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D178+7),"Monthly",IFERROR(EDATE(VLOOKUP(A178,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A178,'VIP Signups'!$A$5:$B$204,2,FALSE),D178,"M")+1),EDATE(D178,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A178,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A178,'VIP Signups'!$A$5:$B$204,2,FALSE),D178,"M")/3)+1)*3),EDATE(D178,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A178,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A178,'VIP Signups'!$A$5:$B$204,2,FALSE),D178,"Y")+1)*12),EDATE(D178,12)),"One-time","Used","Manual","Manual",D178)))</x:f>
       </x:c>
       <x:c r="F178" s="20" t="str">
         <x:f>IF(A178="","",IF(D178="","Yes",IF(E178="Manual","Manual",IF(E178="Used","No",IF(E178&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14496,7 +14508,7 @@
       <x:c r="C179" s="20"/>
       <x:c r="D179" s="21"/>
       <x:c r="E179" s="21" t="str">
-        <x:f>IF(A179="","",IF(D179="","Available",SWITCH(C179,"Daily",D179+1,"Weekly",D179+7,"Monthly",EDATE(D179,1),"Quarterly",EDATE(D179,3),"Yearly",EDATE(D179,12),"One-time","Used","Manual","Manual",D179)))</x:f>
+        <x:f>IF(A179="","",IF(D179="","Available",SWITCH(C179,"Daily",D179+1,"Weekly",IFERROR(VLOOKUP(A179,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D179-VLOOKUP(A179,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D179+7),"Monthly",IFERROR(EDATE(VLOOKUP(A179,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A179,'VIP Signups'!$A$5:$B$204,2,FALSE),D179,"M")+1),EDATE(D179,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A179,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A179,'VIP Signups'!$A$5:$B$204,2,FALSE),D179,"M")/3)+1)*3),EDATE(D179,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A179,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A179,'VIP Signups'!$A$5:$B$204,2,FALSE),D179,"Y")+1)*12),EDATE(D179,12)),"One-time","Used","Manual","Manual",D179)))</x:f>
       </x:c>
       <x:c r="F179" s="20" t="str">
         <x:f>IF(A179="","",IF(D179="","Yes",IF(E179="Manual","Manual",IF(E179="Used","No",IF(E179&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14519,7 +14531,7 @@
       <x:c r="C180" s="20"/>
       <x:c r="D180" s="21"/>
       <x:c r="E180" s="21" t="str">
-        <x:f>IF(A180="","",IF(D180="","Available",SWITCH(C180,"Daily",D180+1,"Weekly",D180+7,"Monthly",EDATE(D180,1),"Quarterly",EDATE(D180,3),"Yearly",EDATE(D180,12),"One-time","Used","Manual","Manual",D180)))</x:f>
+        <x:f>IF(A180="","",IF(D180="","Available",SWITCH(C180,"Daily",D180+1,"Weekly",IFERROR(VLOOKUP(A180,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D180-VLOOKUP(A180,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D180+7),"Monthly",IFERROR(EDATE(VLOOKUP(A180,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A180,'VIP Signups'!$A$5:$B$204,2,FALSE),D180,"M")+1),EDATE(D180,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A180,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A180,'VIP Signups'!$A$5:$B$204,2,FALSE),D180,"M")/3)+1)*3),EDATE(D180,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A180,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A180,'VIP Signups'!$A$5:$B$204,2,FALSE),D180,"Y")+1)*12),EDATE(D180,12)),"One-time","Used","Manual","Manual",D180)))</x:f>
       </x:c>
       <x:c r="F180" s="20" t="str">
         <x:f>IF(A180="","",IF(D180="","Yes",IF(E180="Manual","Manual",IF(E180="Used","No",IF(E180&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14542,7 +14554,7 @@
       <x:c r="C181" s="20"/>
       <x:c r="D181" s="21"/>
       <x:c r="E181" s="21" t="str">
-        <x:f>IF(A181="","",IF(D181="","Available",SWITCH(C181,"Daily",D181+1,"Weekly",D181+7,"Monthly",EDATE(D181,1),"Quarterly",EDATE(D181,3),"Yearly",EDATE(D181,12),"One-time","Used","Manual","Manual",D181)))</x:f>
+        <x:f>IF(A181="","",IF(D181="","Available",SWITCH(C181,"Daily",D181+1,"Weekly",IFERROR(VLOOKUP(A181,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D181-VLOOKUP(A181,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D181+7),"Monthly",IFERROR(EDATE(VLOOKUP(A181,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A181,'VIP Signups'!$A$5:$B$204,2,FALSE),D181,"M")+1),EDATE(D181,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A181,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A181,'VIP Signups'!$A$5:$B$204,2,FALSE),D181,"M")/3)+1)*3),EDATE(D181,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A181,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A181,'VIP Signups'!$A$5:$B$204,2,FALSE),D181,"Y")+1)*12),EDATE(D181,12)),"One-time","Used","Manual","Manual",D181)))</x:f>
       </x:c>
       <x:c r="F181" s="20" t="str">
         <x:f>IF(A181="","",IF(D181="","Yes",IF(E181="Manual","Manual",IF(E181="Used","No",IF(E181&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14565,7 +14577,7 @@
       <x:c r="C182" s="20"/>
       <x:c r="D182" s="21"/>
       <x:c r="E182" s="21" t="str">
-        <x:f>IF(A182="","",IF(D182="","Available",SWITCH(C182,"Daily",D182+1,"Weekly",D182+7,"Monthly",EDATE(D182,1),"Quarterly",EDATE(D182,3),"Yearly",EDATE(D182,12),"One-time","Used","Manual","Manual",D182)))</x:f>
+        <x:f>IF(A182="","",IF(D182="","Available",SWITCH(C182,"Daily",D182+1,"Weekly",IFERROR(VLOOKUP(A182,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D182-VLOOKUP(A182,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D182+7),"Monthly",IFERROR(EDATE(VLOOKUP(A182,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A182,'VIP Signups'!$A$5:$B$204,2,FALSE),D182,"M")+1),EDATE(D182,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A182,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A182,'VIP Signups'!$A$5:$B$204,2,FALSE),D182,"M")/3)+1)*3),EDATE(D182,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A182,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A182,'VIP Signups'!$A$5:$B$204,2,FALSE),D182,"Y")+1)*12),EDATE(D182,12)),"One-time","Used","Manual","Manual",D182)))</x:f>
       </x:c>
       <x:c r="F182" s="20" t="str">
         <x:f>IF(A182="","",IF(D182="","Yes",IF(E182="Manual","Manual",IF(E182="Used","No",IF(E182&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14588,7 +14600,7 @@
       <x:c r="C183" s="20"/>
       <x:c r="D183" s="21"/>
       <x:c r="E183" s="21" t="str">
-        <x:f>IF(A183="","",IF(D183="","Available",SWITCH(C183,"Daily",D183+1,"Weekly",D183+7,"Monthly",EDATE(D183,1),"Quarterly",EDATE(D183,3),"Yearly",EDATE(D183,12),"One-time","Used","Manual","Manual",D183)))</x:f>
+        <x:f>IF(A183="","",IF(D183="","Available",SWITCH(C183,"Daily",D183+1,"Weekly",IFERROR(VLOOKUP(A183,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D183-VLOOKUP(A183,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D183+7),"Monthly",IFERROR(EDATE(VLOOKUP(A183,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A183,'VIP Signups'!$A$5:$B$204,2,FALSE),D183,"M")+1),EDATE(D183,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A183,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A183,'VIP Signups'!$A$5:$B$204,2,FALSE),D183,"M")/3)+1)*3),EDATE(D183,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A183,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A183,'VIP Signups'!$A$5:$B$204,2,FALSE),D183,"Y")+1)*12),EDATE(D183,12)),"One-time","Used","Manual","Manual",D183)))</x:f>
       </x:c>
       <x:c r="F183" s="20" t="str">
         <x:f>IF(A183="","",IF(D183="","Yes",IF(E183="Manual","Manual",IF(E183="Used","No",IF(E183&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14611,7 +14623,7 @@
       <x:c r="C184" s="20"/>
       <x:c r="D184" s="21"/>
       <x:c r="E184" s="21" t="str">
-        <x:f>IF(A184="","",IF(D184="","Available",SWITCH(C184,"Daily",D184+1,"Weekly",D184+7,"Monthly",EDATE(D184,1),"Quarterly",EDATE(D184,3),"Yearly",EDATE(D184,12),"One-time","Used","Manual","Manual",D184)))</x:f>
+        <x:f>IF(A184="","",IF(D184="","Available",SWITCH(C184,"Daily",D184+1,"Weekly",IFERROR(VLOOKUP(A184,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D184-VLOOKUP(A184,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D184+7),"Monthly",IFERROR(EDATE(VLOOKUP(A184,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A184,'VIP Signups'!$A$5:$B$204,2,FALSE),D184,"M")+1),EDATE(D184,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A184,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A184,'VIP Signups'!$A$5:$B$204,2,FALSE),D184,"M")/3)+1)*3),EDATE(D184,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A184,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A184,'VIP Signups'!$A$5:$B$204,2,FALSE),D184,"Y")+1)*12),EDATE(D184,12)),"One-time","Used","Manual","Manual",D184)))</x:f>
       </x:c>
       <x:c r="F184" s="20" t="str">
         <x:f>IF(A184="","",IF(D184="","Yes",IF(E184="Manual","Manual",IF(E184="Used","No",IF(E184&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14634,7 +14646,7 @@
       <x:c r="C185" s="20"/>
       <x:c r="D185" s="21"/>
       <x:c r="E185" s="21" t="str">
-        <x:f>IF(A185="","",IF(D185="","Available",SWITCH(C185,"Daily",D185+1,"Weekly",D185+7,"Monthly",EDATE(D185,1),"Quarterly",EDATE(D185,3),"Yearly",EDATE(D185,12),"One-time","Used","Manual","Manual",D185)))</x:f>
+        <x:f>IF(A185="","",IF(D185="","Available",SWITCH(C185,"Daily",D185+1,"Weekly",IFERROR(VLOOKUP(A185,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D185-VLOOKUP(A185,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D185+7),"Monthly",IFERROR(EDATE(VLOOKUP(A185,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A185,'VIP Signups'!$A$5:$B$204,2,FALSE),D185,"M")+1),EDATE(D185,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A185,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A185,'VIP Signups'!$A$5:$B$204,2,FALSE),D185,"M")/3)+1)*3),EDATE(D185,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A185,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A185,'VIP Signups'!$A$5:$B$204,2,FALSE),D185,"Y")+1)*12),EDATE(D185,12)),"One-time","Used","Manual","Manual",D185)))</x:f>
       </x:c>
       <x:c r="F185" s="20" t="str">
         <x:f>IF(A185="","",IF(D185="","Yes",IF(E185="Manual","Manual",IF(E185="Used","No",IF(E185&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14657,7 +14669,7 @@
       <x:c r="C186" s="20"/>
       <x:c r="D186" s="21"/>
       <x:c r="E186" s="21" t="str">
-        <x:f>IF(A186="","",IF(D186="","Available",SWITCH(C186,"Daily",D186+1,"Weekly",D186+7,"Monthly",EDATE(D186,1),"Quarterly",EDATE(D186,3),"Yearly",EDATE(D186,12),"One-time","Used","Manual","Manual",D186)))</x:f>
+        <x:f>IF(A186="","",IF(D186="","Available",SWITCH(C186,"Daily",D186+1,"Weekly",IFERROR(VLOOKUP(A186,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D186-VLOOKUP(A186,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D186+7),"Monthly",IFERROR(EDATE(VLOOKUP(A186,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A186,'VIP Signups'!$A$5:$B$204,2,FALSE),D186,"M")+1),EDATE(D186,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A186,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A186,'VIP Signups'!$A$5:$B$204,2,FALSE),D186,"M")/3)+1)*3),EDATE(D186,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A186,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A186,'VIP Signups'!$A$5:$B$204,2,FALSE),D186,"Y")+1)*12),EDATE(D186,12)),"One-time","Used","Manual","Manual",D186)))</x:f>
       </x:c>
       <x:c r="F186" s="20" t="str">
         <x:f>IF(A186="","",IF(D186="","Yes",IF(E186="Manual","Manual",IF(E186="Used","No",IF(E186&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14680,7 +14692,7 @@
       <x:c r="C187" s="20"/>
       <x:c r="D187" s="21"/>
       <x:c r="E187" s="21" t="str">
-        <x:f>IF(A187="","",IF(D187="","Available",SWITCH(C187,"Daily",D187+1,"Weekly",D187+7,"Monthly",EDATE(D187,1),"Quarterly",EDATE(D187,3),"Yearly",EDATE(D187,12),"One-time","Used","Manual","Manual",D187)))</x:f>
+        <x:f>IF(A187="","",IF(D187="","Available",SWITCH(C187,"Daily",D187+1,"Weekly",IFERROR(VLOOKUP(A187,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D187-VLOOKUP(A187,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D187+7),"Monthly",IFERROR(EDATE(VLOOKUP(A187,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A187,'VIP Signups'!$A$5:$B$204,2,FALSE),D187,"M")+1),EDATE(D187,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A187,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A187,'VIP Signups'!$A$5:$B$204,2,FALSE),D187,"M")/3)+1)*3),EDATE(D187,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A187,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A187,'VIP Signups'!$A$5:$B$204,2,FALSE),D187,"Y")+1)*12),EDATE(D187,12)),"One-time","Used","Manual","Manual",D187)))</x:f>
       </x:c>
       <x:c r="F187" s="20" t="str">
         <x:f>IF(A187="","",IF(D187="","Yes",IF(E187="Manual","Manual",IF(E187="Used","No",IF(E187&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14703,7 +14715,7 @@
       <x:c r="C188" s="20"/>
       <x:c r="D188" s="21"/>
       <x:c r="E188" s="21" t="str">
-        <x:f>IF(A188="","",IF(D188="","Available",SWITCH(C188,"Daily",D188+1,"Weekly",D188+7,"Monthly",EDATE(D188,1),"Quarterly",EDATE(D188,3),"Yearly",EDATE(D188,12),"One-time","Used","Manual","Manual",D188)))</x:f>
+        <x:f>IF(A188="","",IF(D188="","Available",SWITCH(C188,"Daily",D188+1,"Weekly",IFERROR(VLOOKUP(A188,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D188-VLOOKUP(A188,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D188+7),"Monthly",IFERROR(EDATE(VLOOKUP(A188,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A188,'VIP Signups'!$A$5:$B$204,2,FALSE),D188,"M")+1),EDATE(D188,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A188,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A188,'VIP Signups'!$A$5:$B$204,2,FALSE),D188,"M")/3)+1)*3),EDATE(D188,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A188,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A188,'VIP Signups'!$A$5:$B$204,2,FALSE),D188,"Y")+1)*12),EDATE(D188,12)),"One-time","Used","Manual","Manual",D188)))</x:f>
       </x:c>
       <x:c r="F188" s="20" t="str">
         <x:f>IF(A188="","",IF(D188="","Yes",IF(E188="Manual","Manual",IF(E188="Used","No",IF(E188&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14726,7 +14738,7 @@
       <x:c r="C189" s="20"/>
       <x:c r="D189" s="21"/>
       <x:c r="E189" s="21" t="str">
-        <x:f>IF(A189="","",IF(D189="","Available",SWITCH(C189,"Daily",D189+1,"Weekly",D189+7,"Monthly",EDATE(D189,1),"Quarterly",EDATE(D189,3),"Yearly",EDATE(D189,12),"One-time","Used","Manual","Manual",D189)))</x:f>
+        <x:f>IF(A189="","",IF(D189="","Available",SWITCH(C189,"Daily",D189+1,"Weekly",IFERROR(VLOOKUP(A189,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D189-VLOOKUP(A189,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D189+7),"Monthly",IFERROR(EDATE(VLOOKUP(A189,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A189,'VIP Signups'!$A$5:$B$204,2,FALSE),D189,"M")+1),EDATE(D189,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A189,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A189,'VIP Signups'!$A$5:$B$204,2,FALSE),D189,"M")/3)+1)*3),EDATE(D189,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A189,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A189,'VIP Signups'!$A$5:$B$204,2,FALSE),D189,"Y")+1)*12),EDATE(D189,12)),"One-time","Used","Manual","Manual",D189)))</x:f>
       </x:c>
       <x:c r="F189" s="20" t="str">
         <x:f>IF(A189="","",IF(D189="","Yes",IF(E189="Manual","Manual",IF(E189="Used","No",IF(E189&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14749,7 +14761,7 @@
       <x:c r="C190" s="20"/>
       <x:c r="D190" s="21"/>
       <x:c r="E190" s="21" t="str">
-        <x:f>IF(A190="","",IF(D190="","Available",SWITCH(C190,"Daily",D190+1,"Weekly",D190+7,"Monthly",EDATE(D190,1),"Quarterly",EDATE(D190,3),"Yearly",EDATE(D190,12),"One-time","Used","Manual","Manual",D190)))</x:f>
+        <x:f>IF(A190="","",IF(D190="","Available",SWITCH(C190,"Daily",D190+1,"Weekly",IFERROR(VLOOKUP(A190,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D190-VLOOKUP(A190,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D190+7),"Monthly",IFERROR(EDATE(VLOOKUP(A190,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A190,'VIP Signups'!$A$5:$B$204,2,FALSE),D190,"M")+1),EDATE(D190,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A190,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A190,'VIP Signups'!$A$5:$B$204,2,FALSE),D190,"M")/3)+1)*3),EDATE(D190,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A190,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A190,'VIP Signups'!$A$5:$B$204,2,FALSE),D190,"Y")+1)*12),EDATE(D190,12)),"One-time","Used","Manual","Manual",D190)))</x:f>
       </x:c>
       <x:c r="F190" s="20" t="str">
         <x:f>IF(A190="","",IF(D190="","Yes",IF(E190="Manual","Manual",IF(E190="Used","No",IF(E190&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14772,7 +14784,7 @@
       <x:c r="C191" s="20"/>
       <x:c r="D191" s="21"/>
       <x:c r="E191" s="21" t="str">
-        <x:f>IF(A191="","",IF(D191="","Available",SWITCH(C191,"Daily",D191+1,"Weekly",D191+7,"Monthly",EDATE(D191,1),"Quarterly",EDATE(D191,3),"Yearly",EDATE(D191,12),"One-time","Used","Manual","Manual",D191)))</x:f>
+        <x:f>IF(A191="","",IF(D191="","Available",SWITCH(C191,"Daily",D191+1,"Weekly",IFERROR(VLOOKUP(A191,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D191-VLOOKUP(A191,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D191+7),"Monthly",IFERROR(EDATE(VLOOKUP(A191,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A191,'VIP Signups'!$A$5:$B$204,2,FALSE),D191,"M")+1),EDATE(D191,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A191,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A191,'VIP Signups'!$A$5:$B$204,2,FALSE),D191,"M")/3)+1)*3),EDATE(D191,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A191,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A191,'VIP Signups'!$A$5:$B$204,2,FALSE),D191,"Y")+1)*12),EDATE(D191,12)),"One-time","Used","Manual","Manual",D191)))</x:f>
       </x:c>
       <x:c r="F191" s="20" t="str">
         <x:f>IF(A191="","",IF(D191="","Yes",IF(E191="Manual","Manual",IF(E191="Used","No",IF(E191&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14795,7 +14807,7 @@
       <x:c r="C192" s="20"/>
       <x:c r="D192" s="21"/>
       <x:c r="E192" s="21" t="str">
-        <x:f>IF(A192="","",IF(D192="","Available",SWITCH(C192,"Daily",D192+1,"Weekly",D192+7,"Monthly",EDATE(D192,1),"Quarterly",EDATE(D192,3),"Yearly",EDATE(D192,12),"One-time","Used","Manual","Manual",D192)))</x:f>
+        <x:f>IF(A192="","",IF(D192="","Available",SWITCH(C192,"Daily",D192+1,"Weekly",IFERROR(VLOOKUP(A192,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D192-VLOOKUP(A192,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D192+7),"Monthly",IFERROR(EDATE(VLOOKUP(A192,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A192,'VIP Signups'!$A$5:$B$204,2,FALSE),D192,"M")+1),EDATE(D192,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A192,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A192,'VIP Signups'!$A$5:$B$204,2,FALSE),D192,"M")/3)+1)*3),EDATE(D192,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A192,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A192,'VIP Signups'!$A$5:$B$204,2,FALSE),D192,"Y")+1)*12),EDATE(D192,12)),"One-time","Used","Manual","Manual",D192)))</x:f>
       </x:c>
       <x:c r="F192" s="20" t="str">
         <x:f>IF(A192="","",IF(D192="","Yes",IF(E192="Manual","Manual",IF(E192="Used","No",IF(E192&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14818,7 +14830,7 @@
       <x:c r="C193" s="20"/>
       <x:c r="D193" s="21"/>
       <x:c r="E193" s="21" t="str">
-        <x:f>IF(A193="","",IF(D193="","Available",SWITCH(C193,"Daily",D193+1,"Weekly",D193+7,"Monthly",EDATE(D193,1),"Quarterly",EDATE(D193,3),"Yearly",EDATE(D193,12),"One-time","Used","Manual","Manual",D193)))</x:f>
+        <x:f>IF(A193="","",IF(D193="","Available",SWITCH(C193,"Daily",D193+1,"Weekly",IFERROR(VLOOKUP(A193,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D193-VLOOKUP(A193,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D193+7),"Monthly",IFERROR(EDATE(VLOOKUP(A193,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A193,'VIP Signups'!$A$5:$B$204,2,FALSE),D193,"M")+1),EDATE(D193,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A193,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A193,'VIP Signups'!$A$5:$B$204,2,FALSE),D193,"M")/3)+1)*3),EDATE(D193,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A193,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A193,'VIP Signups'!$A$5:$B$204,2,FALSE),D193,"Y")+1)*12),EDATE(D193,12)),"One-time","Used","Manual","Manual",D193)))</x:f>
       </x:c>
       <x:c r="F193" s="20" t="str">
         <x:f>IF(A193="","",IF(D193="","Yes",IF(E193="Manual","Manual",IF(E193="Used","No",IF(E193&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14841,7 +14853,7 @@
       <x:c r="C194" s="20"/>
       <x:c r="D194" s="21"/>
       <x:c r="E194" s="21" t="str">
-        <x:f>IF(A194="","",IF(D194="","Available",SWITCH(C194,"Daily",D194+1,"Weekly",D194+7,"Monthly",EDATE(D194,1),"Quarterly",EDATE(D194,3),"Yearly",EDATE(D194,12),"One-time","Used","Manual","Manual",D194)))</x:f>
+        <x:f>IF(A194="","",IF(D194="","Available",SWITCH(C194,"Daily",D194+1,"Weekly",IFERROR(VLOOKUP(A194,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D194-VLOOKUP(A194,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D194+7),"Monthly",IFERROR(EDATE(VLOOKUP(A194,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A194,'VIP Signups'!$A$5:$B$204,2,FALSE),D194,"M")+1),EDATE(D194,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A194,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A194,'VIP Signups'!$A$5:$B$204,2,FALSE),D194,"M")/3)+1)*3),EDATE(D194,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A194,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A194,'VIP Signups'!$A$5:$B$204,2,FALSE),D194,"Y")+1)*12),EDATE(D194,12)),"One-time","Used","Manual","Manual",D194)))</x:f>
       </x:c>
       <x:c r="F194" s="20" t="str">
         <x:f>IF(A194="","",IF(D194="","Yes",IF(E194="Manual","Manual",IF(E194="Used","No",IF(E194&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14864,7 +14876,7 @@
       <x:c r="C195" s="20"/>
       <x:c r="D195" s="21"/>
       <x:c r="E195" s="21" t="str">
-        <x:f>IF(A195="","",IF(D195="","Available",SWITCH(C195,"Daily",D195+1,"Weekly",D195+7,"Monthly",EDATE(D195,1),"Quarterly",EDATE(D195,3),"Yearly",EDATE(D195,12),"One-time","Used","Manual","Manual",D195)))</x:f>
+        <x:f>IF(A195="","",IF(D195="","Available",SWITCH(C195,"Daily",D195+1,"Weekly",IFERROR(VLOOKUP(A195,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D195-VLOOKUP(A195,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D195+7),"Monthly",IFERROR(EDATE(VLOOKUP(A195,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A195,'VIP Signups'!$A$5:$B$204,2,FALSE),D195,"M")+1),EDATE(D195,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A195,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A195,'VIP Signups'!$A$5:$B$204,2,FALSE),D195,"M")/3)+1)*3),EDATE(D195,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A195,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A195,'VIP Signups'!$A$5:$B$204,2,FALSE),D195,"Y")+1)*12),EDATE(D195,12)),"One-time","Used","Manual","Manual",D195)))</x:f>
       </x:c>
       <x:c r="F195" s="20" t="str">
         <x:f>IF(A195="","",IF(D195="","Yes",IF(E195="Manual","Manual",IF(E195="Used","No",IF(E195&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14887,7 +14899,7 @@
       <x:c r="C196" s="20"/>
       <x:c r="D196" s="21"/>
       <x:c r="E196" s="21" t="str">
-        <x:f>IF(A196="","",IF(D196="","Available",SWITCH(C196,"Daily",D196+1,"Weekly",D196+7,"Monthly",EDATE(D196,1),"Quarterly",EDATE(D196,3),"Yearly",EDATE(D196,12),"One-time","Used","Manual","Manual",D196)))</x:f>
+        <x:f>IF(A196="","",IF(D196="","Available",SWITCH(C196,"Daily",D196+1,"Weekly",IFERROR(VLOOKUP(A196,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D196-VLOOKUP(A196,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D196+7),"Monthly",IFERROR(EDATE(VLOOKUP(A196,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A196,'VIP Signups'!$A$5:$B$204,2,FALSE),D196,"M")+1),EDATE(D196,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A196,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A196,'VIP Signups'!$A$5:$B$204,2,FALSE),D196,"M")/3)+1)*3),EDATE(D196,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A196,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A196,'VIP Signups'!$A$5:$B$204,2,FALSE),D196,"Y")+1)*12),EDATE(D196,12)),"One-time","Used","Manual","Manual",D196)))</x:f>
       </x:c>
       <x:c r="F196" s="20" t="str">
         <x:f>IF(A196="","",IF(D196="","Yes",IF(E196="Manual","Manual",IF(E196="Used","No",IF(E196&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14910,7 +14922,7 @@
       <x:c r="C197" s="20"/>
       <x:c r="D197" s="21"/>
       <x:c r="E197" s="21" t="str">
-        <x:f>IF(A197="","",IF(D197="","Available",SWITCH(C197,"Daily",D197+1,"Weekly",D197+7,"Monthly",EDATE(D197,1),"Quarterly",EDATE(D197,3),"Yearly",EDATE(D197,12),"One-time","Used","Manual","Manual",D197)))</x:f>
+        <x:f>IF(A197="","",IF(D197="","Available",SWITCH(C197,"Daily",D197+1,"Weekly",IFERROR(VLOOKUP(A197,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D197-VLOOKUP(A197,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D197+7),"Monthly",IFERROR(EDATE(VLOOKUP(A197,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A197,'VIP Signups'!$A$5:$B$204,2,FALSE),D197,"M")+1),EDATE(D197,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A197,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A197,'VIP Signups'!$A$5:$B$204,2,FALSE),D197,"M")/3)+1)*3),EDATE(D197,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A197,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A197,'VIP Signups'!$A$5:$B$204,2,FALSE),D197,"Y")+1)*12),EDATE(D197,12)),"One-time","Used","Manual","Manual",D197)))</x:f>
       </x:c>
       <x:c r="F197" s="20" t="str">
         <x:f>IF(A197="","",IF(D197="","Yes",IF(E197="Manual","Manual",IF(E197="Used","No",IF(E197&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14933,7 +14945,7 @@
       <x:c r="C198" s="20"/>
       <x:c r="D198" s="21"/>
       <x:c r="E198" s="21" t="str">
-        <x:f>IF(A198="","",IF(D198="","Available",SWITCH(C198,"Daily",D198+1,"Weekly",D198+7,"Monthly",EDATE(D198,1),"Quarterly",EDATE(D198,3),"Yearly",EDATE(D198,12),"One-time","Used","Manual","Manual",D198)))</x:f>
+        <x:f>IF(A198="","",IF(D198="","Available",SWITCH(C198,"Daily",D198+1,"Weekly",IFERROR(VLOOKUP(A198,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D198-VLOOKUP(A198,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D198+7),"Monthly",IFERROR(EDATE(VLOOKUP(A198,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A198,'VIP Signups'!$A$5:$B$204,2,FALSE),D198,"M")+1),EDATE(D198,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A198,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A198,'VIP Signups'!$A$5:$B$204,2,FALSE),D198,"M")/3)+1)*3),EDATE(D198,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A198,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A198,'VIP Signups'!$A$5:$B$204,2,FALSE),D198,"Y")+1)*12),EDATE(D198,12)),"One-time","Used","Manual","Manual",D198)))</x:f>
       </x:c>
       <x:c r="F198" s="20" t="str">
         <x:f>IF(A198="","",IF(D198="","Yes",IF(E198="Manual","Manual",IF(E198="Used","No",IF(E198&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14956,7 +14968,7 @@
       <x:c r="C199" s="20"/>
       <x:c r="D199" s="21"/>
       <x:c r="E199" s="21" t="str">
-        <x:f>IF(A199="","",IF(D199="","Available",SWITCH(C199,"Daily",D199+1,"Weekly",D199+7,"Monthly",EDATE(D199,1),"Quarterly",EDATE(D199,3),"Yearly",EDATE(D199,12),"One-time","Used","Manual","Manual",D199)))</x:f>
+        <x:f>IF(A199="","",IF(D199="","Available",SWITCH(C199,"Daily",D199+1,"Weekly",IFERROR(VLOOKUP(A199,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D199-VLOOKUP(A199,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D199+7),"Monthly",IFERROR(EDATE(VLOOKUP(A199,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A199,'VIP Signups'!$A$5:$B$204,2,FALSE),D199,"M")+1),EDATE(D199,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A199,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A199,'VIP Signups'!$A$5:$B$204,2,FALSE),D199,"M")/3)+1)*3),EDATE(D199,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A199,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A199,'VIP Signups'!$A$5:$B$204,2,FALSE),D199,"Y")+1)*12),EDATE(D199,12)),"One-time","Used","Manual","Manual",D199)))</x:f>
       </x:c>
       <x:c r="F199" s="20" t="str">
         <x:f>IF(A199="","",IF(D199="","Yes",IF(E199="Manual","Manual",IF(E199="Used","No",IF(E199&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -14979,7 +14991,7 @@
       <x:c r="C200" s="20"/>
       <x:c r="D200" s="21"/>
       <x:c r="E200" s="21" t="str">
-        <x:f>IF(A200="","",IF(D200="","Available",SWITCH(C200,"Daily",D200+1,"Weekly",D200+7,"Monthly",EDATE(D200,1),"Quarterly",EDATE(D200,3),"Yearly",EDATE(D200,12),"One-time","Used","Manual","Manual",D200)))</x:f>
+        <x:f>IF(A200="","",IF(D200="","Available",SWITCH(C200,"Daily",D200+1,"Weekly",IFERROR(VLOOKUP(A200,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D200-VLOOKUP(A200,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D200+7),"Monthly",IFERROR(EDATE(VLOOKUP(A200,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A200,'VIP Signups'!$A$5:$B$204,2,FALSE),D200,"M")+1),EDATE(D200,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A200,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A200,'VIP Signups'!$A$5:$B$204,2,FALSE),D200,"M")/3)+1)*3),EDATE(D200,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A200,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A200,'VIP Signups'!$A$5:$B$204,2,FALSE),D200,"Y")+1)*12),EDATE(D200,12)),"One-time","Used","Manual","Manual",D200)))</x:f>
       </x:c>
       <x:c r="F200" s="20" t="str">
         <x:f>IF(A200="","",IF(D200="","Yes",IF(E200="Manual","Manual",IF(E200="Used","No",IF(E200&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -15002,7 +15014,7 @@
       <x:c r="C201" s="20"/>
       <x:c r="D201" s="21"/>
       <x:c r="E201" s="21" t="str">
-        <x:f>IF(A201="","",IF(D201="","Available",SWITCH(C201,"Daily",D201+1,"Weekly",D201+7,"Monthly",EDATE(D201,1),"Quarterly",EDATE(D201,3),"Yearly",EDATE(D201,12),"One-time","Used","Manual","Manual",D201)))</x:f>
+        <x:f>IF(A201="","",IF(D201="","Available",SWITCH(C201,"Daily",D201+1,"Weekly",IFERROR(VLOOKUP(A201,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D201-VLOOKUP(A201,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D201+7),"Monthly",IFERROR(EDATE(VLOOKUP(A201,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A201,'VIP Signups'!$A$5:$B$204,2,FALSE),D201,"M")+1),EDATE(D201,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A201,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A201,'VIP Signups'!$A$5:$B$204,2,FALSE),D201,"M")/3)+1)*3),EDATE(D201,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A201,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A201,'VIP Signups'!$A$5:$B$204,2,FALSE),D201,"Y")+1)*12),EDATE(D201,12)),"One-time","Used","Manual","Manual",D201)))</x:f>
       </x:c>
       <x:c r="F201" s="20" t="str">
         <x:f>IF(A201="","",IF(D201="","Yes",IF(E201="Manual","Manual",IF(E201="Used","No",IF(E201&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -15025,7 +15037,7 @@
       <x:c r="C202" s="20"/>
       <x:c r="D202" s="21"/>
       <x:c r="E202" s="21" t="str">
-        <x:f>IF(A202="","",IF(D202="","Available",SWITCH(C202,"Daily",D202+1,"Weekly",D202+7,"Monthly",EDATE(D202,1),"Quarterly",EDATE(D202,3),"Yearly",EDATE(D202,12),"One-time","Used","Manual","Manual",D202)))</x:f>
+        <x:f>IF(A202="","",IF(D202="","Available",SWITCH(C202,"Daily",D202+1,"Weekly",IFERROR(VLOOKUP(A202,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D202-VLOOKUP(A202,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D202+7),"Monthly",IFERROR(EDATE(VLOOKUP(A202,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A202,'VIP Signups'!$A$5:$B$204,2,FALSE),D202,"M")+1),EDATE(D202,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A202,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A202,'VIP Signups'!$A$5:$B$204,2,FALSE),D202,"M")/3)+1)*3),EDATE(D202,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A202,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A202,'VIP Signups'!$A$5:$B$204,2,FALSE),D202,"Y")+1)*12),EDATE(D202,12)),"One-time","Used","Manual","Manual",D202)))</x:f>
       </x:c>
       <x:c r="F202" s="20" t="str">
         <x:f>IF(A202="","",IF(D202="","Yes",IF(E202="Manual","Manual",IF(E202="Used","No",IF(E202&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -15048,7 +15060,7 @@
       <x:c r="C203" s="20"/>
       <x:c r="D203" s="21"/>
       <x:c r="E203" s="21" t="str">
-        <x:f>IF(A203="","",IF(D203="","Available",SWITCH(C203,"Daily",D203+1,"Weekly",D203+7,"Monthly",EDATE(D203,1),"Quarterly",EDATE(D203,3),"Yearly",EDATE(D203,12),"One-time","Used","Manual","Manual",D203)))</x:f>
+        <x:f>IF(A203="","",IF(D203="","Available",SWITCH(C203,"Daily",D203+1,"Weekly",IFERROR(VLOOKUP(A203,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D203-VLOOKUP(A203,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D203+7),"Monthly",IFERROR(EDATE(VLOOKUP(A203,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A203,'VIP Signups'!$A$5:$B$204,2,FALSE),D203,"M")+1),EDATE(D203,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A203,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A203,'VIP Signups'!$A$5:$B$204,2,FALSE),D203,"M")/3)+1)*3),EDATE(D203,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A203,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A203,'VIP Signups'!$A$5:$B$204,2,FALSE),D203,"Y")+1)*12),EDATE(D203,12)),"One-time","Used","Manual","Manual",D203)))</x:f>
       </x:c>
       <x:c r="F203" s="20" t="str">
         <x:f>IF(A203="","",IF(D203="","Yes",IF(E203="Manual","Manual",IF(E203="Used","No",IF(E203&lt;=TODAY(),"Yes","No")))))</x:f>
@@ -15071,7 +15083,7 @@
       <x:c r="C204" s="20"/>
       <x:c r="D204" s="21"/>
       <x:c r="E204" s="21" t="str">
-        <x:f>IF(A204="","",IF(D204="","Available",SWITCH(C204,"Daily",D204+1,"Weekly",D204+7,"Monthly",EDATE(D204,1),"Quarterly",EDATE(D204,3),"Yearly",EDATE(D204,12),"One-time","Used","Manual","Manual",D204)))</x:f>
+        <x:f>IF(A204="","",IF(D204="","Available",SWITCH(C204,"Daily",D204+1,"Weekly",IFERROR(VLOOKUP(A204,'VIP Signups'!$A$5:$B$204,2,FALSE)+CEILING((D204-VLOOKUP(A204,'VIP Signups'!$A$5:$B$204,2,FALSE)+1)/7,1)*7,D204+7),"Monthly",IFERROR(EDATE(VLOOKUP(A204,'VIP Signups'!$A$5:$B$204,2,FALSE),DATEDIF(VLOOKUP(A204,'VIP Signups'!$A$5:$B$204,2,FALSE),D204,"M")+1),EDATE(D204,1)),"Quarterly",IFERROR(EDATE(VLOOKUP(A204,'VIP Signups'!$A$5:$B$204,2,FALSE),(INT(DATEDIF(VLOOKUP(A204,'VIP Signups'!$A$5:$B$204,2,FALSE),D204,"M")/3)+1)*3),EDATE(D204,3)),"Yearly",IFERROR(EDATE(VLOOKUP(A204,'VIP Signups'!$A$5:$B$204,2,FALSE),(DATEDIF(VLOOKUP(A204,'VIP Signups'!$A$5:$B$204,2,FALSE),D204,"Y")+1)*12),EDATE(D204,12)),"One-time","Used","Manual","Manual",D204)))</x:f>
       </x:c>
       <x:c r="F204" s="20" t="str">
         <x:f>IF(A204="","",IF(D204="","Yes",IF(E204="Manual","Manual",IF(E204="Used","No",IF(E204&lt;=TODAY(),"Yes","No")))))</x:f>

</xml_diff>